<commit_message>
test: validate color selection
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/testData_Appium_myDemoApp.xlsx
+++ b/src/test/resources/testData/testData_Appium_myDemoApp.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="42">
   <si>
     <t>CT</t>
   </si>
@@ -26,6 +26,9 @@
   </si>
   <si>
     <t>PRODUCT_NAME</t>
+  </si>
+  <si>
+    <t>PRODUCT_COLOR</t>
   </si>
   <si>
     <t>FIRSTNAME</t>
@@ -103,13 +106,13 @@
     <t>009</t>
   </si>
   <si>
+    <t>Blue color</t>
+  </si>
+  <si>
     <t>010</t>
   </si>
   <si>
     <t>011</t>
-  </si>
-  <si>
-    <t>\</t>
   </si>
   <si>
     <t>012</t>
@@ -417,14 +420,14 @@
     <col customWidth="1" min="1" max="1" width="12.63"/>
     <col customWidth="1" min="2" max="2" width="19.63"/>
     <col customWidth="1" min="3" max="3" width="21.63"/>
-    <col customWidth="1" min="4" max="5" width="31.38"/>
-    <col customWidth="1" min="6" max="6" width="18.38"/>
-    <col customWidth="1" min="7" max="7" width="17.13"/>
-    <col customWidth="1" min="8" max="8" width="16.0"/>
-    <col customWidth="1" min="9" max="10" width="17.13"/>
-    <col customWidth="1" min="11" max="11" width="15.75"/>
-    <col customWidth="1" min="12" max="12" width="14.38"/>
-    <col customWidth="1" min="15" max="15" width="27.0"/>
+    <col customWidth="1" min="4" max="6" width="31.38"/>
+    <col customWidth="1" min="7" max="7" width="18.38"/>
+    <col customWidth="1" min="8" max="8" width="17.13"/>
+    <col customWidth="1" min="9" max="9" width="16.0"/>
+    <col customWidth="1" min="10" max="11" width="17.13"/>
+    <col customWidth="1" min="12" max="12" width="15.75"/>
+    <col customWidth="1" min="13" max="13" width="14.38"/>
+    <col customWidth="1" min="16" max="16" width="27.0"/>
   </cols>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
@@ -443,7 +446,7 @@
       <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
@@ -473,7 +476,9 @@
       <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="4"/>
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="Q1" s="4"/>
       <c r="R1" s="4"/>
       <c r="S1" s="4"/>
@@ -481,16 +486,17 @@
       <c r="U1" s="4"/>
       <c r="V1" s="4"/>
       <c r="W1" s="4"/>
+      <c r="X1" s="4"/>
     </row>
     <row r="2" ht="15.75" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
@@ -504,7 +510,7 @@
       <c r="M2" s="1"/>
       <c r="N2" s="1"/>
       <c r="O2" s="1"/>
-      <c r="P2" s="4"/>
+      <c r="P2" s="1"/>
       <c r="Q2" s="4"/>
       <c r="R2" s="4"/>
       <c r="S2" s="4"/>
@@ -512,10 +518,11 @@
       <c r="U2" s="4"/>
       <c r="V2" s="4"/>
       <c r="W2" s="4"/>
+      <c r="X2" s="4"/>
     </row>
     <row r="3" ht="15.75" customHeight="1">
       <c r="A3" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
@@ -531,7 +538,7 @@
       <c r="M3" s="1"/>
       <c r="N3" s="1"/>
       <c r="O3" s="1"/>
-      <c r="P3" s="4"/>
+      <c r="P3" s="1"/>
       <c r="Q3" s="4"/>
       <c r="R3" s="4"/>
       <c r="S3" s="4"/>
@@ -539,16 +546,17 @@
       <c r="U3" s="4"/>
       <c r="V3" s="4"/>
       <c r="W3" s="4"/>
+      <c r="X3" s="4"/>
     </row>
     <row r="4" ht="15.75" customHeight="1">
       <c r="A4" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
@@ -562,7 +570,7 @@
       <c r="M4" s="1"/>
       <c r="N4" s="1"/>
       <c r="O4" s="1"/>
-      <c r="P4" s="4"/>
+      <c r="P4" s="1"/>
       <c r="Q4" s="4"/>
       <c r="R4" s="4"/>
       <c r="S4" s="4"/>
@@ -570,15 +578,16 @@
       <c r="U4" s="4"/>
       <c r="V4" s="4"/>
       <c r="W4" s="4"/>
+      <c r="X4" s="4"/>
     </row>
     <row r="5" ht="15.75" customHeight="1">
       <c r="A5" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
       <c r="D5" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E5" s="1"/>
       <c r="F5" s="1"/>
@@ -591,7 +600,7 @@
       <c r="M5" s="1"/>
       <c r="N5" s="1"/>
       <c r="O5" s="1"/>
-      <c r="P5" s="4"/>
+      <c r="P5" s="1"/>
       <c r="Q5" s="4"/>
       <c r="R5" s="4"/>
       <c r="S5" s="4"/>
@@ -599,15 +608,16 @@
       <c r="U5" s="4"/>
       <c r="V5" s="4"/>
       <c r="W5" s="4"/>
+      <c r="X5" s="4"/>
     </row>
     <row r="6" ht="15.75" customHeight="1">
       <c r="A6" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
       <c r="D6" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E6" s="1"/>
       <c r="F6" s="1"/>
@@ -620,7 +630,7 @@
       <c r="M6" s="1"/>
       <c r="N6" s="1"/>
       <c r="O6" s="1"/>
-      <c r="P6" s="4"/>
+      <c r="P6" s="1"/>
       <c r="Q6" s="4"/>
       <c r="R6" s="4"/>
       <c r="S6" s="4"/>
@@ -628,15 +638,16 @@
       <c r="U6" s="4"/>
       <c r="V6" s="4"/>
       <c r="W6" s="4"/>
+      <c r="X6" s="4"/>
     </row>
     <row r="7" ht="15.75" customHeight="1">
       <c r="A7" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
       <c r="D7" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E7" s="1"/>
       <c r="F7" s="1"/>
@@ -649,7 +660,7 @@
       <c r="M7" s="1"/>
       <c r="N7" s="1"/>
       <c r="O7" s="1"/>
-      <c r="P7" s="4"/>
+      <c r="P7" s="1"/>
       <c r="Q7" s="4"/>
       <c r="R7" s="4"/>
       <c r="S7" s="4"/>
@@ -657,15 +668,16 @@
       <c r="U7" s="4"/>
       <c r="V7" s="4"/>
       <c r="W7" s="4"/>
+      <c r="X7" s="4"/>
     </row>
     <row r="8" ht="15.75" customHeight="1">
       <c r="A8" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
       <c r="D8" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E8" s="1"/>
       <c r="F8" s="1"/>
@@ -678,7 +690,7 @@
       <c r="M8" s="1"/>
       <c r="N8" s="1"/>
       <c r="O8" s="1"/>
-      <c r="P8" s="4"/>
+      <c r="P8" s="1"/>
       <c r="Q8" s="4"/>
       <c r="R8" s="4"/>
       <c r="S8" s="4"/>
@@ -686,18 +698,19 @@
       <c r="U8" s="4"/>
       <c r="V8" s="4"/>
       <c r="W8" s="4"/>
+      <c r="X8" s="4"/>
     </row>
     <row r="9" ht="15.75" customHeight="1">
       <c r="A9" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
       <c r="D9" s="1"/>
       <c r="E9" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
-      <c r="F9" s="1"/>
+      <c r="F9" s="3"/>
       <c r="G9" s="1"/>
       <c r="H9" s="1"/>
       <c r="I9" s="1"/>
@@ -707,7 +720,7 @@
       <c r="M9" s="1"/>
       <c r="N9" s="1"/>
       <c r="O9" s="1"/>
-      <c r="P9" s="4"/>
+      <c r="P9" s="1"/>
       <c r="Q9" s="4"/>
       <c r="R9" s="4"/>
       <c r="S9" s="4"/>
@@ -715,16 +728,21 @@
       <c r="U9" s="4"/>
       <c r="V9" s="4"/>
       <c r="W9" s="4"/>
+      <c r="X9" s="4"/>
     </row>
     <row r="10" ht="15.75" customHeight="1">
       <c r="A10" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
       <c r="D10" s="1"/>
-      <c r="E10" s="1"/>
-      <c r="F10" s="1"/>
+      <c r="E10" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>31</v>
+      </c>
       <c r="G10" s="1"/>
       <c r="H10" s="1"/>
       <c r="I10" s="1"/>
@@ -734,7 +752,7 @@
       <c r="M10" s="1"/>
       <c r="N10" s="1"/>
       <c r="O10" s="1"/>
-      <c r="P10" s="4"/>
+      <c r="P10" s="1"/>
       <c r="Q10" s="4"/>
       <c r="R10" s="4"/>
       <c r="S10" s="4"/>
@@ -742,10 +760,11 @@
       <c r="U10" s="4"/>
       <c r="V10" s="4"/>
       <c r="W10" s="4"/>
+      <c r="X10" s="4"/>
     </row>
     <row r="11" ht="15.75" customHeight="1">
       <c r="A11" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
@@ -761,7 +780,7 @@
       <c r="M11" s="1"/>
       <c r="N11" s="1"/>
       <c r="O11" s="1"/>
-      <c r="P11" s="4"/>
+      <c r="P11" s="1"/>
       <c r="Q11" s="4"/>
       <c r="R11" s="4"/>
       <c r="S11" s="4"/>
@@ -769,18 +788,17 @@
       <c r="U11" s="4"/>
       <c r="V11" s="4"/>
       <c r="W11" s="4"/>
+      <c r="X11" s="4"/>
     </row>
     <row r="12" ht="15.75" customHeight="1">
       <c r="A12" s="1" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
       <c r="D12" s="1"/>
-      <c r="E12" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="F12" s="1"/>
+      <c r="E12" s="3"/>
+      <c r="F12" s="3"/>
       <c r="G12" s="1"/>
       <c r="H12" s="1"/>
       <c r="I12" s="1"/>
@@ -790,7 +808,7 @@
       <c r="M12" s="1"/>
       <c r="N12" s="1"/>
       <c r="O12" s="1"/>
-      <c r="P12" s="4"/>
+      <c r="P12" s="1"/>
       <c r="Q12" s="4"/>
       <c r="R12" s="4"/>
       <c r="S12" s="4"/>
@@ -798,10 +816,11 @@
       <c r="U12" s="4"/>
       <c r="V12" s="4"/>
       <c r="W12" s="4"/>
+      <c r="X12" s="4"/>
     </row>
     <row r="13" ht="15.75" customHeight="1">
       <c r="A13" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
@@ -817,7 +836,7 @@
       <c r="M13" s="1"/>
       <c r="N13" s="1"/>
       <c r="O13" s="1"/>
-      <c r="P13" s="4"/>
+      <c r="P13" s="1"/>
       <c r="Q13" s="4"/>
       <c r="R13" s="4"/>
       <c r="S13" s="4"/>
@@ -825,10 +844,11 @@
       <c r="U13" s="4"/>
       <c r="V13" s="4"/>
       <c r="W13" s="4"/>
+      <c r="X13" s="4"/>
     </row>
     <row r="14" ht="15.75" customHeight="1">
       <c r="A14" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
@@ -844,7 +864,7 @@
       <c r="M14" s="1"/>
       <c r="N14" s="1"/>
       <c r="O14" s="1"/>
-      <c r="P14" s="4"/>
+      <c r="P14" s="1"/>
       <c r="Q14" s="4"/>
       <c r="R14" s="4"/>
       <c r="S14" s="4"/>
@@ -852,10 +872,11 @@
       <c r="U14" s="4"/>
       <c r="V14" s="4"/>
       <c r="W14" s="4"/>
+      <c r="X14" s="4"/>
     </row>
     <row r="15" ht="15.75" customHeight="1">
       <c r="A15" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
@@ -871,7 +892,7 @@
       <c r="M15" s="1"/>
       <c r="N15" s="1"/>
       <c r="O15" s="1"/>
-      <c r="P15" s="4"/>
+      <c r="P15" s="1"/>
       <c r="Q15" s="4"/>
       <c r="R15" s="4"/>
       <c r="S15" s="4"/>
@@ -879,10 +900,11 @@
       <c r="U15" s="4"/>
       <c r="V15" s="4"/>
       <c r="W15" s="4"/>
+      <c r="X15" s="4"/>
     </row>
     <row r="16" ht="15.75" customHeight="1">
       <c r="A16" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B16" s="1"/>
       <c r="C16" s="1"/>
@@ -898,7 +920,7 @@
       <c r="M16" s="1"/>
       <c r="N16" s="1"/>
       <c r="O16" s="1"/>
-      <c r="P16" s="4"/>
+      <c r="P16" s="1"/>
       <c r="Q16" s="4"/>
       <c r="R16" s="4"/>
       <c r="S16" s="4"/>
@@ -906,10 +928,11 @@
       <c r="U16" s="4"/>
       <c r="V16" s="4"/>
       <c r="W16" s="4"/>
+      <c r="X16" s="4"/>
     </row>
     <row r="17" ht="15.75" customHeight="1">
       <c r="A17" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B17" s="1"/>
       <c r="C17" s="1"/>
@@ -925,7 +948,7 @@
       <c r="M17" s="1"/>
       <c r="N17" s="1"/>
       <c r="O17" s="1"/>
-      <c r="P17" s="4"/>
+      <c r="P17" s="1"/>
       <c r="Q17" s="4"/>
       <c r="R17" s="4"/>
       <c r="S17" s="4"/>
@@ -933,10 +956,11 @@
       <c r="U17" s="4"/>
       <c r="V17" s="4"/>
       <c r="W17" s="4"/>
+      <c r="X17" s="4"/>
     </row>
     <row r="18" ht="15.75" customHeight="1">
       <c r="A18" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B18" s="1"/>
       <c r="C18" s="1"/>
@@ -952,7 +976,7 @@
       <c r="M18" s="1"/>
       <c r="N18" s="1"/>
       <c r="O18" s="1"/>
-      <c r="P18" s="4"/>
+      <c r="P18" s="1"/>
       <c r="Q18" s="4"/>
       <c r="R18" s="4"/>
       <c r="S18" s="4"/>
@@ -960,10 +984,11 @@
       <c r="U18" s="4"/>
       <c r="V18" s="4"/>
       <c r="W18" s="4"/>
+      <c r="X18" s="4"/>
     </row>
     <row r="19" ht="15.75" customHeight="1">
       <c r="A19" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B19" s="1"/>
       <c r="C19" s="1"/>
@@ -979,7 +1004,7 @@
       <c r="M19" s="1"/>
       <c r="N19" s="1"/>
       <c r="O19" s="1"/>
-      <c r="P19" s="4"/>
+      <c r="P19" s="1"/>
       <c r="Q19" s="4"/>
       <c r="R19" s="4"/>
       <c r="S19" s="4"/>
@@ -987,10 +1012,11 @@
       <c r="U19" s="4"/>
       <c r="V19" s="4"/>
       <c r="W19" s="4"/>
+      <c r="X19" s="4"/>
     </row>
     <row r="20" ht="15.75" customHeight="1">
       <c r="A20" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B20" s="1"/>
       <c r="C20" s="1"/>
@@ -1006,7 +1032,7 @@
       <c r="M20" s="1"/>
       <c r="N20" s="1"/>
       <c r="O20" s="1"/>
-      <c r="P20" s="4"/>
+      <c r="P20" s="1"/>
       <c r="Q20" s="4"/>
       <c r="R20" s="4"/>
       <c r="S20" s="4"/>
@@ -1014,6 +1040,7 @@
       <c r="U20" s="4"/>
       <c r="V20" s="4"/>
       <c r="W20" s="4"/>
+      <c r="X20" s="4"/>
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="4"/>
@@ -1039,6 +1066,7 @@
       <c r="U21" s="4"/>
       <c r="V21" s="4"/>
       <c r="W21" s="4"/>
+      <c r="X21" s="4"/>
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="4"/>
@@ -1064,6 +1092,7 @@
       <c r="U22" s="4"/>
       <c r="V22" s="4"/>
       <c r="W22" s="4"/>
+      <c r="X22" s="4"/>
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="4"/>
@@ -1089,6 +1118,7 @@
       <c r="U23" s="4"/>
       <c r="V23" s="4"/>
       <c r="W23" s="4"/>
+      <c r="X23" s="4"/>
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="4"/>
@@ -1114,6 +1144,7 @@
       <c r="U24" s="4"/>
       <c r="V24" s="4"/>
       <c r="W24" s="4"/>
+      <c r="X24" s="4"/>
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="4"/>
@@ -1139,6 +1170,7 @@
       <c r="U25" s="4"/>
       <c r="V25" s="4"/>
       <c r="W25" s="4"/>
+      <c r="X25" s="4"/>
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="4"/>
@@ -1164,6 +1196,7 @@
       <c r="U26" s="4"/>
       <c r="V26" s="4"/>
       <c r="W26" s="4"/>
+      <c r="X26" s="4"/>
     </row>
     <row r="27" ht="15.75" customHeight="1">
       <c r="A27" s="4"/>
@@ -1189,6 +1222,7 @@
       <c r="U27" s="4"/>
       <c r="V27" s="4"/>
       <c r="W27" s="4"/>
+      <c r="X27" s="4"/>
     </row>
     <row r="28" ht="15.75" customHeight="1">
       <c r="A28" s="4"/>
@@ -1214,6 +1248,7 @@
       <c r="U28" s="4"/>
       <c r="V28" s="4"/>
       <c r="W28" s="4"/>
+      <c r="X28" s="4"/>
     </row>
     <row r="29" ht="15.75" customHeight="1">
       <c r="A29" s="4"/>
@@ -1239,6 +1274,7 @@
       <c r="U29" s="4"/>
       <c r="V29" s="4"/>
       <c r="W29" s="4"/>
+      <c r="X29" s="4"/>
     </row>
     <row r="30" ht="15.75" customHeight="1">
       <c r="A30" s="4"/>
@@ -1264,6 +1300,7 @@
       <c r="U30" s="4"/>
       <c r="V30" s="4"/>
       <c r="W30" s="4"/>
+      <c r="X30" s="4"/>
     </row>
     <row r="31" ht="15.75" customHeight="1">
       <c r="A31" s="4"/>
@@ -1289,6 +1326,7 @@
       <c r="U31" s="4"/>
       <c r="V31" s="4"/>
       <c r="W31" s="4"/>
+      <c r="X31" s="4"/>
     </row>
     <row r="32" ht="15.75" customHeight="1">
       <c r="A32" s="4"/>
@@ -1314,6 +1352,7 @@
       <c r="U32" s="4"/>
       <c r="V32" s="4"/>
       <c r="W32" s="4"/>
+      <c r="X32" s="4"/>
     </row>
     <row r="33" ht="15.75" customHeight="1">
       <c r="A33" s="4"/>
@@ -1339,6 +1378,7 @@
       <c r="U33" s="4"/>
       <c r="V33" s="4"/>
       <c r="W33" s="4"/>
+      <c r="X33" s="4"/>
     </row>
     <row r="34" ht="15.75" customHeight="1">
       <c r="A34" s="4"/>
@@ -1364,6 +1404,7 @@
       <c r="U34" s="4"/>
       <c r="V34" s="4"/>
       <c r="W34" s="4"/>
+      <c r="X34" s="4"/>
     </row>
     <row r="35" ht="15.75" customHeight="1">
       <c r="A35" s="4"/>
@@ -1389,6 +1430,7 @@
       <c r="U35" s="4"/>
       <c r="V35" s="4"/>
       <c r="W35" s="4"/>
+      <c r="X35" s="4"/>
     </row>
     <row r="36" ht="15.75" customHeight="1">
       <c r="A36" s="4"/>
@@ -1414,6 +1456,7 @@
       <c r="U36" s="4"/>
       <c r="V36" s="4"/>
       <c r="W36" s="4"/>
+      <c r="X36" s="4"/>
     </row>
     <row r="37" ht="15.75" customHeight="1">
       <c r="A37" s="4"/>
@@ -1439,6 +1482,7 @@
       <c r="U37" s="4"/>
       <c r="V37" s="4"/>
       <c r="W37" s="4"/>
+      <c r="X37" s="4"/>
     </row>
     <row r="38" ht="15.75" customHeight="1">
       <c r="A38" s="4"/>
@@ -1464,6 +1508,7 @@
       <c r="U38" s="4"/>
       <c r="V38" s="4"/>
       <c r="W38" s="4"/>
+      <c r="X38" s="4"/>
     </row>
     <row r="39" ht="15.75" customHeight="1">
       <c r="A39" s="4"/>
@@ -1489,6 +1534,7 @@
       <c r="U39" s="4"/>
       <c r="V39" s="4"/>
       <c r="W39" s="4"/>
+      <c r="X39" s="4"/>
     </row>
     <row r="40" ht="15.75" customHeight="1">
       <c r="A40" s="4"/>
@@ -1514,6 +1560,7 @@
       <c r="U40" s="4"/>
       <c r="V40" s="4"/>
       <c r="W40" s="4"/>
+      <c r="X40" s="4"/>
     </row>
     <row r="41" ht="15.75" customHeight="1">
       <c r="A41" s="4"/>
@@ -1539,6 +1586,7 @@
       <c r="U41" s="4"/>
       <c r="V41" s="4"/>
       <c r="W41" s="4"/>
+      <c r="X41" s="4"/>
     </row>
     <row r="42" ht="15.75" customHeight="1">
       <c r="A42" s="4"/>
@@ -1564,6 +1612,7 @@
       <c r="U42" s="4"/>
       <c r="V42" s="4"/>
       <c r="W42" s="4"/>
+      <c r="X42" s="4"/>
     </row>
     <row r="43" ht="15.75" customHeight="1">
       <c r="A43" s="4"/>
@@ -1589,6 +1638,7 @@
       <c r="U43" s="4"/>
       <c r="V43" s="4"/>
       <c r="W43" s="4"/>
+      <c r="X43" s="4"/>
     </row>
     <row r="44" ht="15.75" customHeight="1">
       <c r="A44" s="4"/>
@@ -1614,6 +1664,7 @@
       <c r="U44" s="4"/>
       <c r="V44" s="4"/>
       <c r="W44" s="4"/>
+      <c r="X44" s="4"/>
     </row>
     <row r="45" ht="15.75" customHeight="1">
       <c r="A45" s="4"/>
@@ -1639,6 +1690,7 @@
       <c r="U45" s="4"/>
       <c r="V45" s="4"/>
       <c r="W45" s="4"/>
+      <c r="X45" s="4"/>
     </row>
     <row r="46" ht="15.75" customHeight="1">
       <c r="A46" s="4"/>
@@ -1664,6 +1716,7 @@
       <c r="U46" s="4"/>
       <c r="V46" s="4"/>
       <c r="W46" s="4"/>
+      <c r="X46" s="4"/>
     </row>
     <row r="47" ht="15.75" customHeight="1">
       <c r="A47" s="4"/>
@@ -1689,6 +1742,7 @@
       <c r="U47" s="4"/>
       <c r="V47" s="4"/>
       <c r="W47" s="4"/>
+      <c r="X47" s="4"/>
     </row>
     <row r="48" ht="15.75" customHeight="1">
       <c r="A48" s="4"/>
@@ -1714,6 +1768,7 @@
       <c r="U48" s="4"/>
       <c r="V48" s="4"/>
       <c r="W48" s="4"/>
+      <c r="X48" s="4"/>
     </row>
     <row r="49" ht="15.75" customHeight="1">
       <c r="A49" s="4"/>
@@ -1739,6 +1794,7 @@
       <c r="U49" s="4"/>
       <c r="V49" s="4"/>
       <c r="W49" s="4"/>
+      <c r="X49" s="4"/>
     </row>
     <row r="50" ht="15.75" customHeight="1">
       <c r="A50" s="4"/>
@@ -1764,6 +1820,7 @@
       <c r="U50" s="4"/>
       <c r="V50" s="4"/>
       <c r="W50" s="4"/>
+      <c r="X50" s="4"/>
     </row>
     <row r="51" ht="15.75" customHeight="1">
       <c r="A51" s="4"/>
@@ -1789,6 +1846,7 @@
       <c r="U51" s="4"/>
       <c r="V51" s="4"/>
       <c r="W51" s="4"/>
+      <c r="X51" s="4"/>
     </row>
     <row r="52" ht="15.75" customHeight="1">
       <c r="A52" s="4"/>
@@ -1814,6 +1872,7 @@
       <c r="U52" s="4"/>
       <c r="V52" s="4"/>
       <c r="W52" s="4"/>
+      <c r="X52" s="4"/>
     </row>
     <row r="53" ht="15.75" customHeight="1">
       <c r="A53" s="4"/>
@@ -1839,6 +1898,7 @@
       <c r="U53" s="4"/>
       <c r="V53" s="4"/>
       <c r="W53" s="4"/>
+      <c r="X53" s="4"/>
     </row>
     <row r="54" ht="15.75" customHeight="1">
       <c r="A54" s="4"/>
@@ -1864,6 +1924,7 @@
       <c r="U54" s="4"/>
       <c r="V54" s="4"/>
       <c r="W54" s="4"/>
+      <c r="X54" s="4"/>
     </row>
     <row r="55" ht="15.75" customHeight="1">
       <c r="A55" s="4"/>
@@ -1889,6 +1950,7 @@
       <c r="U55" s="4"/>
       <c r="V55" s="4"/>
       <c r="W55" s="4"/>
+      <c r="X55" s="4"/>
     </row>
     <row r="56" ht="15.75" customHeight="1">
       <c r="A56" s="4"/>
@@ -1914,6 +1976,7 @@
       <c r="U56" s="4"/>
       <c r="V56" s="4"/>
       <c r="W56" s="4"/>
+      <c r="X56" s="4"/>
     </row>
     <row r="57" ht="15.75" customHeight="1">
       <c r="A57" s="4"/>
@@ -1939,6 +2002,7 @@
       <c r="U57" s="4"/>
       <c r="V57" s="4"/>
       <c r="W57" s="4"/>
+      <c r="X57" s="4"/>
     </row>
     <row r="58" ht="15.75" customHeight="1">
       <c r="A58" s="4"/>
@@ -1964,6 +2028,7 @@
       <c r="U58" s="4"/>
       <c r="V58" s="4"/>
       <c r="W58" s="4"/>
+      <c r="X58" s="4"/>
     </row>
     <row r="59" ht="15.75" customHeight="1">
       <c r="A59" s="4"/>
@@ -1989,6 +2054,7 @@
       <c r="U59" s="4"/>
       <c r="V59" s="4"/>
       <c r="W59" s="4"/>
+      <c r="X59" s="4"/>
     </row>
     <row r="60" ht="15.75" customHeight="1">
       <c r="A60" s="4"/>
@@ -2014,6 +2080,7 @@
       <c r="U60" s="4"/>
       <c r="V60" s="4"/>
       <c r="W60" s="4"/>
+      <c r="X60" s="4"/>
     </row>
     <row r="61" ht="15.75" customHeight="1">
       <c r="A61" s="4"/>
@@ -2039,6 +2106,7 @@
       <c r="U61" s="4"/>
       <c r="V61" s="4"/>
       <c r="W61" s="4"/>
+      <c r="X61" s="4"/>
     </row>
     <row r="62" ht="15.75" customHeight="1">
       <c r="A62" s="4"/>
@@ -2064,6 +2132,7 @@
       <c r="U62" s="4"/>
       <c r="V62" s="4"/>
       <c r="W62" s="4"/>
+      <c r="X62" s="4"/>
     </row>
     <row r="63" ht="15.75" customHeight="1">
       <c r="A63" s="4"/>
@@ -2089,6 +2158,7 @@
       <c r="U63" s="4"/>
       <c r="V63" s="4"/>
       <c r="W63" s="4"/>
+      <c r="X63" s="4"/>
     </row>
     <row r="64" ht="15.75" customHeight="1">
       <c r="A64" s="4"/>
@@ -2114,6 +2184,7 @@
       <c r="U64" s="4"/>
       <c r="V64" s="4"/>
       <c r="W64" s="4"/>
+      <c r="X64" s="4"/>
     </row>
     <row r="65" ht="15.75" customHeight="1">
       <c r="A65" s="4"/>
@@ -2139,6 +2210,7 @@
       <c r="U65" s="4"/>
       <c r="V65" s="4"/>
       <c r="W65" s="4"/>
+      <c r="X65" s="4"/>
     </row>
     <row r="66" ht="15.75" customHeight="1">
       <c r="A66" s="4"/>
@@ -2164,6 +2236,7 @@
       <c r="U66" s="4"/>
       <c r="V66" s="4"/>
       <c r="W66" s="4"/>
+      <c r="X66" s="4"/>
     </row>
     <row r="67" ht="15.75" customHeight="1">
       <c r="A67" s="4"/>
@@ -2189,6 +2262,7 @@
       <c r="U67" s="4"/>
       <c r="V67" s="4"/>
       <c r="W67" s="4"/>
+      <c r="X67" s="4"/>
     </row>
     <row r="68" ht="15.75" customHeight="1">
       <c r="A68" s="4"/>
@@ -2214,6 +2288,7 @@
       <c r="U68" s="4"/>
       <c r="V68" s="4"/>
       <c r="W68" s="4"/>
+      <c r="X68" s="4"/>
     </row>
     <row r="69" ht="15.75" customHeight="1">
       <c r="A69" s="4"/>
@@ -2239,6 +2314,7 @@
       <c r="U69" s="4"/>
       <c r="V69" s="4"/>
       <c r="W69" s="4"/>
+      <c r="X69" s="4"/>
     </row>
     <row r="70" ht="15.75" customHeight="1">
       <c r="A70" s="4"/>
@@ -2264,6 +2340,7 @@
       <c r="U70" s="4"/>
       <c r="V70" s="4"/>
       <c r="W70" s="4"/>
+      <c r="X70" s="4"/>
     </row>
     <row r="71" ht="15.75" customHeight="1">
       <c r="A71" s="4"/>
@@ -2289,6 +2366,7 @@
       <c r="U71" s="4"/>
       <c r="V71" s="4"/>
       <c r="W71" s="4"/>
+      <c r="X71" s="4"/>
     </row>
     <row r="72" ht="15.75" customHeight="1">
       <c r="A72" s="4"/>
@@ -2314,6 +2392,7 @@
       <c r="U72" s="4"/>
       <c r="V72" s="4"/>
       <c r="W72" s="4"/>
+      <c r="X72" s="4"/>
     </row>
     <row r="73" ht="15.75" customHeight="1">
       <c r="A73" s="4"/>
@@ -2339,6 +2418,7 @@
       <c r="U73" s="4"/>
       <c r="V73" s="4"/>
       <c r="W73" s="4"/>
+      <c r="X73" s="4"/>
     </row>
     <row r="74" ht="15.75" customHeight="1">
       <c r="A74" s="4"/>
@@ -2364,6 +2444,7 @@
       <c r="U74" s="4"/>
       <c r="V74" s="4"/>
       <c r="W74" s="4"/>
+      <c r="X74" s="4"/>
     </row>
     <row r="75" ht="15.75" customHeight="1">
       <c r="A75" s="4"/>
@@ -2389,6 +2470,7 @@
       <c r="U75" s="4"/>
       <c r="V75" s="4"/>
       <c r="W75" s="4"/>
+      <c r="X75" s="4"/>
     </row>
     <row r="76" ht="15.75" customHeight="1">
       <c r="A76" s="4"/>
@@ -2414,6 +2496,7 @@
       <c r="U76" s="4"/>
       <c r="V76" s="4"/>
       <c r="W76" s="4"/>
+      <c r="X76" s="4"/>
     </row>
     <row r="77" ht="15.75" customHeight="1">
       <c r="A77" s="4"/>
@@ -2439,6 +2522,7 @@
       <c r="U77" s="4"/>
       <c r="V77" s="4"/>
       <c r="W77" s="4"/>
+      <c r="X77" s="4"/>
     </row>
     <row r="78" ht="15.75" customHeight="1">
       <c r="A78" s="4"/>
@@ -2464,6 +2548,7 @@
       <c r="U78" s="4"/>
       <c r="V78" s="4"/>
       <c r="W78" s="4"/>
+      <c r="X78" s="4"/>
     </row>
     <row r="79" ht="15.75" customHeight="1">
       <c r="A79" s="4"/>
@@ -2489,6 +2574,7 @@
       <c r="U79" s="4"/>
       <c r="V79" s="4"/>
       <c r="W79" s="4"/>
+      <c r="X79" s="4"/>
     </row>
     <row r="80" ht="15.75" customHeight="1">
       <c r="A80" s="4"/>
@@ -2514,6 +2600,7 @@
       <c r="U80" s="4"/>
       <c r="V80" s="4"/>
       <c r="W80" s="4"/>
+      <c r="X80" s="4"/>
     </row>
     <row r="81" ht="15.75" customHeight="1">
       <c r="A81" s="4"/>
@@ -2539,6 +2626,7 @@
       <c r="U81" s="4"/>
       <c r="V81" s="4"/>
       <c r="W81" s="4"/>
+      <c r="X81" s="4"/>
     </row>
     <row r="82" ht="15.75" customHeight="1">
       <c r="A82" s="4"/>
@@ -2564,6 +2652,7 @@
       <c r="U82" s="4"/>
       <c r="V82" s="4"/>
       <c r="W82" s="4"/>
+      <c r="X82" s="4"/>
     </row>
     <row r="83" ht="15.75" customHeight="1">
       <c r="A83" s="4"/>
@@ -2589,6 +2678,7 @@
       <c r="U83" s="4"/>
       <c r="V83" s="4"/>
       <c r="W83" s="4"/>
+      <c r="X83" s="4"/>
     </row>
     <row r="84" ht="15.75" customHeight="1">
       <c r="A84" s="4"/>
@@ -2614,6 +2704,7 @@
       <c r="U84" s="4"/>
       <c r="V84" s="4"/>
       <c r="W84" s="4"/>
+      <c r="X84" s="4"/>
     </row>
     <row r="85" ht="15.75" customHeight="1">
       <c r="A85" s="4"/>
@@ -2639,6 +2730,7 @@
       <c r="U85" s="4"/>
       <c r="V85" s="4"/>
       <c r="W85" s="4"/>
+      <c r="X85" s="4"/>
     </row>
     <row r="86" ht="15.75" customHeight="1">
       <c r="A86" s="4"/>
@@ -2664,6 +2756,7 @@
       <c r="U86" s="4"/>
       <c r="V86" s="4"/>
       <c r="W86" s="4"/>
+      <c r="X86" s="4"/>
     </row>
     <row r="87" ht="15.75" customHeight="1">
       <c r="A87" s="4"/>
@@ -2689,6 +2782,7 @@
       <c r="U87" s="4"/>
       <c r="V87" s="4"/>
       <c r="W87" s="4"/>
+      <c r="X87" s="4"/>
     </row>
     <row r="88" ht="15.75" customHeight="1">
       <c r="A88" s="4"/>
@@ -2714,6 +2808,7 @@
       <c r="U88" s="4"/>
       <c r="V88" s="4"/>
       <c r="W88" s="4"/>
+      <c r="X88" s="4"/>
     </row>
     <row r="89" ht="15.75" customHeight="1">
       <c r="A89" s="4"/>
@@ -2739,6 +2834,7 @@
       <c r="U89" s="4"/>
       <c r="V89" s="4"/>
       <c r="W89" s="4"/>
+      <c r="X89" s="4"/>
     </row>
     <row r="90" ht="15.75" customHeight="1">
       <c r="A90" s="4"/>
@@ -2764,6 +2860,7 @@
       <c r="U90" s="4"/>
       <c r="V90" s="4"/>
       <c r="W90" s="4"/>
+      <c r="X90" s="4"/>
     </row>
     <row r="91" ht="15.75" customHeight="1">
       <c r="A91" s="4"/>
@@ -2789,6 +2886,7 @@
       <c r="U91" s="4"/>
       <c r="V91" s="4"/>
       <c r="W91" s="4"/>
+      <c r="X91" s="4"/>
     </row>
     <row r="92" ht="15.75" customHeight="1">
       <c r="A92" s="4"/>
@@ -2814,6 +2912,7 @@
       <c r="U92" s="4"/>
       <c r="V92" s="4"/>
       <c r="W92" s="4"/>
+      <c r="X92" s="4"/>
     </row>
     <row r="93" ht="15.75" customHeight="1">
       <c r="A93" s="4"/>
@@ -2839,6 +2938,7 @@
       <c r="U93" s="4"/>
       <c r="V93" s="4"/>
       <c r="W93" s="4"/>
+      <c r="X93" s="4"/>
     </row>
     <row r="94" ht="15.75" customHeight="1">
       <c r="A94" s="4"/>
@@ -2864,6 +2964,7 @@
       <c r="U94" s="4"/>
       <c r="V94" s="4"/>
       <c r="W94" s="4"/>
+      <c r="X94" s="4"/>
     </row>
     <row r="95" ht="15.75" customHeight="1">
       <c r="A95" s="4"/>
@@ -2889,6 +2990,7 @@
       <c r="U95" s="4"/>
       <c r="V95" s="4"/>
       <c r="W95" s="4"/>
+      <c r="X95" s="4"/>
     </row>
     <row r="96" ht="15.75" customHeight="1">
       <c r="A96" s="4"/>
@@ -2914,6 +3016,7 @@
       <c r="U96" s="4"/>
       <c r="V96" s="4"/>
       <c r="W96" s="4"/>
+      <c r="X96" s="4"/>
     </row>
     <row r="97" ht="15.75" customHeight="1">
       <c r="A97" s="4"/>
@@ -2939,6 +3042,7 @@
       <c r="U97" s="4"/>
       <c r="V97" s="4"/>
       <c r="W97" s="4"/>
+      <c r="X97" s="4"/>
     </row>
     <row r="98" ht="15.75" customHeight="1">
       <c r="A98" s="4"/>
@@ -2964,6 +3068,7 @@
       <c r="U98" s="4"/>
       <c r="V98" s="4"/>
       <c r="W98" s="4"/>
+      <c r="X98" s="4"/>
     </row>
     <row r="99" ht="15.75" customHeight="1">
       <c r="A99" s="4"/>
@@ -2989,6 +3094,7 @@
       <c r="U99" s="4"/>
       <c r="V99" s="4"/>
       <c r="W99" s="4"/>
+      <c r="X99" s="4"/>
     </row>
     <row r="100" ht="15.75" customHeight="1">
       <c r="A100" s="4"/>
@@ -3014,6 +3120,7 @@
       <c r="U100" s="4"/>
       <c r="V100" s="4"/>
       <c r="W100" s="4"/>
+      <c r="X100" s="4"/>
     </row>
     <row r="101" ht="15.75" customHeight="1">
       <c r="A101" s="4"/>
@@ -3039,6 +3146,7 @@
       <c r="U101" s="4"/>
       <c r="V101" s="4"/>
       <c r="W101" s="4"/>
+      <c r="X101" s="4"/>
     </row>
     <row r="102" ht="15.75" customHeight="1">
       <c r="A102" s="4"/>
@@ -3064,6 +3172,7 @@
       <c r="U102" s="4"/>
       <c r="V102" s="4"/>
       <c r="W102" s="4"/>
+      <c r="X102" s="4"/>
     </row>
     <row r="103" ht="15.75" customHeight="1">
       <c r="A103" s="4"/>
@@ -3089,6 +3198,7 @@
       <c r="U103" s="4"/>
       <c r="V103" s="4"/>
       <c r="W103" s="4"/>
+      <c r="X103" s="4"/>
     </row>
     <row r="104" ht="15.75" customHeight="1">
       <c r="A104" s="4"/>
@@ -3114,6 +3224,7 @@
       <c r="U104" s="4"/>
       <c r="V104" s="4"/>
       <c r="W104" s="4"/>
+      <c r="X104" s="4"/>
     </row>
     <row r="105" ht="15.75" customHeight="1">
       <c r="A105" s="4"/>
@@ -3139,6 +3250,7 @@
       <c r="U105" s="4"/>
       <c r="V105" s="4"/>
       <c r="W105" s="4"/>
+      <c r="X105" s="4"/>
     </row>
     <row r="106" ht="15.75" customHeight="1">
       <c r="A106" s="4"/>
@@ -3164,6 +3276,7 @@
       <c r="U106" s="4"/>
       <c r="V106" s="4"/>
       <c r="W106" s="4"/>
+      <c r="X106" s="4"/>
     </row>
     <row r="107" ht="15.75" customHeight="1">
       <c r="A107" s="4"/>
@@ -3189,6 +3302,7 @@
       <c r="U107" s="4"/>
       <c r="V107" s="4"/>
       <c r="W107" s="4"/>
+      <c r="X107" s="4"/>
     </row>
     <row r="108" ht="15.75" customHeight="1">
       <c r="A108" s="4"/>
@@ -3214,6 +3328,7 @@
       <c r="U108" s="4"/>
       <c r="V108" s="4"/>
       <c r="W108" s="4"/>
+      <c r="X108" s="4"/>
     </row>
     <row r="109" ht="15.75" customHeight="1">
       <c r="A109" s="4"/>
@@ -3239,6 +3354,7 @@
       <c r="U109" s="4"/>
       <c r="V109" s="4"/>
       <c r="W109" s="4"/>
+      <c r="X109" s="4"/>
     </row>
     <row r="110" ht="15.75" customHeight="1">
       <c r="A110" s="4"/>
@@ -3264,6 +3380,7 @@
       <c r="U110" s="4"/>
       <c r="V110" s="4"/>
       <c r="W110" s="4"/>
+      <c r="X110" s="4"/>
     </row>
     <row r="111" ht="15.75" customHeight="1">
       <c r="A111" s="4"/>
@@ -3289,6 +3406,7 @@
       <c r="U111" s="4"/>
       <c r="V111" s="4"/>
       <c r="W111" s="4"/>
+      <c r="X111" s="4"/>
     </row>
     <row r="112" ht="15.75" customHeight="1">
       <c r="A112" s="4"/>
@@ -3314,6 +3432,7 @@
       <c r="U112" s="4"/>
       <c r="V112" s="4"/>
       <c r="W112" s="4"/>
+      <c r="X112" s="4"/>
     </row>
     <row r="113" ht="15.75" customHeight="1">
       <c r="A113" s="4"/>
@@ -3339,6 +3458,7 @@
       <c r="U113" s="4"/>
       <c r="V113" s="4"/>
       <c r="W113" s="4"/>
+      <c r="X113" s="4"/>
     </row>
     <row r="114" ht="15.75" customHeight="1">
       <c r="A114" s="4"/>
@@ -3364,6 +3484,7 @@
       <c r="U114" s="4"/>
       <c r="V114" s="4"/>
       <c r="W114" s="4"/>
+      <c r="X114" s="4"/>
     </row>
     <row r="115" ht="15.75" customHeight="1">
       <c r="A115" s="4"/>
@@ -3389,6 +3510,7 @@
       <c r="U115" s="4"/>
       <c r="V115" s="4"/>
       <c r="W115" s="4"/>
+      <c r="X115" s="4"/>
     </row>
     <row r="116" ht="15.75" customHeight="1">
       <c r="A116" s="4"/>
@@ -3414,6 +3536,7 @@
       <c r="U116" s="4"/>
       <c r="V116" s="4"/>
       <c r="W116" s="4"/>
+      <c r="X116" s="4"/>
     </row>
     <row r="117" ht="15.75" customHeight="1">
       <c r="A117" s="4"/>
@@ -3439,6 +3562,7 @@
       <c r="U117" s="4"/>
       <c r="V117" s="4"/>
       <c r="W117" s="4"/>
+      <c r="X117" s="4"/>
     </row>
     <row r="118" ht="15.75" customHeight="1">
       <c r="A118" s="4"/>
@@ -3464,6 +3588,7 @@
       <c r="U118" s="4"/>
       <c r="V118" s="4"/>
       <c r="W118" s="4"/>
+      <c r="X118" s="4"/>
     </row>
     <row r="119" ht="15.75" customHeight="1">
       <c r="A119" s="4"/>
@@ -3489,6 +3614,7 @@
       <c r="U119" s="4"/>
       <c r="V119" s="4"/>
       <c r="W119" s="4"/>
+      <c r="X119" s="4"/>
     </row>
     <row r="120" ht="15.75" customHeight="1">
       <c r="A120" s="4"/>
@@ -3514,6 +3640,7 @@
       <c r="U120" s="4"/>
       <c r="V120" s="4"/>
       <c r="W120" s="4"/>
+      <c r="X120" s="4"/>
     </row>
     <row r="121" ht="15.75" customHeight="1">
       <c r="A121" s="4"/>
@@ -3539,6 +3666,7 @@
       <c r="U121" s="4"/>
       <c r="V121" s="4"/>
       <c r="W121" s="4"/>
+      <c r="X121" s="4"/>
     </row>
     <row r="122" ht="15.75" customHeight="1">
       <c r="A122" s="4"/>
@@ -3564,6 +3692,7 @@
       <c r="U122" s="4"/>
       <c r="V122" s="4"/>
       <c r="W122" s="4"/>
+      <c r="X122" s="4"/>
     </row>
     <row r="123" ht="15.75" customHeight="1">
       <c r="A123" s="4"/>
@@ -3589,6 +3718,7 @@
       <c r="U123" s="4"/>
       <c r="V123" s="4"/>
       <c r="W123" s="4"/>
+      <c r="X123" s="4"/>
     </row>
     <row r="124" ht="15.75" customHeight="1">
       <c r="A124" s="4"/>
@@ -3614,6 +3744,7 @@
       <c r="U124" s="4"/>
       <c r="V124" s="4"/>
       <c r="W124" s="4"/>
+      <c r="X124" s="4"/>
     </row>
     <row r="125" ht="15.75" customHeight="1">
       <c r="A125" s="4"/>
@@ -3639,6 +3770,7 @@
       <c r="U125" s="4"/>
       <c r="V125" s="4"/>
       <c r="W125" s="4"/>
+      <c r="X125" s="4"/>
     </row>
     <row r="126" ht="15.75" customHeight="1">
       <c r="A126" s="4"/>
@@ -3664,6 +3796,7 @@
       <c r="U126" s="4"/>
       <c r="V126" s="4"/>
       <c r="W126" s="4"/>
+      <c r="X126" s="4"/>
     </row>
     <row r="127" ht="15.75" customHeight="1">
       <c r="A127" s="4"/>
@@ -3689,6 +3822,7 @@
       <c r="U127" s="4"/>
       <c r="V127" s="4"/>
       <c r="W127" s="4"/>
+      <c r="X127" s="4"/>
     </row>
     <row r="128" ht="15.75" customHeight="1">
       <c r="A128" s="4"/>
@@ -3714,6 +3848,7 @@
       <c r="U128" s="4"/>
       <c r="V128" s="4"/>
       <c r="W128" s="4"/>
+      <c r="X128" s="4"/>
     </row>
     <row r="129" ht="15.75" customHeight="1">
       <c r="A129" s="4"/>
@@ -3739,6 +3874,7 @@
       <c r="U129" s="4"/>
       <c r="V129" s="4"/>
       <c r="W129" s="4"/>
+      <c r="X129" s="4"/>
     </row>
     <row r="130" ht="15.75" customHeight="1">
       <c r="A130" s="4"/>
@@ -3764,6 +3900,7 @@
       <c r="U130" s="4"/>
       <c r="V130" s="4"/>
       <c r="W130" s="4"/>
+      <c r="X130" s="4"/>
     </row>
     <row r="131" ht="15.75" customHeight="1">
       <c r="A131" s="4"/>
@@ -3789,6 +3926,7 @@
       <c r="U131" s="4"/>
       <c r="V131" s="4"/>
       <c r="W131" s="4"/>
+      <c r="X131" s="4"/>
     </row>
     <row r="132" ht="15.75" customHeight="1">
       <c r="A132" s="4"/>
@@ -3814,6 +3952,7 @@
       <c r="U132" s="4"/>
       <c r="V132" s="4"/>
       <c r="W132" s="4"/>
+      <c r="X132" s="4"/>
     </row>
     <row r="133" ht="15.75" customHeight="1">
       <c r="A133" s="4"/>
@@ -3839,6 +3978,7 @@
       <c r="U133" s="4"/>
       <c r="V133" s="4"/>
       <c r="W133" s="4"/>
+      <c r="X133" s="4"/>
     </row>
     <row r="134" ht="15.75" customHeight="1">
       <c r="A134" s="4"/>
@@ -3864,6 +4004,7 @@
       <c r="U134" s="4"/>
       <c r="V134" s="4"/>
       <c r="W134" s="4"/>
+      <c r="X134" s="4"/>
     </row>
     <row r="135" ht="15.75" customHeight="1">
       <c r="A135" s="4"/>
@@ -3889,6 +4030,7 @@
       <c r="U135" s="4"/>
       <c r="V135" s="4"/>
       <c r="W135" s="4"/>
+      <c r="X135" s="4"/>
     </row>
     <row r="136" ht="15.75" customHeight="1">
       <c r="A136" s="4"/>
@@ -3914,6 +4056,7 @@
       <c r="U136" s="4"/>
       <c r="V136" s="4"/>
       <c r="W136" s="4"/>
+      <c r="X136" s="4"/>
     </row>
     <row r="137" ht="15.75" customHeight="1">
       <c r="A137" s="4"/>
@@ -3939,6 +4082,7 @@
       <c r="U137" s="4"/>
       <c r="V137" s="4"/>
       <c r="W137" s="4"/>
+      <c r="X137" s="4"/>
     </row>
     <row r="138" ht="15.75" customHeight="1">
       <c r="A138" s="4"/>
@@ -3964,6 +4108,7 @@
       <c r="U138" s="4"/>
       <c r="V138" s="4"/>
       <c r="W138" s="4"/>
+      <c r="X138" s="4"/>
     </row>
     <row r="139" ht="15.75" customHeight="1">
       <c r="A139" s="4"/>
@@ -3989,6 +4134,7 @@
       <c r="U139" s="4"/>
       <c r="V139" s="4"/>
       <c r="W139" s="4"/>
+      <c r="X139" s="4"/>
     </row>
     <row r="140" ht="15.75" customHeight="1">
       <c r="A140" s="4"/>
@@ -4014,6 +4160,7 @@
       <c r="U140" s="4"/>
       <c r="V140" s="4"/>
       <c r="W140" s="4"/>
+      <c r="X140" s="4"/>
     </row>
     <row r="141" ht="15.75" customHeight="1">
       <c r="A141" s="4"/>
@@ -4039,6 +4186,7 @@
       <c r="U141" s="4"/>
       <c r="V141" s="4"/>
       <c r="W141" s="4"/>
+      <c r="X141" s="4"/>
     </row>
     <row r="142" ht="15.75" customHeight="1">
       <c r="A142" s="4"/>
@@ -4064,6 +4212,7 @@
       <c r="U142" s="4"/>
       <c r="V142" s="4"/>
       <c r="W142" s="4"/>
+      <c r="X142" s="4"/>
     </row>
     <row r="143" ht="15.75" customHeight="1">
       <c r="A143" s="4"/>
@@ -4089,6 +4238,7 @@
       <c r="U143" s="4"/>
       <c r="V143" s="4"/>
       <c r="W143" s="4"/>
+      <c r="X143" s="4"/>
     </row>
     <row r="144" ht="15.75" customHeight="1">
       <c r="A144" s="4"/>
@@ -4114,6 +4264,7 @@
       <c r="U144" s="4"/>
       <c r="V144" s="4"/>
       <c r="W144" s="4"/>
+      <c r="X144" s="4"/>
     </row>
     <row r="145" ht="15.75" customHeight="1">
       <c r="A145" s="4"/>
@@ -4139,6 +4290,7 @@
       <c r="U145" s="4"/>
       <c r="V145" s="4"/>
       <c r="W145" s="4"/>
+      <c r="X145" s="4"/>
     </row>
     <row r="146" ht="15.75" customHeight="1">
       <c r="A146" s="4"/>
@@ -4164,6 +4316,7 @@
       <c r="U146" s="4"/>
       <c r="V146" s="4"/>
       <c r="W146" s="4"/>
+      <c r="X146" s="4"/>
     </row>
     <row r="147" ht="15.75" customHeight="1">
       <c r="A147" s="4"/>
@@ -4189,6 +4342,7 @@
       <c r="U147" s="4"/>
       <c r="V147" s="4"/>
       <c r="W147" s="4"/>
+      <c r="X147" s="4"/>
     </row>
     <row r="148" ht="15.75" customHeight="1">
       <c r="A148" s="4"/>
@@ -4214,6 +4368,7 @@
       <c r="U148" s="4"/>
       <c r="V148" s="4"/>
       <c r="W148" s="4"/>
+      <c r="X148" s="4"/>
     </row>
     <row r="149" ht="15.75" customHeight="1">
       <c r="A149" s="4"/>
@@ -4239,6 +4394,7 @@
       <c r="U149" s="4"/>
       <c r="V149" s="4"/>
       <c r="W149" s="4"/>
+      <c r="X149" s="4"/>
     </row>
     <row r="150" ht="15.75" customHeight="1">
       <c r="A150" s="4"/>
@@ -4264,6 +4420,7 @@
       <c r="U150" s="4"/>
       <c r="V150" s="4"/>
       <c r="W150" s="4"/>
+      <c r="X150" s="4"/>
     </row>
     <row r="151" ht="15.75" customHeight="1">
       <c r="A151" s="4"/>
@@ -4289,6 +4446,7 @@
       <c r="U151" s="4"/>
       <c r="V151" s="4"/>
       <c r="W151" s="4"/>
+      <c r="X151" s="4"/>
     </row>
     <row r="152" ht="15.75" customHeight="1">
       <c r="A152" s="4"/>
@@ -4314,6 +4472,7 @@
       <c r="U152" s="4"/>
       <c r="V152" s="4"/>
       <c r="W152" s="4"/>
+      <c r="X152" s="4"/>
     </row>
     <row r="153" ht="15.75" customHeight="1">
       <c r="A153" s="4"/>
@@ -4339,6 +4498,7 @@
       <c r="U153" s="4"/>
       <c r="V153" s="4"/>
       <c r="W153" s="4"/>
+      <c r="X153" s="4"/>
     </row>
     <row r="154" ht="15.75" customHeight="1">
       <c r="A154" s="4"/>
@@ -4364,6 +4524,7 @@
       <c r="U154" s="4"/>
       <c r="V154" s="4"/>
       <c r="W154" s="4"/>
+      <c r="X154" s="4"/>
     </row>
     <row r="155" ht="15.75" customHeight="1">
       <c r="A155" s="4"/>
@@ -4389,6 +4550,7 @@
       <c r="U155" s="4"/>
       <c r="V155" s="4"/>
       <c r="W155" s="4"/>
+      <c r="X155" s="4"/>
     </row>
     <row r="156" ht="15.75" customHeight="1">
       <c r="A156" s="4"/>
@@ -4414,6 +4576,7 @@
       <c r="U156" s="4"/>
       <c r="V156" s="4"/>
       <c r="W156" s="4"/>
+      <c r="X156" s="4"/>
     </row>
     <row r="157" ht="15.75" customHeight="1">
       <c r="A157" s="4"/>
@@ -4439,6 +4602,7 @@
       <c r="U157" s="4"/>
       <c r="V157" s="4"/>
       <c r="W157" s="4"/>
+      <c r="X157" s="4"/>
     </row>
     <row r="158" ht="15.75" customHeight="1">
       <c r="A158" s="4"/>
@@ -4464,6 +4628,7 @@
       <c r="U158" s="4"/>
       <c r="V158" s="4"/>
       <c r="W158" s="4"/>
+      <c r="X158" s="4"/>
     </row>
     <row r="159" ht="15.75" customHeight="1">
       <c r="A159" s="4"/>
@@ -4489,6 +4654,7 @@
       <c r="U159" s="4"/>
       <c r="V159" s="4"/>
       <c r="W159" s="4"/>
+      <c r="X159" s="4"/>
     </row>
     <row r="160" ht="15.75" customHeight="1">
       <c r="A160" s="4"/>
@@ -4514,6 +4680,7 @@
       <c r="U160" s="4"/>
       <c r="V160" s="4"/>
       <c r="W160" s="4"/>
+      <c r="X160" s="4"/>
     </row>
     <row r="161" ht="15.75" customHeight="1">
       <c r="A161" s="4"/>
@@ -4539,6 +4706,7 @@
       <c r="U161" s="4"/>
       <c r="V161" s="4"/>
       <c r="W161" s="4"/>
+      <c r="X161" s="4"/>
     </row>
     <row r="162" ht="15.75" customHeight="1">
       <c r="A162" s="4"/>
@@ -4564,6 +4732,7 @@
       <c r="U162" s="4"/>
       <c r="V162" s="4"/>
       <c r="W162" s="4"/>
+      <c r="X162" s="4"/>
     </row>
     <row r="163" ht="15.75" customHeight="1">
       <c r="A163" s="4"/>
@@ -4589,6 +4758,7 @@
       <c r="U163" s="4"/>
       <c r="V163" s="4"/>
       <c r="W163" s="4"/>
+      <c r="X163" s="4"/>
     </row>
     <row r="164" ht="15.75" customHeight="1">
       <c r="A164" s="4"/>
@@ -4614,6 +4784,7 @@
       <c r="U164" s="4"/>
       <c r="V164" s="4"/>
       <c r="W164" s="4"/>
+      <c r="X164" s="4"/>
     </row>
     <row r="165" ht="15.75" customHeight="1">
       <c r="A165" s="4"/>
@@ -4639,6 +4810,7 @@
       <c r="U165" s="4"/>
       <c r="V165" s="4"/>
       <c r="W165" s="4"/>
+      <c r="X165" s="4"/>
     </row>
     <row r="166" ht="15.75" customHeight="1">
       <c r="A166" s="4"/>
@@ -4664,6 +4836,7 @@
       <c r="U166" s="4"/>
       <c r="V166" s="4"/>
       <c r="W166" s="4"/>
+      <c r="X166" s="4"/>
     </row>
     <row r="167" ht="15.75" customHeight="1">
       <c r="A167" s="4"/>
@@ -4689,6 +4862,7 @@
       <c r="U167" s="4"/>
       <c r="V167" s="4"/>
       <c r="W167" s="4"/>
+      <c r="X167" s="4"/>
     </row>
     <row r="168" ht="15.75" customHeight="1">
       <c r="A168" s="4"/>
@@ -4714,6 +4888,7 @@
       <c r="U168" s="4"/>
       <c r="V168" s="4"/>
       <c r="W168" s="4"/>
+      <c r="X168" s="4"/>
     </row>
     <row r="169" ht="15.75" customHeight="1">
       <c r="A169" s="4"/>
@@ -4739,6 +4914,7 @@
       <c r="U169" s="4"/>
       <c r="V169" s="4"/>
       <c r="W169" s="4"/>
+      <c r="X169" s="4"/>
     </row>
     <row r="170" ht="15.75" customHeight="1">
       <c r="A170" s="4"/>
@@ -4764,6 +4940,7 @@
       <c r="U170" s="4"/>
       <c r="V170" s="4"/>
       <c r="W170" s="4"/>
+      <c r="X170" s="4"/>
     </row>
     <row r="171" ht="15.75" customHeight="1">
       <c r="A171" s="4"/>
@@ -4789,6 +4966,7 @@
       <c r="U171" s="4"/>
       <c r="V171" s="4"/>
       <c r="W171" s="4"/>
+      <c r="X171" s="4"/>
     </row>
     <row r="172" ht="15.75" customHeight="1">
       <c r="A172" s="4"/>
@@ -4814,6 +4992,7 @@
       <c r="U172" s="4"/>
       <c r="V172" s="4"/>
       <c r="W172" s="4"/>
+      <c r="X172" s="4"/>
     </row>
     <row r="173" ht="15.75" customHeight="1">
       <c r="A173" s="4"/>
@@ -4839,6 +5018,7 @@
       <c r="U173" s="4"/>
       <c r="V173" s="4"/>
       <c r="W173" s="4"/>
+      <c r="X173" s="4"/>
     </row>
     <row r="174" ht="15.75" customHeight="1">
       <c r="A174" s="4"/>
@@ -4864,6 +5044,7 @@
       <c r="U174" s="4"/>
       <c r="V174" s="4"/>
       <c r="W174" s="4"/>
+      <c r="X174" s="4"/>
     </row>
     <row r="175" ht="15.75" customHeight="1">
       <c r="A175" s="4"/>
@@ -4889,6 +5070,7 @@
       <c r="U175" s="4"/>
       <c r="V175" s="4"/>
       <c r="W175" s="4"/>
+      <c r="X175" s="4"/>
     </row>
     <row r="176" ht="15.75" customHeight="1">
       <c r="A176" s="4"/>
@@ -4914,6 +5096,7 @@
       <c r="U176" s="4"/>
       <c r="V176" s="4"/>
       <c r="W176" s="4"/>
+      <c r="X176" s="4"/>
     </row>
     <row r="177" ht="15.75" customHeight="1">
       <c r="A177" s="4"/>
@@ -4939,6 +5122,7 @@
       <c r="U177" s="4"/>
       <c r="V177" s="4"/>
       <c r="W177" s="4"/>
+      <c r="X177" s="4"/>
     </row>
     <row r="178" ht="15.75" customHeight="1">
       <c r="A178" s="4"/>
@@ -4964,6 +5148,7 @@
       <c r="U178" s="4"/>
       <c r="V178" s="4"/>
       <c r="W178" s="4"/>
+      <c r="X178" s="4"/>
     </row>
     <row r="179" ht="15.75" customHeight="1">
       <c r="A179" s="4"/>
@@ -4989,6 +5174,7 @@
       <c r="U179" s="4"/>
       <c r="V179" s="4"/>
       <c r="W179" s="4"/>
+      <c r="X179" s="4"/>
     </row>
     <row r="180" ht="15.75" customHeight="1">
       <c r="A180" s="4"/>
@@ -5014,6 +5200,7 @@
       <c r="U180" s="4"/>
       <c r="V180" s="4"/>
       <c r="W180" s="4"/>
+      <c r="X180" s="4"/>
     </row>
     <row r="181" ht="15.75" customHeight="1">
       <c r="A181" s="4"/>
@@ -5039,6 +5226,7 @@
       <c r="U181" s="4"/>
       <c r="V181" s="4"/>
       <c r="W181" s="4"/>
+      <c r="X181" s="4"/>
     </row>
     <row r="182" ht="15.75" customHeight="1">
       <c r="A182" s="4"/>
@@ -5064,6 +5252,7 @@
       <c r="U182" s="4"/>
       <c r="V182" s="4"/>
       <c r="W182" s="4"/>
+      <c r="X182" s="4"/>
     </row>
     <row r="183" ht="15.75" customHeight="1">
       <c r="A183" s="4"/>
@@ -5089,6 +5278,7 @@
       <c r="U183" s="4"/>
       <c r="V183" s="4"/>
       <c r="W183" s="4"/>
+      <c r="X183" s="4"/>
     </row>
     <row r="184" ht="15.75" customHeight="1">
       <c r="A184" s="4"/>
@@ -5114,6 +5304,7 @@
       <c r="U184" s="4"/>
       <c r="V184" s="4"/>
       <c r="W184" s="4"/>
+      <c r="X184" s="4"/>
     </row>
     <row r="185" ht="15.75" customHeight="1">
       <c r="A185" s="4"/>
@@ -5139,6 +5330,7 @@
       <c r="U185" s="4"/>
       <c r="V185" s="4"/>
       <c r="W185" s="4"/>
+      <c r="X185" s="4"/>
     </row>
     <row r="186" ht="15.75" customHeight="1">
       <c r="A186" s="4"/>
@@ -5164,6 +5356,7 @@
       <c r="U186" s="4"/>
       <c r="V186" s="4"/>
       <c r="W186" s="4"/>
+      <c r="X186" s="4"/>
     </row>
     <row r="187" ht="15.75" customHeight="1">
       <c r="A187" s="4"/>
@@ -5189,6 +5382,7 @@
       <c r="U187" s="4"/>
       <c r="V187" s="4"/>
       <c r="W187" s="4"/>
+      <c r="X187" s="4"/>
     </row>
     <row r="188" ht="15.75" customHeight="1">
       <c r="A188" s="4"/>
@@ -5214,6 +5408,7 @@
       <c r="U188" s="4"/>
       <c r="V188" s="4"/>
       <c r="W188" s="4"/>
+      <c r="X188" s="4"/>
     </row>
     <row r="189" ht="15.75" customHeight="1">
       <c r="A189" s="4"/>
@@ -5239,6 +5434,7 @@
       <c r="U189" s="4"/>
       <c r="V189" s="4"/>
       <c r="W189" s="4"/>
+      <c r="X189" s="4"/>
     </row>
     <row r="190" ht="15.75" customHeight="1">
       <c r="A190" s="4"/>
@@ -5264,6 +5460,7 @@
       <c r="U190" s="4"/>
       <c r="V190" s="4"/>
       <c r="W190" s="4"/>
+      <c r="X190" s="4"/>
     </row>
     <row r="191" ht="15.75" customHeight="1">
       <c r="A191" s="4"/>
@@ -5289,6 +5486,7 @@
       <c r="U191" s="4"/>
       <c r="V191" s="4"/>
       <c r="W191" s="4"/>
+      <c r="X191" s="4"/>
     </row>
     <row r="192" ht="15.75" customHeight="1">
       <c r="A192" s="4"/>
@@ -5314,6 +5512,7 @@
       <c r="U192" s="4"/>
       <c r="V192" s="4"/>
       <c r="W192" s="4"/>
+      <c r="X192" s="4"/>
     </row>
     <row r="193" ht="15.75" customHeight="1">
       <c r="A193" s="4"/>
@@ -5339,6 +5538,7 @@
       <c r="U193" s="4"/>
       <c r="V193" s="4"/>
       <c r="W193" s="4"/>
+      <c r="X193" s="4"/>
     </row>
     <row r="194" ht="15.75" customHeight="1">
       <c r="A194" s="4"/>
@@ -5364,6 +5564,7 @@
       <c r="U194" s="4"/>
       <c r="V194" s="4"/>
       <c r="W194" s="4"/>
+      <c r="X194" s="4"/>
     </row>
     <row r="195" ht="15.75" customHeight="1">
       <c r="A195" s="4"/>
@@ -5389,6 +5590,7 @@
       <c r="U195" s="4"/>
       <c r="V195" s="4"/>
       <c r="W195" s="4"/>
+      <c r="X195" s="4"/>
     </row>
     <row r="196" ht="15.75" customHeight="1">
       <c r="A196" s="4"/>
@@ -5414,6 +5616,7 @@
       <c r="U196" s="4"/>
       <c r="V196" s="4"/>
       <c r="W196" s="4"/>
+      <c r="X196" s="4"/>
     </row>
     <row r="197" ht="15.75" customHeight="1">
       <c r="A197" s="4"/>
@@ -5439,6 +5642,7 @@
       <c r="U197" s="4"/>
       <c r="V197" s="4"/>
       <c r="W197" s="4"/>
+      <c r="X197" s="4"/>
     </row>
     <row r="198" ht="15.75" customHeight="1">
       <c r="A198" s="4"/>
@@ -5464,6 +5668,7 @@
       <c r="U198" s="4"/>
       <c r="V198" s="4"/>
       <c r="W198" s="4"/>
+      <c r="X198" s="4"/>
     </row>
     <row r="199" ht="15.75" customHeight="1">
       <c r="A199" s="4"/>
@@ -5489,6 +5694,7 @@
       <c r="U199" s="4"/>
       <c r="V199" s="4"/>
       <c r="W199" s="4"/>
+      <c r="X199" s="4"/>
     </row>
     <row r="200" ht="15.75" customHeight="1">
       <c r="A200" s="4"/>
@@ -5514,6 +5720,7 @@
       <c r="U200" s="4"/>
       <c r="V200" s="4"/>
       <c r="W200" s="4"/>
+      <c r="X200" s="4"/>
     </row>
     <row r="201" ht="15.75" customHeight="1">
       <c r="A201" s="4"/>
@@ -5539,6 +5746,7 @@
       <c r="U201" s="4"/>
       <c r="V201" s="4"/>
       <c r="W201" s="4"/>
+      <c r="X201" s="4"/>
     </row>
     <row r="202" ht="15.75" customHeight="1">
       <c r="A202" s="4"/>
@@ -5564,6 +5772,7 @@
       <c r="U202" s="4"/>
       <c r="V202" s="4"/>
       <c r="W202" s="4"/>
+      <c r="X202" s="4"/>
     </row>
     <row r="203" ht="15.75" customHeight="1">
       <c r="A203" s="4"/>
@@ -5589,6 +5798,7 @@
       <c r="U203" s="4"/>
       <c r="V203" s="4"/>
       <c r="W203" s="4"/>
+      <c r="X203" s="4"/>
     </row>
     <row r="204" ht="15.75" customHeight="1">
       <c r="A204" s="4"/>
@@ -5614,6 +5824,7 @@
       <c r="U204" s="4"/>
       <c r="V204" s="4"/>
       <c r="W204" s="4"/>
+      <c r="X204" s="4"/>
     </row>
     <row r="205" ht="15.75" customHeight="1">
       <c r="A205" s="4"/>
@@ -5639,6 +5850,7 @@
       <c r="U205" s="4"/>
       <c r="V205" s="4"/>
       <c r="W205" s="4"/>
+      <c r="X205" s="4"/>
     </row>
     <row r="206" ht="15.75" customHeight="1">
       <c r="A206" s="4"/>
@@ -5664,6 +5876,7 @@
       <c r="U206" s="4"/>
       <c r="V206" s="4"/>
       <c r="W206" s="4"/>
+      <c r="X206" s="4"/>
     </row>
     <row r="207" ht="15.75" customHeight="1">
       <c r="A207" s="4"/>
@@ -5689,6 +5902,7 @@
       <c r="U207" s="4"/>
       <c r="V207" s="4"/>
       <c r="W207" s="4"/>
+      <c r="X207" s="4"/>
     </row>
     <row r="208" ht="15.75" customHeight="1">
       <c r="A208" s="4"/>
@@ -5714,6 +5928,7 @@
       <c r="U208" s="4"/>
       <c r="V208" s="4"/>
       <c r="W208" s="4"/>
+      <c r="X208" s="4"/>
     </row>
     <row r="209" ht="15.75" customHeight="1">
       <c r="A209" s="4"/>
@@ -5739,6 +5954,7 @@
       <c r="U209" s="4"/>
       <c r="V209" s="4"/>
       <c r="W209" s="4"/>
+      <c r="X209" s="4"/>
     </row>
     <row r="210" ht="15.75" customHeight="1">
       <c r="A210" s="4"/>
@@ -5764,6 +5980,7 @@
       <c r="U210" s="4"/>
       <c r="V210" s="4"/>
       <c r="W210" s="4"/>
+      <c r="X210" s="4"/>
     </row>
     <row r="211" ht="15.75" customHeight="1">
       <c r="A211" s="4"/>
@@ -5789,6 +6006,7 @@
       <c r="U211" s="4"/>
       <c r="V211" s="4"/>
       <c r="W211" s="4"/>
+      <c r="X211" s="4"/>
     </row>
     <row r="212" ht="15.75" customHeight="1">
       <c r="A212" s="4"/>
@@ -5814,6 +6032,7 @@
       <c r="U212" s="4"/>
       <c r="V212" s="4"/>
       <c r="W212" s="4"/>
+      <c r="X212" s="4"/>
     </row>
     <row r="213" ht="15.75" customHeight="1">
       <c r="A213" s="4"/>
@@ -5839,6 +6058,7 @@
       <c r="U213" s="4"/>
       <c r="V213" s="4"/>
       <c r="W213" s="4"/>
+      <c r="X213" s="4"/>
     </row>
     <row r="214" ht="15.75" customHeight="1">
       <c r="A214" s="4"/>
@@ -5864,6 +6084,7 @@
       <c r="U214" s="4"/>
       <c r="V214" s="4"/>
       <c r="W214" s="4"/>
+      <c r="X214" s="4"/>
     </row>
     <row r="215" ht="15.75" customHeight="1">
       <c r="A215" s="4"/>
@@ -5889,6 +6110,7 @@
       <c r="U215" s="4"/>
       <c r="V215" s="4"/>
       <c r="W215" s="4"/>
+      <c r="X215" s="4"/>
     </row>
     <row r="216" ht="15.75" customHeight="1">
       <c r="A216" s="4"/>
@@ -5914,6 +6136,7 @@
       <c r="U216" s="4"/>
       <c r="V216" s="4"/>
       <c r="W216" s="4"/>
+      <c r="X216" s="4"/>
     </row>
     <row r="217" ht="15.75" customHeight="1">
       <c r="A217" s="4"/>
@@ -5939,6 +6162,7 @@
       <c r="U217" s="4"/>
       <c r="V217" s="4"/>
       <c r="W217" s="4"/>
+      <c r="X217" s="4"/>
     </row>
     <row r="218" ht="15.75" customHeight="1">
       <c r="A218" s="4"/>
@@ -5964,6 +6188,7 @@
       <c r="U218" s="4"/>
       <c r="V218" s="4"/>
       <c r="W218" s="4"/>
+      <c r="X218" s="4"/>
     </row>
     <row r="219" ht="15.75" customHeight="1">
       <c r="A219" s="4"/>
@@ -5989,6 +6214,7 @@
       <c r="U219" s="4"/>
       <c r="V219" s="4"/>
       <c r="W219" s="4"/>
+      <c r="X219" s="4"/>
     </row>
     <row r="220" ht="15.75" customHeight="1">
       <c r="A220" s="4"/>
@@ -6014,6 +6240,7 @@
       <c r="U220" s="4"/>
       <c r="V220" s="4"/>
       <c r="W220" s="4"/>
+      <c r="X220" s="4"/>
     </row>
     <row r="221" ht="15.75" customHeight="1"/>
     <row r="222" ht="15.75" customHeight="1"/>

</xml_diff>

<commit_message>
test: add product to cart validation
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/testData_Appium_myDemoApp.xlsx
+++ b/src/test/resources/testData/testData_Appium_myDemoApp.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="42">
   <si>
     <t>CT</t>
   </si>
@@ -769,8 +769,10 @@
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
       <c r="D11" s="1"/>
-      <c r="E11" s="1"/>
-      <c r="F11" s="1"/>
+      <c r="E11" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="F11" s="3"/>
       <c r="G11" s="1"/>
       <c r="H11" s="1"/>
       <c r="I11" s="1"/>

</xml_diff>

<commit_message>
test: validate product color display in cart
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/testData_Appium_myDemoApp.xlsx
+++ b/src/test/resources/testData/testData_Appium_myDemoApp.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="44">
   <si>
     <t>CT</t>
   </si>
@@ -26,6 +26,9 @@
   </si>
   <si>
     <t>PRODUCT_NAME</t>
+  </si>
+  <si>
+    <t>PRODUCT_NAME_2</t>
   </si>
   <si>
     <t>PRODUCT_COLOR</t>
@@ -113,6 +116,9 @@
   </si>
   <si>
     <t>011</t>
+  </si>
+  <si>
+    <t>Sauce Labs Backpack (orange)</t>
   </si>
   <si>
     <t>012</t>
@@ -420,14 +426,17 @@
     <col customWidth="1" min="1" max="1" width="12.63"/>
     <col customWidth="1" min="2" max="2" width="19.63"/>
     <col customWidth="1" min="3" max="3" width="21.63"/>
-    <col customWidth="1" min="4" max="6" width="31.38"/>
-    <col customWidth="1" min="7" max="7" width="18.38"/>
-    <col customWidth="1" min="8" max="8" width="17.13"/>
-    <col customWidth="1" min="9" max="9" width="16.0"/>
-    <col customWidth="1" min="10" max="11" width="17.13"/>
-    <col customWidth="1" min="12" max="12" width="15.75"/>
-    <col customWidth="1" min="13" max="13" width="14.38"/>
-    <col customWidth="1" min="16" max="16" width="27.0"/>
+    <col customWidth="1" min="4" max="4" width="31.38"/>
+    <col customWidth="1" min="5" max="5" width="33.25"/>
+    <col customWidth="1" min="6" max="6" width="42.88"/>
+    <col customWidth="1" min="7" max="7" width="31.38"/>
+    <col customWidth="1" min="8" max="8" width="18.38"/>
+    <col customWidth="1" min="9" max="9" width="17.13"/>
+    <col customWidth="1" min="10" max="10" width="16.0"/>
+    <col customWidth="1" min="11" max="12" width="17.13"/>
+    <col customWidth="1" min="13" max="13" width="15.75"/>
+    <col customWidth="1" min="14" max="14" width="14.38"/>
+    <col customWidth="1" min="17" max="17" width="27.0"/>
   </cols>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
@@ -449,7 +458,7 @@
       <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="3" t="s">
         <v>6</v>
       </c>
       <c r="H1" s="1" t="s">
@@ -479,7 +488,9 @@
       <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="4"/>
+      <c r="Q1" s="1" t="s">
+        <v>16</v>
+      </c>
       <c r="R1" s="4"/>
       <c r="S1" s="4"/>
       <c r="T1" s="4"/>
@@ -487,16 +498,17 @@
       <c r="V1" s="4"/>
       <c r="W1" s="4"/>
       <c r="X1" s="4"/>
+      <c r="Y1" s="4"/>
     </row>
     <row r="2" ht="15.75" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
@@ -511,7 +523,7 @@
       <c r="N2" s="1"/>
       <c r="O2" s="1"/>
       <c r="P2" s="1"/>
-      <c r="Q2" s="4"/>
+      <c r="Q2" s="1"/>
       <c r="R2" s="4"/>
       <c r="S2" s="4"/>
       <c r="T2" s="4"/>
@@ -519,10 +531,11 @@
       <c r="V2" s="4"/>
       <c r="W2" s="4"/>
       <c r="X2" s="4"/>
+      <c r="Y2" s="4"/>
     </row>
     <row r="3" ht="15.75" customHeight="1">
       <c r="A3" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
@@ -539,7 +552,7 @@
       <c r="N3" s="1"/>
       <c r="O3" s="1"/>
       <c r="P3" s="1"/>
-      <c r="Q3" s="4"/>
+      <c r="Q3" s="1"/>
       <c r="R3" s="4"/>
       <c r="S3" s="4"/>
       <c r="T3" s="4"/>
@@ -547,16 +560,17 @@
       <c r="V3" s="4"/>
       <c r="W3" s="4"/>
       <c r="X3" s="4"/>
+      <c r="Y3" s="4"/>
     </row>
     <row r="4" ht="15.75" customHeight="1">
       <c r="A4" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
@@ -571,7 +585,7 @@
       <c r="N4" s="1"/>
       <c r="O4" s="1"/>
       <c r="P4" s="1"/>
-      <c r="Q4" s="4"/>
+      <c r="Q4" s="1"/>
       <c r="R4" s="4"/>
       <c r="S4" s="4"/>
       <c r="T4" s="4"/>
@@ -579,15 +593,16 @@
       <c r="V4" s="4"/>
       <c r="W4" s="4"/>
       <c r="X4" s="4"/>
+      <c r="Y4" s="4"/>
     </row>
     <row r="5" ht="15.75" customHeight="1">
       <c r="A5" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
       <c r="D5" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E5" s="1"/>
       <c r="F5" s="1"/>
@@ -601,7 +616,7 @@
       <c r="N5" s="1"/>
       <c r="O5" s="1"/>
       <c r="P5" s="1"/>
-      <c r="Q5" s="4"/>
+      <c r="Q5" s="1"/>
       <c r="R5" s="4"/>
       <c r="S5" s="4"/>
       <c r="T5" s="4"/>
@@ -609,15 +624,16 @@
       <c r="V5" s="4"/>
       <c r="W5" s="4"/>
       <c r="X5" s="4"/>
+      <c r="Y5" s="4"/>
     </row>
     <row r="6" ht="15.75" customHeight="1">
       <c r="A6" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
       <c r="D6" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E6" s="1"/>
       <c r="F6" s="1"/>
@@ -631,7 +647,7 @@
       <c r="N6" s="1"/>
       <c r="O6" s="1"/>
       <c r="P6" s="1"/>
-      <c r="Q6" s="4"/>
+      <c r="Q6" s="1"/>
       <c r="R6" s="4"/>
       <c r="S6" s="4"/>
       <c r="T6" s="4"/>
@@ -639,15 +655,16 @@
       <c r="V6" s="4"/>
       <c r="W6" s="4"/>
       <c r="X6" s="4"/>
+      <c r="Y6" s="4"/>
     </row>
     <row r="7" ht="15.75" customHeight="1">
       <c r="A7" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
       <c r="D7" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E7" s="1"/>
       <c r="F7" s="1"/>
@@ -661,7 +678,7 @@
       <c r="N7" s="1"/>
       <c r="O7" s="1"/>
       <c r="P7" s="1"/>
-      <c r="Q7" s="4"/>
+      <c r="Q7" s="1"/>
       <c r="R7" s="4"/>
       <c r="S7" s="4"/>
       <c r="T7" s="4"/>
@@ -669,15 +686,16 @@
       <c r="V7" s="4"/>
       <c r="W7" s="4"/>
       <c r="X7" s="4"/>
+      <c r="Y7" s="4"/>
     </row>
     <row r="8" ht="15.75" customHeight="1">
       <c r="A8" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
       <c r="D8" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E8" s="1"/>
       <c r="F8" s="1"/>
@@ -691,7 +709,7 @@
       <c r="N8" s="1"/>
       <c r="O8" s="1"/>
       <c r="P8" s="1"/>
-      <c r="Q8" s="4"/>
+      <c r="Q8" s="1"/>
       <c r="R8" s="4"/>
       <c r="S8" s="4"/>
       <c r="T8" s="4"/>
@@ -699,19 +717,20 @@
       <c r="V8" s="4"/>
       <c r="W8" s="4"/>
       <c r="X8" s="4"/>
+      <c r="Y8" s="4"/>
     </row>
     <row r="9" ht="15.75" customHeight="1">
       <c r="A9" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
       <c r="D9" s="1"/>
       <c r="E9" s="3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F9" s="3"/>
-      <c r="G9" s="1"/>
+      <c r="G9" s="3"/>
       <c r="H9" s="1"/>
       <c r="I9" s="1"/>
       <c r="J9" s="1"/>
@@ -721,7 +740,7 @@
       <c r="N9" s="1"/>
       <c r="O9" s="1"/>
       <c r="P9" s="1"/>
-      <c r="Q9" s="4"/>
+      <c r="Q9" s="1"/>
       <c r="R9" s="4"/>
       <c r="S9" s="4"/>
       <c r="T9" s="4"/>
@@ -729,21 +748,22 @@
       <c r="V9" s="4"/>
       <c r="W9" s="4"/>
       <c r="X9" s="4"/>
+      <c r="Y9" s="4"/>
     </row>
     <row r="10" ht="15.75" customHeight="1">
       <c r="A10" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
       <c r="D10" s="1"/>
       <c r="E10" s="3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
-      <c r="F10" s="3" t="s">
-        <v>31</v>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3" t="s">
+        <v>32</v>
       </c>
-      <c r="G10" s="1"/>
       <c r="H10" s="1"/>
       <c r="I10" s="1"/>
       <c r="J10" s="1"/>
@@ -753,7 +773,7 @@
       <c r="N10" s="1"/>
       <c r="O10" s="1"/>
       <c r="P10" s="1"/>
-      <c r="Q10" s="4"/>
+      <c r="Q10" s="1"/>
       <c r="R10" s="4"/>
       <c r="S10" s="4"/>
       <c r="T10" s="4"/>
@@ -761,19 +781,20 @@
       <c r="V10" s="4"/>
       <c r="W10" s="4"/>
       <c r="X10" s="4"/>
+      <c r="Y10" s="4"/>
     </row>
     <row r="11" ht="15.75" customHeight="1">
       <c r="A11" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
       <c r="D11" s="1"/>
       <c r="E11" s="3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F11" s="3"/>
-      <c r="G11" s="1"/>
+      <c r="G11" s="3"/>
       <c r="H11" s="1"/>
       <c r="I11" s="1"/>
       <c r="J11" s="1"/>
@@ -783,7 +804,7 @@
       <c r="N11" s="1"/>
       <c r="O11" s="1"/>
       <c r="P11" s="1"/>
-      <c r="Q11" s="4"/>
+      <c r="Q11" s="1"/>
       <c r="R11" s="4"/>
       <c r="S11" s="4"/>
       <c r="T11" s="4"/>
@@ -791,17 +812,26 @@
       <c r="V11" s="4"/>
       <c r="W11" s="4"/>
       <c r="X11" s="4"/>
+      <c r="Y11" s="4"/>
     </row>
     <row r="12" ht="15.75" customHeight="1">
       <c r="A12" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
-      <c r="B12" s="1"/>
-      <c r="C12" s="1"/>
+      <c r="B12" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>18</v>
+      </c>
       <c r="D12" s="1"/>
-      <c r="E12" s="3"/>
-      <c r="F12" s="3"/>
-      <c r="G12" s="1"/>
+      <c r="E12" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="G12" s="3"/>
       <c r="H12" s="1"/>
       <c r="I12" s="1"/>
       <c r="J12" s="1"/>
@@ -811,7 +841,7 @@
       <c r="N12" s="1"/>
       <c r="O12" s="1"/>
       <c r="P12" s="1"/>
-      <c r="Q12" s="4"/>
+      <c r="Q12" s="1"/>
       <c r="R12" s="4"/>
       <c r="S12" s="4"/>
       <c r="T12" s="4"/>
@@ -819,17 +849,26 @@
       <c r="V12" s="4"/>
       <c r="W12" s="4"/>
       <c r="X12" s="4"/>
+      <c r="Y12" s="4"/>
     </row>
     <row r="13" ht="15.75" customHeight="1">
       <c r="A13" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
-      <c r="B13" s="1"/>
-      <c r="C13" s="1"/>
+      <c r="B13" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>18</v>
+      </c>
       <c r="D13" s="1"/>
-      <c r="E13" s="1"/>
+      <c r="E13" s="3" t="s">
+        <v>30</v>
+      </c>
       <c r="F13" s="1"/>
-      <c r="G13" s="1"/>
+      <c r="G13" s="3" t="s">
+        <v>32</v>
+      </c>
       <c r="H13" s="1"/>
       <c r="I13" s="1"/>
       <c r="J13" s="1"/>
@@ -839,7 +878,7 @@
       <c r="N13" s="1"/>
       <c r="O13" s="1"/>
       <c r="P13" s="1"/>
-      <c r="Q13" s="4"/>
+      <c r="Q13" s="1"/>
       <c r="R13" s="4"/>
       <c r="S13" s="4"/>
       <c r="T13" s="4"/>
@@ -847,10 +886,11 @@
       <c r="V13" s="4"/>
       <c r="W13" s="4"/>
       <c r="X13" s="4"/>
+      <c r="Y13" s="4"/>
     </row>
     <row r="14" ht="15.75" customHeight="1">
       <c r="A14" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
@@ -867,7 +907,7 @@
       <c r="N14" s="1"/>
       <c r="O14" s="1"/>
       <c r="P14" s="1"/>
-      <c r="Q14" s="4"/>
+      <c r="Q14" s="1"/>
       <c r="R14" s="4"/>
       <c r="S14" s="4"/>
       <c r="T14" s="4"/>
@@ -875,10 +915,11 @@
       <c r="V14" s="4"/>
       <c r="W14" s="4"/>
       <c r="X14" s="4"/>
+      <c r="Y14" s="4"/>
     </row>
     <row r="15" ht="15.75" customHeight="1">
       <c r="A15" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
@@ -895,7 +936,7 @@
       <c r="N15" s="1"/>
       <c r="O15" s="1"/>
       <c r="P15" s="1"/>
-      <c r="Q15" s="4"/>
+      <c r="Q15" s="1"/>
       <c r="R15" s="4"/>
       <c r="S15" s="4"/>
       <c r="T15" s="4"/>
@@ -903,10 +944,11 @@
       <c r="V15" s="4"/>
       <c r="W15" s="4"/>
       <c r="X15" s="4"/>
+      <c r="Y15" s="4"/>
     </row>
     <row r="16" ht="15.75" customHeight="1">
       <c r="A16" s="1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B16" s="1"/>
       <c r="C16" s="1"/>
@@ -923,7 +965,7 @@
       <c r="N16" s="1"/>
       <c r="O16" s="1"/>
       <c r="P16" s="1"/>
-      <c r="Q16" s="4"/>
+      <c r="Q16" s="1"/>
       <c r="R16" s="4"/>
       <c r="S16" s="4"/>
       <c r="T16" s="4"/>
@@ -931,10 +973,11 @@
       <c r="V16" s="4"/>
       <c r="W16" s="4"/>
       <c r="X16" s="4"/>
+      <c r="Y16" s="4"/>
     </row>
     <row r="17" ht="15.75" customHeight="1">
       <c r="A17" s="1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B17" s="1"/>
       <c r="C17" s="1"/>
@@ -951,7 +994,7 @@
       <c r="N17" s="1"/>
       <c r="O17" s="1"/>
       <c r="P17" s="1"/>
-      <c r="Q17" s="4"/>
+      <c r="Q17" s="1"/>
       <c r="R17" s="4"/>
       <c r="S17" s="4"/>
       <c r="T17" s="4"/>
@@ -959,10 +1002,11 @@
       <c r="V17" s="4"/>
       <c r="W17" s="4"/>
       <c r="X17" s="4"/>
+      <c r="Y17" s="4"/>
     </row>
     <row r="18" ht="15.75" customHeight="1">
       <c r="A18" s="1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B18" s="1"/>
       <c r="C18" s="1"/>
@@ -979,7 +1023,7 @@
       <c r="N18" s="1"/>
       <c r="O18" s="1"/>
       <c r="P18" s="1"/>
-      <c r="Q18" s="4"/>
+      <c r="Q18" s="1"/>
       <c r="R18" s="4"/>
       <c r="S18" s="4"/>
       <c r="T18" s="4"/>
@@ -987,10 +1031,11 @@
       <c r="V18" s="4"/>
       <c r="W18" s="4"/>
       <c r="X18" s="4"/>
+      <c r="Y18" s="4"/>
     </row>
     <row r="19" ht="15.75" customHeight="1">
       <c r="A19" s="1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B19" s="1"/>
       <c r="C19" s="1"/>
@@ -1007,7 +1052,7 @@
       <c r="N19" s="1"/>
       <c r="O19" s="1"/>
       <c r="P19" s="1"/>
-      <c r="Q19" s="4"/>
+      <c r="Q19" s="1"/>
       <c r="R19" s="4"/>
       <c r="S19" s="4"/>
       <c r="T19" s="4"/>
@@ -1015,10 +1060,11 @@
       <c r="V19" s="4"/>
       <c r="W19" s="4"/>
       <c r="X19" s="4"/>
+      <c r="Y19" s="4"/>
     </row>
     <row r="20" ht="15.75" customHeight="1">
       <c r="A20" s="1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B20" s="1"/>
       <c r="C20" s="1"/>
@@ -1035,7 +1081,7 @@
       <c r="N20" s="1"/>
       <c r="O20" s="1"/>
       <c r="P20" s="1"/>
-      <c r="Q20" s="4"/>
+      <c r="Q20" s="1"/>
       <c r="R20" s="4"/>
       <c r="S20" s="4"/>
       <c r="T20" s="4"/>
@@ -1043,6 +1089,7 @@
       <c r="V20" s="4"/>
       <c r="W20" s="4"/>
       <c r="X20" s="4"/>
+      <c r="Y20" s="4"/>
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="4"/>
@@ -1069,6 +1116,7 @@
       <c r="V21" s="4"/>
       <c r="W21" s="4"/>
       <c r="X21" s="4"/>
+      <c r="Y21" s="4"/>
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="4"/>
@@ -1095,6 +1143,7 @@
       <c r="V22" s="4"/>
       <c r="W22" s="4"/>
       <c r="X22" s="4"/>
+      <c r="Y22" s="4"/>
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="4"/>
@@ -1121,6 +1170,7 @@
       <c r="V23" s="4"/>
       <c r="W23" s="4"/>
       <c r="X23" s="4"/>
+      <c r="Y23" s="4"/>
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="4"/>
@@ -1147,6 +1197,7 @@
       <c r="V24" s="4"/>
       <c r="W24" s="4"/>
       <c r="X24" s="4"/>
+      <c r="Y24" s="4"/>
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="4"/>
@@ -1173,6 +1224,7 @@
       <c r="V25" s="4"/>
       <c r="W25" s="4"/>
       <c r="X25" s="4"/>
+      <c r="Y25" s="4"/>
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="4"/>
@@ -1199,6 +1251,7 @@
       <c r="V26" s="4"/>
       <c r="W26" s="4"/>
       <c r="X26" s="4"/>
+      <c r="Y26" s="4"/>
     </row>
     <row r="27" ht="15.75" customHeight="1">
       <c r="A27" s="4"/>
@@ -1225,6 +1278,7 @@
       <c r="V27" s="4"/>
       <c r="W27" s="4"/>
       <c r="X27" s="4"/>
+      <c r="Y27" s="4"/>
     </row>
     <row r="28" ht="15.75" customHeight="1">
       <c r="A28" s="4"/>
@@ -1251,6 +1305,7 @@
       <c r="V28" s="4"/>
       <c r="W28" s="4"/>
       <c r="X28" s="4"/>
+      <c r="Y28" s="4"/>
     </row>
     <row r="29" ht="15.75" customHeight="1">
       <c r="A29" s="4"/>
@@ -1277,6 +1332,7 @@
       <c r="V29" s="4"/>
       <c r="W29" s="4"/>
       <c r="X29" s="4"/>
+      <c r="Y29" s="4"/>
     </row>
     <row r="30" ht="15.75" customHeight="1">
       <c r="A30" s="4"/>
@@ -1303,6 +1359,7 @@
       <c r="V30" s="4"/>
       <c r="W30" s="4"/>
       <c r="X30" s="4"/>
+      <c r="Y30" s="4"/>
     </row>
     <row r="31" ht="15.75" customHeight="1">
       <c r="A31" s="4"/>
@@ -1329,6 +1386,7 @@
       <c r="V31" s="4"/>
       <c r="W31" s="4"/>
       <c r="X31" s="4"/>
+      <c r="Y31" s="4"/>
     </row>
     <row r="32" ht="15.75" customHeight="1">
       <c r="A32" s="4"/>
@@ -1355,6 +1413,7 @@
       <c r="V32" s="4"/>
       <c r="W32" s="4"/>
       <c r="X32" s="4"/>
+      <c r="Y32" s="4"/>
     </row>
     <row r="33" ht="15.75" customHeight="1">
       <c r="A33" s="4"/>
@@ -1381,6 +1440,7 @@
       <c r="V33" s="4"/>
       <c r="W33" s="4"/>
       <c r="X33" s="4"/>
+      <c r="Y33" s="4"/>
     </row>
     <row r="34" ht="15.75" customHeight="1">
       <c r="A34" s="4"/>
@@ -1407,6 +1467,7 @@
       <c r="V34" s="4"/>
       <c r="W34" s="4"/>
       <c r="X34" s="4"/>
+      <c r="Y34" s="4"/>
     </row>
     <row r="35" ht="15.75" customHeight="1">
       <c r="A35" s="4"/>
@@ -1433,6 +1494,7 @@
       <c r="V35" s="4"/>
       <c r="W35" s="4"/>
       <c r="X35" s="4"/>
+      <c r="Y35" s="4"/>
     </row>
     <row r="36" ht="15.75" customHeight="1">
       <c r="A36" s="4"/>
@@ -1459,6 +1521,7 @@
       <c r="V36" s="4"/>
       <c r="W36" s="4"/>
       <c r="X36" s="4"/>
+      <c r="Y36" s="4"/>
     </row>
     <row r="37" ht="15.75" customHeight="1">
       <c r="A37" s="4"/>
@@ -1485,6 +1548,7 @@
       <c r="V37" s="4"/>
       <c r="W37" s="4"/>
       <c r="X37" s="4"/>
+      <c r="Y37" s="4"/>
     </row>
     <row r="38" ht="15.75" customHeight="1">
       <c r="A38" s="4"/>
@@ -1511,6 +1575,7 @@
       <c r="V38" s="4"/>
       <c r="W38" s="4"/>
       <c r="X38" s="4"/>
+      <c r="Y38" s="4"/>
     </row>
     <row r="39" ht="15.75" customHeight="1">
       <c r="A39" s="4"/>
@@ -1537,6 +1602,7 @@
       <c r="V39" s="4"/>
       <c r="W39" s="4"/>
       <c r="X39" s="4"/>
+      <c r="Y39" s="4"/>
     </row>
     <row r="40" ht="15.75" customHeight="1">
       <c r="A40" s="4"/>
@@ -1563,6 +1629,7 @@
       <c r="V40" s="4"/>
       <c r="W40" s="4"/>
       <c r="X40" s="4"/>
+      <c r="Y40" s="4"/>
     </row>
     <row r="41" ht="15.75" customHeight="1">
       <c r="A41" s="4"/>
@@ -1589,6 +1656,7 @@
       <c r="V41" s="4"/>
       <c r="W41" s="4"/>
       <c r="X41" s="4"/>
+      <c r="Y41" s="4"/>
     </row>
     <row r="42" ht="15.75" customHeight="1">
       <c r="A42" s="4"/>
@@ -1615,6 +1683,7 @@
       <c r="V42" s="4"/>
       <c r="W42" s="4"/>
       <c r="X42" s="4"/>
+      <c r="Y42" s="4"/>
     </row>
     <row r="43" ht="15.75" customHeight="1">
       <c r="A43" s="4"/>
@@ -1641,6 +1710,7 @@
       <c r="V43" s="4"/>
       <c r="W43" s="4"/>
       <c r="X43" s="4"/>
+      <c r="Y43" s="4"/>
     </row>
     <row r="44" ht="15.75" customHeight="1">
       <c r="A44" s="4"/>
@@ -1667,6 +1737,7 @@
       <c r="V44" s="4"/>
       <c r="W44" s="4"/>
       <c r="X44" s="4"/>
+      <c r="Y44" s="4"/>
     </row>
     <row r="45" ht="15.75" customHeight="1">
       <c r="A45" s="4"/>
@@ -1693,6 +1764,7 @@
       <c r="V45" s="4"/>
       <c r="W45" s="4"/>
       <c r="X45" s="4"/>
+      <c r="Y45" s="4"/>
     </row>
     <row r="46" ht="15.75" customHeight="1">
       <c r="A46" s="4"/>
@@ -1719,6 +1791,7 @@
       <c r="V46" s="4"/>
       <c r="W46" s="4"/>
       <c r="X46" s="4"/>
+      <c r="Y46" s="4"/>
     </row>
     <row r="47" ht="15.75" customHeight="1">
       <c r="A47" s="4"/>
@@ -1745,6 +1818,7 @@
       <c r="V47" s="4"/>
       <c r="W47" s="4"/>
       <c r="X47" s="4"/>
+      <c r="Y47" s="4"/>
     </row>
     <row r="48" ht="15.75" customHeight="1">
       <c r="A48" s="4"/>
@@ -1771,6 +1845,7 @@
       <c r="V48" s="4"/>
       <c r="W48" s="4"/>
       <c r="X48" s="4"/>
+      <c r="Y48" s="4"/>
     </row>
     <row r="49" ht="15.75" customHeight="1">
       <c r="A49" s="4"/>
@@ -1797,6 +1872,7 @@
       <c r="V49" s="4"/>
       <c r="W49" s="4"/>
       <c r="X49" s="4"/>
+      <c r="Y49" s="4"/>
     </row>
     <row r="50" ht="15.75" customHeight="1">
       <c r="A50" s="4"/>
@@ -1823,6 +1899,7 @@
       <c r="V50" s="4"/>
       <c r="W50" s="4"/>
       <c r="X50" s="4"/>
+      <c r="Y50" s="4"/>
     </row>
     <row r="51" ht="15.75" customHeight="1">
       <c r="A51" s="4"/>
@@ -1849,6 +1926,7 @@
       <c r="V51" s="4"/>
       <c r="W51" s="4"/>
       <c r="X51" s="4"/>
+      <c r="Y51" s="4"/>
     </row>
     <row r="52" ht="15.75" customHeight="1">
       <c r="A52" s="4"/>
@@ -1875,6 +1953,7 @@
       <c r="V52" s="4"/>
       <c r="W52" s="4"/>
       <c r="X52" s="4"/>
+      <c r="Y52" s="4"/>
     </row>
     <row r="53" ht="15.75" customHeight="1">
       <c r="A53" s="4"/>
@@ -1901,6 +1980,7 @@
       <c r="V53" s="4"/>
       <c r="W53" s="4"/>
       <c r="X53" s="4"/>
+      <c r="Y53" s="4"/>
     </row>
     <row r="54" ht="15.75" customHeight="1">
       <c r="A54" s="4"/>
@@ -1927,6 +2007,7 @@
       <c r="V54" s="4"/>
       <c r="W54" s="4"/>
       <c r="X54" s="4"/>
+      <c r="Y54" s="4"/>
     </row>
     <row r="55" ht="15.75" customHeight="1">
       <c r="A55" s="4"/>
@@ -1953,6 +2034,7 @@
       <c r="V55" s="4"/>
       <c r="W55" s="4"/>
       <c r="X55" s="4"/>
+      <c r="Y55" s="4"/>
     </row>
     <row r="56" ht="15.75" customHeight="1">
       <c r="A56" s="4"/>
@@ -1979,6 +2061,7 @@
       <c r="V56" s="4"/>
       <c r="W56" s="4"/>
       <c r="X56" s="4"/>
+      <c r="Y56" s="4"/>
     </row>
     <row r="57" ht="15.75" customHeight="1">
       <c r="A57" s="4"/>
@@ -2005,6 +2088,7 @@
       <c r="V57" s="4"/>
       <c r="W57" s="4"/>
       <c r="X57" s="4"/>
+      <c r="Y57" s="4"/>
     </row>
     <row r="58" ht="15.75" customHeight="1">
       <c r="A58" s="4"/>
@@ -2031,6 +2115,7 @@
       <c r="V58" s="4"/>
       <c r="W58" s="4"/>
       <c r="X58" s="4"/>
+      <c r="Y58" s="4"/>
     </row>
     <row r="59" ht="15.75" customHeight="1">
       <c r="A59" s="4"/>
@@ -2057,6 +2142,7 @@
       <c r="V59" s="4"/>
       <c r="W59" s="4"/>
       <c r="X59" s="4"/>
+      <c r="Y59" s="4"/>
     </row>
     <row r="60" ht="15.75" customHeight="1">
       <c r="A60" s="4"/>
@@ -2083,6 +2169,7 @@
       <c r="V60" s="4"/>
       <c r="W60" s="4"/>
       <c r="X60" s="4"/>
+      <c r="Y60" s="4"/>
     </row>
     <row r="61" ht="15.75" customHeight="1">
       <c r="A61" s="4"/>
@@ -2109,6 +2196,7 @@
       <c r="V61" s="4"/>
       <c r="W61" s="4"/>
       <c r="X61" s="4"/>
+      <c r="Y61" s="4"/>
     </row>
     <row r="62" ht="15.75" customHeight="1">
       <c r="A62" s="4"/>
@@ -2135,6 +2223,7 @@
       <c r="V62" s="4"/>
       <c r="W62" s="4"/>
       <c r="X62" s="4"/>
+      <c r="Y62" s="4"/>
     </row>
     <row r="63" ht="15.75" customHeight="1">
       <c r="A63" s="4"/>
@@ -2161,6 +2250,7 @@
       <c r="V63" s="4"/>
       <c r="W63" s="4"/>
       <c r="X63" s="4"/>
+      <c r="Y63" s="4"/>
     </row>
     <row r="64" ht="15.75" customHeight="1">
       <c r="A64" s="4"/>
@@ -2187,6 +2277,7 @@
       <c r="V64" s="4"/>
       <c r="W64" s="4"/>
       <c r="X64" s="4"/>
+      <c r="Y64" s="4"/>
     </row>
     <row r="65" ht="15.75" customHeight="1">
       <c r="A65" s="4"/>
@@ -2213,6 +2304,7 @@
       <c r="V65" s="4"/>
       <c r="W65" s="4"/>
       <c r="X65" s="4"/>
+      <c r="Y65" s="4"/>
     </row>
     <row r="66" ht="15.75" customHeight="1">
       <c r="A66" s="4"/>
@@ -2239,6 +2331,7 @@
       <c r="V66" s="4"/>
       <c r="W66" s="4"/>
       <c r="X66" s="4"/>
+      <c r="Y66" s="4"/>
     </row>
     <row r="67" ht="15.75" customHeight="1">
       <c r="A67" s="4"/>
@@ -2265,6 +2358,7 @@
       <c r="V67" s="4"/>
       <c r="W67" s="4"/>
       <c r="X67" s="4"/>
+      <c r="Y67" s="4"/>
     </row>
     <row r="68" ht="15.75" customHeight="1">
       <c r="A68" s="4"/>
@@ -2291,6 +2385,7 @@
       <c r="V68" s="4"/>
       <c r="W68" s="4"/>
       <c r="X68" s="4"/>
+      <c r="Y68" s="4"/>
     </row>
     <row r="69" ht="15.75" customHeight="1">
       <c r="A69" s="4"/>
@@ -2317,6 +2412,7 @@
       <c r="V69" s="4"/>
       <c r="W69" s="4"/>
       <c r="X69" s="4"/>
+      <c r="Y69" s="4"/>
     </row>
     <row r="70" ht="15.75" customHeight="1">
       <c r="A70" s="4"/>
@@ -2343,6 +2439,7 @@
       <c r="V70" s="4"/>
       <c r="W70" s="4"/>
       <c r="X70" s="4"/>
+      <c r="Y70" s="4"/>
     </row>
     <row r="71" ht="15.75" customHeight="1">
       <c r="A71" s="4"/>
@@ -2369,6 +2466,7 @@
       <c r="V71" s="4"/>
       <c r="W71" s="4"/>
       <c r="X71" s="4"/>
+      <c r="Y71" s="4"/>
     </row>
     <row r="72" ht="15.75" customHeight="1">
       <c r="A72" s="4"/>
@@ -2395,6 +2493,7 @@
       <c r="V72" s="4"/>
       <c r="W72" s="4"/>
       <c r="X72" s="4"/>
+      <c r="Y72" s="4"/>
     </row>
     <row r="73" ht="15.75" customHeight="1">
       <c r="A73" s="4"/>
@@ -2421,6 +2520,7 @@
       <c r="V73" s="4"/>
       <c r="W73" s="4"/>
       <c r="X73" s="4"/>
+      <c r="Y73" s="4"/>
     </row>
     <row r="74" ht="15.75" customHeight="1">
       <c r="A74" s="4"/>
@@ -2447,6 +2547,7 @@
       <c r="V74" s="4"/>
       <c r="W74" s="4"/>
       <c r="X74" s="4"/>
+      <c r="Y74" s="4"/>
     </row>
     <row r="75" ht="15.75" customHeight="1">
       <c r="A75" s="4"/>
@@ -2473,6 +2574,7 @@
       <c r="V75" s="4"/>
       <c r="W75" s="4"/>
       <c r="X75" s="4"/>
+      <c r="Y75" s="4"/>
     </row>
     <row r="76" ht="15.75" customHeight="1">
       <c r="A76" s="4"/>
@@ -2499,6 +2601,7 @@
       <c r="V76" s="4"/>
       <c r="W76" s="4"/>
       <c r="X76" s="4"/>
+      <c r="Y76" s="4"/>
     </row>
     <row r="77" ht="15.75" customHeight="1">
       <c r="A77" s="4"/>
@@ -2525,6 +2628,7 @@
       <c r="V77" s="4"/>
       <c r="W77" s="4"/>
       <c r="X77" s="4"/>
+      <c r="Y77" s="4"/>
     </row>
     <row r="78" ht="15.75" customHeight="1">
       <c r="A78" s="4"/>
@@ -2551,6 +2655,7 @@
       <c r="V78" s="4"/>
       <c r="W78" s="4"/>
       <c r="X78" s="4"/>
+      <c r="Y78" s="4"/>
     </row>
     <row r="79" ht="15.75" customHeight="1">
       <c r="A79" s="4"/>
@@ -2577,6 +2682,7 @@
       <c r="V79" s="4"/>
       <c r="W79" s="4"/>
       <c r="X79" s="4"/>
+      <c r="Y79" s="4"/>
     </row>
     <row r="80" ht="15.75" customHeight="1">
       <c r="A80" s="4"/>
@@ -2603,6 +2709,7 @@
       <c r="V80" s="4"/>
       <c r="W80" s="4"/>
       <c r="X80" s="4"/>
+      <c r="Y80" s="4"/>
     </row>
     <row r="81" ht="15.75" customHeight="1">
       <c r="A81" s="4"/>
@@ -2629,6 +2736,7 @@
       <c r="V81" s="4"/>
       <c r="W81" s="4"/>
       <c r="X81" s="4"/>
+      <c r="Y81" s="4"/>
     </row>
     <row r="82" ht="15.75" customHeight="1">
       <c r="A82" s="4"/>
@@ -2655,6 +2763,7 @@
       <c r="V82" s="4"/>
       <c r="W82" s="4"/>
       <c r="X82" s="4"/>
+      <c r="Y82" s="4"/>
     </row>
     <row r="83" ht="15.75" customHeight="1">
       <c r="A83" s="4"/>
@@ -2681,6 +2790,7 @@
       <c r="V83" s="4"/>
       <c r="W83" s="4"/>
       <c r="X83" s="4"/>
+      <c r="Y83" s="4"/>
     </row>
     <row r="84" ht="15.75" customHeight="1">
       <c r="A84" s="4"/>
@@ -2707,6 +2817,7 @@
       <c r="V84" s="4"/>
       <c r="W84" s="4"/>
       <c r="X84" s="4"/>
+      <c r="Y84" s="4"/>
     </row>
     <row r="85" ht="15.75" customHeight="1">
       <c r="A85" s="4"/>
@@ -2733,6 +2844,7 @@
       <c r="V85" s="4"/>
       <c r="W85" s="4"/>
       <c r="X85" s="4"/>
+      <c r="Y85" s="4"/>
     </row>
     <row r="86" ht="15.75" customHeight="1">
       <c r="A86" s="4"/>
@@ -2759,6 +2871,7 @@
       <c r="V86" s="4"/>
       <c r="W86" s="4"/>
       <c r="X86" s="4"/>
+      <c r="Y86" s="4"/>
     </row>
     <row r="87" ht="15.75" customHeight="1">
       <c r="A87" s="4"/>
@@ -2785,6 +2898,7 @@
       <c r="V87" s="4"/>
       <c r="W87" s="4"/>
       <c r="X87" s="4"/>
+      <c r="Y87" s="4"/>
     </row>
     <row r="88" ht="15.75" customHeight="1">
       <c r="A88" s="4"/>
@@ -2811,6 +2925,7 @@
       <c r="V88" s="4"/>
       <c r="W88" s="4"/>
       <c r="X88" s="4"/>
+      <c r="Y88" s="4"/>
     </row>
     <row r="89" ht="15.75" customHeight="1">
       <c r="A89" s="4"/>
@@ -2837,6 +2952,7 @@
       <c r="V89" s="4"/>
       <c r="W89" s="4"/>
       <c r="X89" s="4"/>
+      <c r="Y89" s="4"/>
     </row>
     <row r="90" ht="15.75" customHeight="1">
       <c r="A90" s="4"/>
@@ -2863,6 +2979,7 @@
       <c r="V90" s="4"/>
       <c r="W90" s="4"/>
       <c r="X90" s="4"/>
+      <c r="Y90" s="4"/>
     </row>
     <row r="91" ht="15.75" customHeight="1">
       <c r="A91" s="4"/>
@@ -2889,6 +3006,7 @@
       <c r="V91" s="4"/>
       <c r="W91" s="4"/>
       <c r="X91" s="4"/>
+      <c r="Y91" s="4"/>
     </row>
     <row r="92" ht="15.75" customHeight="1">
       <c r="A92" s="4"/>
@@ -2915,6 +3033,7 @@
       <c r="V92" s="4"/>
       <c r="W92" s="4"/>
       <c r="X92" s="4"/>
+      <c r="Y92" s="4"/>
     </row>
     <row r="93" ht="15.75" customHeight="1">
       <c r="A93" s="4"/>
@@ -2941,6 +3060,7 @@
       <c r="V93" s="4"/>
       <c r="W93" s="4"/>
       <c r="X93" s="4"/>
+      <c r="Y93" s="4"/>
     </row>
     <row r="94" ht="15.75" customHeight="1">
       <c r="A94" s="4"/>
@@ -2967,6 +3087,7 @@
       <c r="V94" s="4"/>
       <c r="W94" s="4"/>
       <c r="X94" s="4"/>
+      <c r="Y94" s="4"/>
     </row>
     <row r="95" ht="15.75" customHeight="1">
       <c r="A95" s="4"/>
@@ -2993,6 +3114,7 @@
       <c r="V95" s="4"/>
       <c r="W95" s="4"/>
       <c r="X95" s="4"/>
+      <c r="Y95" s="4"/>
     </row>
     <row r="96" ht="15.75" customHeight="1">
       <c r="A96" s="4"/>
@@ -3019,6 +3141,7 @@
       <c r="V96" s="4"/>
       <c r="W96" s="4"/>
       <c r="X96" s="4"/>
+      <c r="Y96" s="4"/>
     </row>
     <row r="97" ht="15.75" customHeight="1">
       <c r="A97" s="4"/>
@@ -3045,6 +3168,7 @@
       <c r="V97" s="4"/>
       <c r="W97" s="4"/>
       <c r="X97" s="4"/>
+      <c r="Y97" s="4"/>
     </row>
     <row r="98" ht="15.75" customHeight="1">
       <c r="A98" s="4"/>
@@ -3071,6 +3195,7 @@
       <c r="V98" s="4"/>
       <c r="W98" s="4"/>
       <c r="X98" s="4"/>
+      <c r="Y98" s="4"/>
     </row>
     <row r="99" ht="15.75" customHeight="1">
       <c r="A99" s="4"/>
@@ -3097,6 +3222,7 @@
       <c r="V99" s="4"/>
       <c r="W99" s="4"/>
       <c r="X99" s="4"/>
+      <c r="Y99" s="4"/>
     </row>
     <row r="100" ht="15.75" customHeight="1">
       <c r="A100" s="4"/>
@@ -3123,6 +3249,7 @@
       <c r="V100" s="4"/>
       <c r="W100" s="4"/>
       <c r="X100" s="4"/>
+      <c r="Y100" s="4"/>
     </row>
     <row r="101" ht="15.75" customHeight="1">
       <c r="A101" s="4"/>
@@ -3149,6 +3276,7 @@
       <c r="V101" s="4"/>
       <c r="W101" s="4"/>
       <c r="X101" s="4"/>
+      <c r="Y101" s="4"/>
     </row>
     <row r="102" ht="15.75" customHeight="1">
       <c r="A102" s="4"/>
@@ -3175,6 +3303,7 @@
       <c r="V102" s="4"/>
       <c r="W102" s="4"/>
       <c r="X102" s="4"/>
+      <c r="Y102" s="4"/>
     </row>
     <row r="103" ht="15.75" customHeight="1">
       <c r="A103" s="4"/>
@@ -3201,6 +3330,7 @@
       <c r="V103" s="4"/>
       <c r="W103" s="4"/>
       <c r="X103" s="4"/>
+      <c r="Y103" s="4"/>
     </row>
     <row r="104" ht="15.75" customHeight="1">
       <c r="A104" s="4"/>
@@ -3227,6 +3357,7 @@
       <c r="V104" s="4"/>
       <c r="W104" s="4"/>
       <c r="X104" s="4"/>
+      <c r="Y104" s="4"/>
     </row>
     <row r="105" ht="15.75" customHeight="1">
       <c r="A105" s="4"/>
@@ -3253,6 +3384,7 @@
       <c r="V105" s="4"/>
       <c r="W105" s="4"/>
       <c r="X105" s="4"/>
+      <c r="Y105" s="4"/>
     </row>
     <row r="106" ht="15.75" customHeight="1">
       <c r="A106" s="4"/>
@@ -3279,6 +3411,7 @@
       <c r="V106" s="4"/>
       <c r="W106" s="4"/>
       <c r="X106" s="4"/>
+      <c r="Y106" s="4"/>
     </row>
     <row r="107" ht="15.75" customHeight="1">
       <c r="A107" s="4"/>
@@ -3305,6 +3438,7 @@
       <c r="V107" s="4"/>
       <c r="W107" s="4"/>
       <c r="X107" s="4"/>
+      <c r="Y107" s="4"/>
     </row>
     <row r="108" ht="15.75" customHeight="1">
       <c r="A108" s="4"/>
@@ -3331,6 +3465,7 @@
       <c r="V108" s="4"/>
       <c r="W108" s="4"/>
       <c r="X108" s="4"/>
+      <c r="Y108" s="4"/>
     </row>
     <row r="109" ht="15.75" customHeight="1">
       <c r="A109" s="4"/>
@@ -3357,6 +3492,7 @@
       <c r="V109" s="4"/>
       <c r="W109" s="4"/>
       <c r="X109" s="4"/>
+      <c r="Y109" s="4"/>
     </row>
     <row r="110" ht="15.75" customHeight="1">
       <c r="A110" s="4"/>
@@ -3383,6 +3519,7 @@
       <c r="V110" s="4"/>
       <c r="W110" s="4"/>
       <c r="X110" s="4"/>
+      <c r="Y110" s="4"/>
     </row>
     <row r="111" ht="15.75" customHeight="1">
       <c r="A111" s="4"/>
@@ -3409,6 +3546,7 @@
       <c r="V111" s="4"/>
       <c r="W111" s="4"/>
       <c r="X111" s="4"/>
+      <c r="Y111" s="4"/>
     </row>
     <row r="112" ht="15.75" customHeight="1">
       <c r="A112" s="4"/>
@@ -3435,6 +3573,7 @@
       <c r="V112" s="4"/>
       <c r="W112" s="4"/>
       <c r="X112" s="4"/>
+      <c r="Y112" s="4"/>
     </row>
     <row r="113" ht="15.75" customHeight="1">
       <c r="A113" s="4"/>
@@ -3461,6 +3600,7 @@
       <c r="V113" s="4"/>
       <c r="W113" s="4"/>
       <c r="X113" s="4"/>
+      <c r="Y113" s="4"/>
     </row>
     <row r="114" ht="15.75" customHeight="1">
       <c r="A114" s="4"/>
@@ -3487,6 +3627,7 @@
       <c r="V114" s="4"/>
       <c r="W114" s="4"/>
       <c r="X114" s="4"/>
+      <c r="Y114" s="4"/>
     </row>
     <row r="115" ht="15.75" customHeight="1">
       <c r="A115" s="4"/>
@@ -3513,6 +3654,7 @@
       <c r="V115" s="4"/>
       <c r="W115" s="4"/>
       <c r="X115" s="4"/>
+      <c r="Y115" s="4"/>
     </row>
     <row r="116" ht="15.75" customHeight="1">
       <c r="A116" s="4"/>
@@ -3539,6 +3681,7 @@
       <c r="V116" s="4"/>
       <c r="W116" s="4"/>
       <c r="X116" s="4"/>
+      <c r="Y116" s="4"/>
     </row>
     <row r="117" ht="15.75" customHeight="1">
       <c r="A117" s="4"/>
@@ -3565,6 +3708,7 @@
       <c r="V117" s="4"/>
       <c r="W117" s="4"/>
       <c r="X117" s="4"/>
+      <c r="Y117" s="4"/>
     </row>
     <row r="118" ht="15.75" customHeight="1">
       <c r="A118" s="4"/>
@@ -3591,6 +3735,7 @@
       <c r="V118" s="4"/>
       <c r="W118" s="4"/>
       <c r="X118" s="4"/>
+      <c r="Y118" s="4"/>
     </row>
     <row r="119" ht="15.75" customHeight="1">
       <c r="A119" s="4"/>
@@ -3617,6 +3762,7 @@
       <c r="V119" s="4"/>
       <c r="W119" s="4"/>
       <c r="X119" s="4"/>
+      <c r="Y119" s="4"/>
     </row>
     <row r="120" ht="15.75" customHeight="1">
       <c r="A120" s="4"/>
@@ -3643,6 +3789,7 @@
       <c r="V120" s="4"/>
       <c r="W120" s="4"/>
       <c r="X120" s="4"/>
+      <c r="Y120" s="4"/>
     </row>
     <row r="121" ht="15.75" customHeight="1">
       <c r="A121" s="4"/>
@@ -3669,6 +3816,7 @@
       <c r="V121" s="4"/>
       <c r="W121" s="4"/>
       <c r="X121" s="4"/>
+      <c r="Y121" s="4"/>
     </row>
     <row r="122" ht="15.75" customHeight="1">
       <c r="A122" s="4"/>
@@ -3695,6 +3843,7 @@
       <c r="V122" s="4"/>
       <c r="W122" s="4"/>
       <c r="X122" s="4"/>
+      <c r="Y122" s="4"/>
     </row>
     <row r="123" ht="15.75" customHeight="1">
       <c r="A123" s="4"/>
@@ -3721,6 +3870,7 @@
       <c r="V123" s="4"/>
       <c r="W123" s="4"/>
       <c r="X123" s="4"/>
+      <c r="Y123" s="4"/>
     </row>
     <row r="124" ht="15.75" customHeight="1">
       <c r="A124" s="4"/>
@@ -3747,6 +3897,7 @@
       <c r="V124" s="4"/>
       <c r="W124" s="4"/>
       <c r="X124" s="4"/>
+      <c r="Y124" s="4"/>
     </row>
     <row r="125" ht="15.75" customHeight="1">
       <c r="A125" s="4"/>
@@ -3773,6 +3924,7 @@
       <c r="V125" s="4"/>
       <c r="W125" s="4"/>
       <c r="X125" s="4"/>
+      <c r="Y125" s="4"/>
     </row>
     <row r="126" ht="15.75" customHeight="1">
       <c r="A126" s="4"/>
@@ -3799,6 +3951,7 @@
       <c r="V126" s="4"/>
       <c r="W126" s="4"/>
       <c r="X126" s="4"/>
+      <c r="Y126" s="4"/>
     </row>
     <row r="127" ht="15.75" customHeight="1">
       <c r="A127" s="4"/>
@@ -3825,6 +3978,7 @@
       <c r="V127" s="4"/>
       <c r="W127" s="4"/>
       <c r="X127" s="4"/>
+      <c r="Y127" s="4"/>
     </row>
     <row r="128" ht="15.75" customHeight="1">
       <c r="A128" s="4"/>
@@ -3851,6 +4005,7 @@
       <c r="V128" s="4"/>
       <c r="W128" s="4"/>
       <c r="X128" s="4"/>
+      <c r="Y128" s="4"/>
     </row>
     <row r="129" ht="15.75" customHeight="1">
       <c r="A129" s="4"/>
@@ -3877,6 +4032,7 @@
       <c r="V129" s="4"/>
       <c r="W129" s="4"/>
       <c r="X129" s="4"/>
+      <c r="Y129" s="4"/>
     </row>
     <row r="130" ht="15.75" customHeight="1">
       <c r="A130" s="4"/>
@@ -3903,6 +4059,7 @@
       <c r="V130" s="4"/>
       <c r="W130" s="4"/>
       <c r="X130" s="4"/>
+      <c r="Y130" s="4"/>
     </row>
     <row r="131" ht="15.75" customHeight="1">
       <c r="A131" s="4"/>
@@ -3929,6 +4086,7 @@
       <c r="V131" s="4"/>
       <c r="W131" s="4"/>
       <c r="X131" s="4"/>
+      <c r="Y131" s="4"/>
     </row>
     <row r="132" ht="15.75" customHeight="1">
       <c r="A132" s="4"/>
@@ -3955,6 +4113,7 @@
       <c r="V132" s="4"/>
       <c r="W132" s="4"/>
       <c r="X132" s="4"/>
+      <c r="Y132" s="4"/>
     </row>
     <row r="133" ht="15.75" customHeight="1">
       <c r="A133" s="4"/>
@@ -3981,6 +4140,7 @@
       <c r="V133" s="4"/>
       <c r="W133" s="4"/>
       <c r="X133" s="4"/>
+      <c r="Y133" s="4"/>
     </row>
     <row r="134" ht="15.75" customHeight="1">
       <c r="A134" s="4"/>
@@ -4007,6 +4167,7 @@
       <c r="V134" s="4"/>
       <c r="W134" s="4"/>
       <c r="X134" s="4"/>
+      <c r="Y134" s="4"/>
     </row>
     <row r="135" ht="15.75" customHeight="1">
       <c r="A135" s="4"/>
@@ -4033,6 +4194,7 @@
       <c r="V135" s="4"/>
       <c r="W135" s="4"/>
       <c r="X135" s="4"/>
+      <c r="Y135" s="4"/>
     </row>
     <row r="136" ht="15.75" customHeight="1">
       <c r="A136" s="4"/>
@@ -4059,6 +4221,7 @@
       <c r="V136" s="4"/>
       <c r="W136" s="4"/>
       <c r="X136" s="4"/>
+      <c r="Y136" s="4"/>
     </row>
     <row r="137" ht="15.75" customHeight="1">
       <c r="A137" s="4"/>
@@ -4085,6 +4248,7 @@
       <c r="V137" s="4"/>
       <c r="W137" s="4"/>
       <c r="X137" s="4"/>
+      <c r="Y137" s="4"/>
     </row>
     <row r="138" ht="15.75" customHeight="1">
       <c r="A138" s="4"/>
@@ -4111,6 +4275,7 @@
       <c r="V138" s="4"/>
       <c r="W138" s="4"/>
       <c r="X138" s="4"/>
+      <c r="Y138" s="4"/>
     </row>
     <row r="139" ht="15.75" customHeight="1">
       <c r="A139" s="4"/>
@@ -4137,6 +4302,7 @@
       <c r="V139" s="4"/>
       <c r="W139" s="4"/>
       <c r="X139" s="4"/>
+      <c r="Y139" s="4"/>
     </row>
     <row r="140" ht="15.75" customHeight="1">
       <c r="A140" s="4"/>
@@ -4163,6 +4329,7 @@
       <c r="V140" s="4"/>
       <c r="W140" s="4"/>
       <c r="X140" s="4"/>
+      <c r="Y140" s="4"/>
     </row>
     <row r="141" ht="15.75" customHeight="1">
       <c r="A141" s="4"/>
@@ -4189,6 +4356,7 @@
       <c r="V141" s="4"/>
       <c r="W141" s="4"/>
       <c r="X141" s="4"/>
+      <c r="Y141" s="4"/>
     </row>
     <row r="142" ht="15.75" customHeight="1">
       <c r="A142" s="4"/>
@@ -4215,6 +4383,7 @@
       <c r="V142" s="4"/>
       <c r="W142" s="4"/>
       <c r="X142" s="4"/>
+      <c r="Y142" s="4"/>
     </row>
     <row r="143" ht="15.75" customHeight="1">
       <c r="A143" s="4"/>
@@ -4241,6 +4410,7 @@
       <c r="V143" s="4"/>
       <c r="W143" s="4"/>
       <c r="X143" s="4"/>
+      <c r="Y143" s="4"/>
     </row>
     <row r="144" ht="15.75" customHeight="1">
       <c r="A144" s="4"/>
@@ -4267,6 +4437,7 @@
       <c r="V144" s="4"/>
       <c r="W144" s="4"/>
       <c r="X144" s="4"/>
+      <c r="Y144" s="4"/>
     </row>
     <row r="145" ht="15.75" customHeight="1">
       <c r="A145" s="4"/>
@@ -4293,6 +4464,7 @@
       <c r="V145" s="4"/>
       <c r="W145" s="4"/>
       <c r="X145" s="4"/>
+      <c r="Y145" s="4"/>
     </row>
     <row r="146" ht="15.75" customHeight="1">
       <c r="A146" s="4"/>
@@ -4319,6 +4491,7 @@
       <c r="V146" s="4"/>
       <c r="W146" s="4"/>
       <c r="X146" s="4"/>
+      <c r="Y146" s="4"/>
     </row>
     <row r="147" ht="15.75" customHeight="1">
       <c r="A147" s="4"/>
@@ -4345,6 +4518,7 @@
       <c r="V147" s="4"/>
       <c r="W147" s="4"/>
       <c r="X147" s="4"/>
+      <c r="Y147" s="4"/>
     </row>
     <row r="148" ht="15.75" customHeight="1">
       <c r="A148" s="4"/>
@@ -4371,6 +4545,7 @@
       <c r="V148" s="4"/>
       <c r="W148" s="4"/>
       <c r="X148" s="4"/>
+      <c r="Y148" s="4"/>
     </row>
     <row r="149" ht="15.75" customHeight="1">
       <c r="A149" s="4"/>
@@ -4397,6 +4572,7 @@
       <c r="V149" s="4"/>
       <c r="W149" s="4"/>
       <c r="X149" s="4"/>
+      <c r="Y149" s="4"/>
     </row>
     <row r="150" ht="15.75" customHeight="1">
       <c r="A150" s="4"/>
@@ -4423,6 +4599,7 @@
       <c r="V150" s="4"/>
       <c r="W150" s="4"/>
       <c r="X150" s="4"/>
+      <c r="Y150" s="4"/>
     </row>
     <row r="151" ht="15.75" customHeight="1">
       <c r="A151" s="4"/>
@@ -4449,6 +4626,7 @@
       <c r="V151" s="4"/>
       <c r="W151" s="4"/>
       <c r="X151" s="4"/>
+      <c r="Y151" s="4"/>
     </row>
     <row r="152" ht="15.75" customHeight="1">
       <c r="A152" s="4"/>
@@ -4475,6 +4653,7 @@
       <c r="V152" s="4"/>
       <c r="W152" s="4"/>
       <c r="X152" s="4"/>
+      <c r="Y152" s="4"/>
     </row>
     <row r="153" ht="15.75" customHeight="1">
       <c r="A153" s="4"/>
@@ -4501,6 +4680,7 @@
       <c r="V153" s="4"/>
       <c r="W153" s="4"/>
       <c r="X153" s="4"/>
+      <c r="Y153" s="4"/>
     </row>
     <row r="154" ht="15.75" customHeight="1">
       <c r="A154" s="4"/>
@@ -4527,6 +4707,7 @@
       <c r="V154" s="4"/>
       <c r="W154" s="4"/>
       <c r="X154" s="4"/>
+      <c r="Y154" s="4"/>
     </row>
     <row r="155" ht="15.75" customHeight="1">
       <c r="A155" s="4"/>
@@ -4553,6 +4734,7 @@
       <c r="V155" s="4"/>
       <c r="W155" s="4"/>
       <c r="X155" s="4"/>
+      <c r="Y155" s="4"/>
     </row>
     <row r="156" ht="15.75" customHeight="1">
       <c r="A156" s="4"/>
@@ -4579,6 +4761,7 @@
       <c r="V156" s="4"/>
       <c r="W156" s="4"/>
       <c r="X156" s="4"/>
+      <c r="Y156" s="4"/>
     </row>
     <row r="157" ht="15.75" customHeight="1">
       <c r="A157" s="4"/>
@@ -4605,6 +4788,7 @@
       <c r="V157" s="4"/>
       <c r="W157" s="4"/>
       <c r="X157" s="4"/>
+      <c r="Y157" s="4"/>
     </row>
     <row r="158" ht="15.75" customHeight="1">
       <c r="A158" s="4"/>
@@ -4631,6 +4815,7 @@
       <c r="V158" s="4"/>
       <c r="W158" s="4"/>
       <c r="X158" s="4"/>
+      <c r="Y158" s="4"/>
     </row>
     <row r="159" ht="15.75" customHeight="1">
       <c r="A159" s="4"/>
@@ -4657,6 +4842,7 @@
       <c r="V159" s="4"/>
       <c r="W159" s="4"/>
       <c r="X159" s="4"/>
+      <c r="Y159" s="4"/>
     </row>
     <row r="160" ht="15.75" customHeight="1">
       <c r="A160" s="4"/>
@@ -4683,6 +4869,7 @@
       <c r="V160" s="4"/>
       <c r="W160" s="4"/>
       <c r="X160" s="4"/>
+      <c r="Y160" s="4"/>
     </row>
     <row r="161" ht="15.75" customHeight="1">
       <c r="A161" s="4"/>
@@ -4709,6 +4896,7 @@
       <c r="V161" s="4"/>
       <c r="W161" s="4"/>
       <c r="X161" s="4"/>
+      <c r="Y161" s="4"/>
     </row>
     <row r="162" ht="15.75" customHeight="1">
       <c r="A162" s="4"/>
@@ -4735,6 +4923,7 @@
       <c r="V162" s="4"/>
       <c r="W162" s="4"/>
       <c r="X162" s="4"/>
+      <c r="Y162" s="4"/>
     </row>
     <row r="163" ht="15.75" customHeight="1">
       <c r="A163" s="4"/>
@@ -4761,6 +4950,7 @@
       <c r="V163" s="4"/>
       <c r="W163" s="4"/>
       <c r="X163" s="4"/>
+      <c r="Y163" s="4"/>
     </row>
     <row r="164" ht="15.75" customHeight="1">
       <c r="A164" s="4"/>
@@ -4787,6 +4977,7 @@
       <c r="V164" s="4"/>
       <c r="W164" s="4"/>
       <c r="X164" s="4"/>
+      <c r="Y164" s="4"/>
     </row>
     <row r="165" ht="15.75" customHeight="1">
       <c r="A165" s="4"/>
@@ -4813,6 +5004,7 @@
       <c r="V165" s="4"/>
       <c r="W165" s="4"/>
       <c r="X165" s="4"/>
+      <c r="Y165" s="4"/>
     </row>
     <row r="166" ht="15.75" customHeight="1">
       <c r="A166" s="4"/>
@@ -4839,6 +5031,7 @@
       <c r="V166" s="4"/>
       <c r="W166" s="4"/>
       <c r="X166" s="4"/>
+      <c r="Y166" s="4"/>
     </row>
     <row r="167" ht="15.75" customHeight="1">
       <c r="A167" s="4"/>
@@ -4865,6 +5058,7 @@
       <c r="V167" s="4"/>
       <c r="W167" s="4"/>
       <c r="X167" s="4"/>
+      <c r="Y167" s="4"/>
     </row>
     <row r="168" ht="15.75" customHeight="1">
       <c r="A168" s="4"/>
@@ -4891,6 +5085,7 @@
       <c r="V168" s="4"/>
       <c r="W168" s="4"/>
       <c r="X168" s="4"/>
+      <c r="Y168" s="4"/>
     </row>
     <row r="169" ht="15.75" customHeight="1">
       <c r="A169" s="4"/>
@@ -4917,6 +5112,7 @@
       <c r="V169" s="4"/>
       <c r="W169" s="4"/>
       <c r="X169" s="4"/>
+      <c r="Y169" s="4"/>
     </row>
     <row r="170" ht="15.75" customHeight="1">
       <c r="A170" s="4"/>
@@ -4943,6 +5139,7 @@
       <c r="V170" s="4"/>
       <c r="W170" s="4"/>
       <c r="X170" s="4"/>
+      <c r="Y170" s="4"/>
     </row>
     <row r="171" ht="15.75" customHeight="1">
       <c r="A171" s="4"/>
@@ -4969,6 +5166,7 @@
       <c r="V171" s="4"/>
       <c r="W171" s="4"/>
       <c r="X171" s="4"/>
+      <c r="Y171" s="4"/>
     </row>
     <row r="172" ht="15.75" customHeight="1">
       <c r="A172" s="4"/>
@@ -4995,6 +5193,7 @@
       <c r="V172" s="4"/>
       <c r="W172" s="4"/>
       <c r="X172" s="4"/>
+      <c r="Y172" s="4"/>
     </row>
     <row r="173" ht="15.75" customHeight="1">
       <c r="A173" s="4"/>
@@ -5021,6 +5220,7 @@
       <c r="V173" s="4"/>
       <c r="W173" s="4"/>
       <c r="X173" s="4"/>
+      <c r="Y173" s="4"/>
     </row>
     <row r="174" ht="15.75" customHeight="1">
       <c r="A174" s="4"/>
@@ -5047,6 +5247,7 @@
       <c r="V174" s="4"/>
       <c r="W174" s="4"/>
       <c r="X174" s="4"/>
+      <c r="Y174" s="4"/>
     </row>
     <row r="175" ht="15.75" customHeight="1">
       <c r="A175" s="4"/>
@@ -5073,6 +5274,7 @@
       <c r="V175" s="4"/>
       <c r="W175" s="4"/>
       <c r="X175" s="4"/>
+      <c r="Y175" s="4"/>
     </row>
     <row r="176" ht="15.75" customHeight="1">
       <c r="A176" s="4"/>
@@ -5099,6 +5301,7 @@
       <c r="V176" s="4"/>
       <c r="W176" s="4"/>
       <c r="X176" s="4"/>
+      <c r="Y176" s="4"/>
     </row>
     <row r="177" ht="15.75" customHeight="1">
       <c r="A177" s="4"/>
@@ -5125,6 +5328,7 @@
       <c r="V177" s="4"/>
       <c r="W177" s="4"/>
       <c r="X177" s="4"/>
+      <c r="Y177" s="4"/>
     </row>
     <row r="178" ht="15.75" customHeight="1">
       <c r="A178" s="4"/>
@@ -5151,6 +5355,7 @@
       <c r="V178" s="4"/>
       <c r="W178" s="4"/>
       <c r="X178" s="4"/>
+      <c r="Y178" s="4"/>
     </row>
     <row r="179" ht="15.75" customHeight="1">
       <c r="A179" s="4"/>
@@ -5177,6 +5382,7 @@
       <c r="V179" s="4"/>
       <c r="W179" s="4"/>
       <c r="X179" s="4"/>
+      <c r="Y179" s="4"/>
     </row>
     <row r="180" ht="15.75" customHeight="1">
       <c r="A180" s="4"/>
@@ -5203,6 +5409,7 @@
       <c r="V180" s="4"/>
       <c r="W180" s="4"/>
       <c r="X180" s="4"/>
+      <c r="Y180" s="4"/>
     </row>
     <row r="181" ht="15.75" customHeight="1">
       <c r="A181" s="4"/>
@@ -5229,6 +5436,7 @@
       <c r="V181" s="4"/>
       <c r="W181" s="4"/>
       <c r="X181" s="4"/>
+      <c r="Y181" s="4"/>
     </row>
     <row r="182" ht="15.75" customHeight="1">
       <c r="A182" s="4"/>
@@ -5255,6 +5463,7 @@
       <c r="V182" s="4"/>
       <c r="W182" s="4"/>
       <c r="X182" s="4"/>
+      <c r="Y182" s="4"/>
     </row>
     <row r="183" ht="15.75" customHeight="1">
       <c r="A183" s="4"/>
@@ -5281,6 +5490,7 @@
       <c r="V183" s="4"/>
       <c r="W183" s="4"/>
       <c r="X183" s="4"/>
+      <c r="Y183" s="4"/>
     </row>
     <row r="184" ht="15.75" customHeight="1">
       <c r="A184" s="4"/>
@@ -5307,6 +5517,7 @@
       <c r="V184" s="4"/>
       <c r="W184" s="4"/>
       <c r="X184" s="4"/>
+      <c r="Y184" s="4"/>
     </row>
     <row r="185" ht="15.75" customHeight="1">
       <c r="A185" s="4"/>
@@ -5333,6 +5544,7 @@
       <c r="V185" s="4"/>
       <c r="W185" s="4"/>
       <c r="X185" s="4"/>
+      <c r="Y185" s="4"/>
     </row>
     <row r="186" ht="15.75" customHeight="1">
       <c r="A186" s="4"/>
@@ -5359,6 +5571,7 @@
       <c r="V186" s="4"/>
       <c r="W186" s="4"/>
       <c r="X186" s="4"/>
+      <c r="Y186" s="4"/>
     </row>
     <row r="187" ht="15.75" customHeight="1">
       <c r="A187" s="4"/>
@@ -5385,6 +5598,7 @@
       <c r="V187" s="4"/>
       <c r="W187" s="4"/>
       <c r="X187" s="4"/>
+      <c r="Y187" s="4"/>
     </row>
     <row r="188" ht="15.75" customHeight="1">
       <c r="A188" s="4"/>
@@ -5411,6 +5625,7 @@
       <c r="V188" s="4"/>
       <c r="W188" s="4"/>
       <c r="X188" s="4"/>
+      <c r="Y188" s="4"/>
     </row>
     <row r="189" ht="15.75" customHeight="1">
       <c r="A189" s="4"/>
@@ -5437,6 +5652,7 @@
       <c r="V189" s="4"/>
       <c r="W189" s="4"/>
       <c r="X189" s="4"/>
+      <c r="Y189" s="4"/>
     </row>
     <row r="190" ht="15.75" customHeight="1">
       <c r="A190" s="4"/>
@@ -5463,6 +5679,7 @@
       <c r="V190" s="4"/>
       <c r="W190" s="4"/>
       <c r="X190" s="4"/>
+      <c r="Y190" s="4"/>
     </row>
     <row r="191" ht="15.75" customHeight="1">
       <c r="A191" s="4"/>
@@ -5489,6 +5706,7 @@
       <c r="V191" s="4"/>
       <c r="W191" s="4"/>
       <c r="X191" s="4"/>
+      <c r="Y191" s="4"/>
     </row>
     <row r="192" ht="15.75" customHeight="1">
       <c r="A192" s="4"/>
@@ -5515,6 +5733,7 @@
       <c r="V192" s="4"/>
       <c r="W192" s="4"/>
       <c r="X192" s="4"/>
+      <c r="Y192" s="4"/>
     </row>
     <row r="193" ht="15.75" customHeight="1">
       <c r="A193" s="4"/>
@@ -5541,6 +5760,7 @@
       <c r="V193" s="4"/>
       <c r="W193" s="4"/>
       <c r="X193" s="4"/>
+      <c r="Y193" s="4"/>
     </row>
     <row r="194" ht="15.75" customHeight="1">
       <c r="A194" s="4"/>
@@ -5567,6 +5787,7 @@
       <c r="V194" s="4"/>
       <c r="W194" s="4"/>
       <c r="X194" s="4"/>
+      <c r="Y194" s="4"/>
     </row>
     <row r="195" ht="15.75" customHeight="1">
       <c r="A195" s="4"/>
@@ -5593,6 +5814,7 @@
       <c r="V195" s="4"/>
       <c r="W195" s="4"/>
       <c r="X195" s="4"/>
+      <c r="Y195" s="4"/>
     </row>
     <row r="196" ht="15.75" customHeight="1">
       <c r="A196" s="4"/>
@@ -5619,6 +5841,7 @@
       <c r="V196" s="4"/>
       <c r="W196" s="4"/>
       <c r="X196" s="4"/>
+      <c r="Y196" s="4"/>
     </row>
     <row r="197" ht="15.75" customHeight="1">
       <c r="A197" s="4"/>
@@ -5645,6 +5868,7 @@
       <c r="V197" s="4"/>
       <c r="W197" s="4"/>
       <c r="X197" s="4"/>
+      <c r="Y197" s="4"/>
     </row>
     <row r="198" ht="15.75" customHeight="1">
       <c r="A198" s="4"/>
@@ -5671,6 +5895,7 @@
       <c r="V198" s="4"/>
       <c r="W198" s="4"/>
       <c r="X198" s="4"/>
+      <c r="Y198" s="4"/>
     </row>
     <row r="199" ht="15.75" customHeight="1">
       <c r="A199" s="4"/>
@@ -5697,6 +5922,7 @@
       <c r="V199" s="4"/>
       <c r="W199" s="4"/>
       <c r="X199" s="4"/>
+      <c r="Y199" s="4"/>
     </row>
     <row r="200" ht="15.75" customHeight="1">
       <c r="A200" s="4"/>
@@ -5723,6 +5949,7 @@
       <c r="V200" s="4"/>
       <c r="W200" s="4"/>
       <c r="X200" s="4"/>
+      <c r="Y200" s="4"/>
     </row>
     <row r="201" ht="15.75" customHeight="1">
       <c r="A201" s="4"/>
@@ -5749,6 +5976,7 @@
       <c r="V201" s="4"/>
       <c r="W201" s="4"/>
       <c r="X201" s="4"/>
+      <c r="Y201" s="4"/>
     </row>
     <row r="202" ht="15.75" customHeight="1">
       <c r="A202" s="4"/>
@@ -5775,6 +6003,7 @@
       <c r="V202" s="4"/>
       <c r="W202" s="4"/>
       <c r="X202" s="4"/>
+      <c r="Y202" s="4"/>
     </row>
     <row r="203" ht="15.75" customHeight="1">
       <c r="A203" s="4"/>
@@ -5801,6 +6030,7 @@
       <c r="V203" s="4"/>
       <c r="W203" s="4"/>
       <c r="X203" s="4"/>
+      <c r="Y203" s="4"/>
     </row>
     <row r="204" ht="15.75" customHeight="1">
       <c r="A204" s="4"/>
@@ -5827,6 +6057,7 @@
       <c r="V204" s="4"/>
       <c r="W204" s="4"/>
       <c r="X204" s="4"/>
+      <c r="Y204" s="4"/>
     </row>
     <row r="205" ht="15.75" customHeight="1">
       <c r="A205" s="4"/>
@@ -5853,6 +6084,7 @@
       <c r="V205" s="4"/>
       <c r="W205" s="4"/>
       <c r="X205" s="4"/>
+      <c r="Y205" s="4"/>
     </row>
     <row r="206" ht="15.75" customHeight="1">
       <c r="A206" s="4"/>
@@ -5879,6 +6111,7 @@
       <c r="V206" s="4"/>
       <c r="W206" s="4"/>
       <c r="X206" s="4"/>
+      <c r="Y206" s="4"/>
     </row>
     <row r="207" ht="15.75" customHeight="1">
       <c r="A207" s="4"/>
@@ -5905,6 +6138,7 @@
       <c r="V207" s="4"/>
       <c r="W207" s="4"/>
       <c r="X207" s="4"/>
+      <c r="Y207" s="4"/>
     </row>
     <row r="208" ht="15.75" customHeight="1">
       <c r="A208" s="4"/>
@@ -5931,6 +6165,7 @@
       <c r="V208" s="4"/>
       <c r="W208" s="4"/>
       <c r="X208" s="4"/>
+      <c r="Y208" s="4"/>
     </row>
     <row r="209" ht="15.75" customHeight="1">
       <c r="A209" s="4"/>
@@ -5957,6 +6192,7 @@
       <c r="V209" s="4"/>
       <c r="W209" s="4"/>
       <c r="X209" s="4"/>
+      <c r="Y209" s="4"/>
     </row>
     <row r="210" ht="15.75" customHeight="1">
       <c r="A210" s="4"/>
@@ -5983,6 +6219,7 @@
       <c r="V210" s="4"/>
       <c r="W210" s="4"/>
       <c r="X210" s="4"/>
+      <c r="Y210" s="4"/>
     </row>
     <row r="211" ht="15.75" customHeight="1">
       <c r="A211" s="4"/>
@@ -6009,6 +6246,7 @@
       <c r="V211" s="4"/>
       <c r="W211" s="4"/>
       <c r="X211" s="4"/>
+      <c r="Y211" s="4"/>
     </row>
     <row r="212" ht="15.75" customHeight="1">
       <c r="A212" s="4"/>
@@ -6035,6 +6273,7 @@
       <c r="V212" s="4"/>
       <c r="W212" s="4"/>
       <c r="X212" s="4"/>
+      <c r="Y212" s="4"/>
     </row>
     <row r="213" ht="15.75" customHeight="1">
       <c r="A213" s="4"/>
@@ -6061,6 +6300,7 @@
       <c r="V213" s="4"/>
       <c r="W213" s="4"/>
       <c r="X213" s="4"/>
+      <c r="Y213" s="4"/>
     </row>
     <row r="214" ht="15.75" customHeight="1">
       <c r="A214" s="4"/>
@@ -6087,6 +6327,7 @@
       <c r="V214" s="4"/>
       <c r="W214" s="4"/>
       <c r="X214" s="4"/>
+      <c r="Y214" s="4"/>
     </row>
     <row r="215" ht="15.75" customHeight="1">
       <c r="A215" s="4"/>
@@ -6113,6 +6354,7 @@
       <c r="V215" s="4"/>
       <c r="W215" s="4"/>
       <c r="X215" s="4"/>
+      <c r="Y215" s="4"/>
     </row>
     <row r="216" ht="15.75" customHeight="1">
       <c r="A216" s="4"/>
@@ -6139,6 +6381,7 @@
       <c r="V216" s="4"/>
       <c r="W216" s="4"/>
       <c r="X216" s="4"/>
+      <c r="Y216" s="4"/>
     </row>
     <row r="217" ht="15.75" customHeight="1">
       <c r="A217" s="4"/>
@@ -6165,6 +6408,7 @@
       <c r="V217" s="4"/>
       <c r="W217" s="4"/>
       <c r="X217" s="4"/>
+      <c r="Y217" s="4"/>
     </row>
     <row r="218" ht="15.75" customHeight="1">
       <c r="A218" s="4"/>
@@ -6191,6 +6435,7 @@
       <c r="V218" s="4"/>
       <c r="W218" s="4"/>
       <c r="X218" s="4"/>
+      <c r="Y218" s="4"/>
     </row>
     <row r="219" ht="15.75" customHeight="1">
       <c r="A219" s="4"/>
@@ -6217,6 +6462,7 @@
       <c r="V219" s="4"/>
       <c r="W219" s="4"/>
       <c r="X219" s="4"/>
+      <c r="Y219" s="4"/>
     </row>
     <row r="220" ht="15.75" customHeight="1">
       <c r="A220" s="4"/>
@@ -6243,6 +6489,7 @@
       <c r="V220" s="4"/>
       <c r="W220" s="4"/>
       <c r="X220" s="4"/>
+      <c r="Y220" s="4"/>
     </row>
     <row r="221" ht="15.75" customHeight="1"/>
     <row r="222" ht="15.75" customHeight="1"/>

</xml_diff>

<commit_message>
test: validate product removal from cart
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/testData_Appium_myDemoApp.xlsx
+++ b/src/test/resources/testData/testData_Appium_myDemoApp.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="44">
   <si>
     <t>CT</t>
   </si>
@@ -794,7 +794,9 @@
         <v>30</v>
       </c>
       <c r="F11" s="3"/>
-      <c r="G11" s="3"/>
+      <c r="G11" s="3" t="s">
+        <v>32</v>
+      </c>
       <c r="H11" s="1"/>
       <c r="I11" s="1"/>
       <c r="J11" s="1"/>
@@ -895,9 +897,13 @@
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
       <c r="D14" s="1"/>
-      <c r="E14" s="1"/>
+      <c r="E14" s="3" t="s">
+        <v>30</v>
+      </c>
       <c r="F14" s="1"/>
-      <c r="G14" s="1"/>
+      <c r="G14" s="3" t="s">
+        <v>32</v>
+      </c>
       <c r="H14" s="1"/>
       <c r="I14" s="1"/>
       <c r="J14" s="1"/>

</xml_diff>

<commit_message>
test: validate total price on cart page
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/testData_Appium_myDemoApp.xlsx
+++ b/src/test/resources/testData/testData_Appium_myDemoApp.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="45">
   <si>
     <t>CT</t>
   </si>
@@ -28,7 +28,7 @@
     <t>PRODUCT_NAME</t>
   </si>
   <si>
-    <t>PRODUCT_NAME_2</t>
+    <t>PRODUCT_QUANTITY</t>
   </si>
   <si>
     <t>PRODUCT_COLOR</t>
@@ -130,6 +130,9 @@
     <t>014</t>
   </si>
   <si>
+    <t>5</t>
+  </si>
+  <si>
     <t>015</t>
   </si>
   <si>
@@ -190,7 +193,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -205,6 +208,9 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf quotePrefix="1" borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="bottom"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -930,8 +936,12 @@
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
       <c r="D15" s="1"/>
-      <c r="E15" s="1"/>
-      <c r="F15" s="1"/>
+      <c r="E15" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="F15" s="5" t="s">
+        <v>39</v>
+      </c>
       <c r="G15" s="1"/>
       <c r="H15" s="1"/>
       <c r="I15" s="1"/>
@@ -954,7 +964,7 @@
     </row>
     <row r="16" ht="15.75" customHeight="1">
       <c r="A16" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B16" s="1"/>
       <c r="C16" s="1"/>
@@ -983,7 +993,7 @@
     </row>
     <row r="17" ht="15.75" customHeight="1">
       <c r="A17" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B17" s="1"/>
       <c r="C17" s="1"/>
@@ -1012,7 +1022,7 @@
     </row>
     <row r="18" ht="15.75" customHeight="1">
       <c r="A18" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B18" s="1"/>
       <c r="C18" s="1"/>
@@ -1041,7 +1051,7 @@
     </row>
     <row r="19" ht="15.75" customHeight="1">
       <c r="A19" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B19" s="1"/>
       <c r="C19" s="1"/>
@@ -1070,7 +1080,7 @@
     </row>
     <row r="20" ht="15.75" customHeight="1">
       <c r="A20" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B20" s="1"/>
       <c r="C20" s="1"/>

</xml_diff>

<commit_message>
test: validate address error message
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/testData_Appium_myDemoApp.xlsx
+++ b/src/test/resources/testData/testData_Appium_myDemoApp.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="41">
   <si>
     <t>CT</t>
   </si>
@@ -34,28 +34,16 @@
     <t>PRODUCT_COLOR</t>
   </si>
   <si>
-    <t>FIRSTNAME</t>
+    <t>FULL_NAME</t>
   </si>
   <si>
-    <t>LASTNAME</t>
-  </si>
-  <si>
-    <t>COMPANY</t>
-  </si>
-  <si>
-    <t>ADDRESS1</t>
-  </si>
-  <si>
-    <t>ADDRESS2</t>
+    <t>ADDRESS</t>
   </si>
   <si>
     <t>COUNTRY</t>
   </si>
   <si>
     <t>ZIPCODE</t>
-  </si>
-  <si>
-    <t>STATE</t>
   </si>
   <si>
     <t>CITY</t>
@@ -436,13 +424,11 @@
     <col customWidth="1" min="5" max="5" width="33.25"/>
     <col customWidth="1" min="6" max="6" width="42.88"/>
     <col customWidth="1" min="7" max="7" width="31.38"/>
-    <col customWidth="1" min="8" max="8" width="18.38"/>
+    <col customWidth="1" min="8" max="8" width="18.63"/>
     <col customWidth="1" min="9" max="9" width="17.13"/>
-    <col customWidth="1" min="10" max="10" width="16.0"/>
-    <col customWidth="1" min="11" max="12" width="17.13"/>
-    <col customWidth="1" min="13" max="13" width="15.75"/>
-    <col customWidth="1" min="14" max="14" width="14.38"/>
-    <col customWidth="1" min="17" max="17" width="27.0"/>
+    <col customWidth="1" min="10" max="10" width="15.75"/>
+    <col customWidth="1" min="11" max="11" width="14.38"/>
+    <col customWidth="1" min="13" max="13" width="27.0"/>
   </cols>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
@@ -467,10 +453,10 @@
       <c r="G1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="3" t="s">
         <v>8</v>
       </c>
       <c r="J1" s="1" t="s">
@@ -485,36 +471,24 @@
       <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="P1" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="Q1" s="1" t="s">
-        <v>16</v>
-      </c>
+      <c r="N1" s="4"/>
+      <c r="O1" s="4"/>
+      <c r="P1" s="4"/>
+      <c r="Q1" s="4"/>
       <c r="R1" s="4"/>
       <c r="S1" s="4"/>
       <c r="T1" s="4"/>
       <c r="U1" s="4"/>
-      <c r="V1" s="4"/>
-      <c r="W1" s="4"/>
-      <c r="X1" s="4"/>
-      <c r="Y1" s="4"/>
     </row>
     <row r="2" ht="15.75" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
@@ -526,22 +500,18 @@
       <c r="K2" s="1"/>
       <c r="L2" s="1"/>
       <c r="M2" s="1"/>
-      <c r="N2" s="1"/>
-      <c r="O2" s="1"/>
-      <c r="P2" s="1"/>
-      <c r="Q2" s="1"/>
+      <c r="N2" s="4"/>
+      <c r="O2" s="4"/>
+      <c r="P2" s="4"/>
+      <c r="Q2" s="4"/>
       <c r="R2" s="4"/>
       <c r="S2" s="4"/>
       <c r="T2" s="4"/>
       <c r="U2" s="4"/>
-      <c r="V2" s="4"/>
-      <c r="W2" s="4"/>
-      <c r="X2" s="4"/>
-      <c r="Y2" s="4"/>
     </row>
     <row r="3" ht="15.75" customHeight="1">
       <c r="A3" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
@@ -555,28 +525,24 @@
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
-      <c r="N3" s="1"/>
-      <c r="O3" s="1"/>
-      <c r="P3" s="1"/>
-      <c r="Q3" s="1"/>
+      <c r="N3" s="4"/>
+      <c r="O3" s="4"/>
+      <c r="P3" s="4"/>
+      <c r="Q3" s="4"/>
       <c r="R3" s="4"/>
       <c r="S3" s="4"/>
       <c r="T3" s="4"/>
       <c r="U3" s="4"/>
-      <c r="V3" s="4"/>
-      <c r="W3" s="4"/>
-      <c r="X3" s="4"/>
-      <c r="Y3" s="4"/>
     </row>
     <row r="4" ht="15.75" customHeight="1">
       <c r="A4" s="1" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
@@ -588,27 +554,23 @@
       <c r="K4" s="1"/>
       <c r="L4" s="1"/>
       <c r="M4" s="1"/>
-      <c r="N4" s="1"/>
-      <c r="O4" s="1"/>
-      <c r="P4" s="1"/>
-      <c r="Q4" s="1"/>
+      <c r="N4" s="4"/>
+      <c r="O4" s="4"/>
+      <c r="P4" s="4"/>
+      <c r="Q4" s="4"/>
       <c r="R4" s="4"/>
       <c r="S4" s="4"/>
       <c r="T4" s="4"/>
       <c r="U4" s="4"/>
-      <c r="V4" s="4"/>
-      <c r="W4" s="4"/>
-      <c r="X4" s="4"/>
-      <c r="Y4" s="4"/>
     </row>
     <row r="5" ht="15.75" customHeight="1">
       <c r="A5" s="1" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
       <c r="D5" s="1" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="E5" s="1"/>
       <c r="F5" s="1"/>
@@ -619,27 +581,23 @@
       <c r="K5" s="1"/>
       <c r="L5" s="1"/>
       <c r="M5" s="1"/>
-      <c r="N5" s="1"/>
-      <c r="O5" s="1"/>
-      <c r="P5" s="1"/>
-      <c r="Q5" s="1"/>
+      <c r="N5" s="4"/>
+      <c r="O5" s="4"/>
+      <c r="P5" s="4"/>
+      <c r="Q5" s="4"/>
       <c r="R5" s="4"/>
       <c r="S5" s="4"/>
       <c r="T5" s="4"/>
       <c r="U5" s="4"/>
-      <c r="V5" s="4"/>
-      <c r="W5" s="4"/>
-      <c r="X5" s="4"/>
-      <c r="Y5" s="4"/>
     </row>
     <row r="6" ht="15.75" customHeight="1">
       <c r="A6" s="1" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
       <c r="D6" s="1" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="E6" s="1"/>
       <c r="F6" s="1"/>
@@ -650,27 +608,23 @@
       <c r="K6" s="1"/>
       <c r="L6" s="1"/>
       <c r="M6" s="1"/>
-      <c r="N6" s="1"/>
-      <c r="O6" s="1"/>
-      <c r="P6" s="1"/>
-      <c r="Q6" s="1"/>
+      <c r="N6" s="4"/>
+      <c r="O6" s="4"/>
+      <c r="P6" s="4"/>
+      <c r="Q6" s="4"/>
       <c r="R6" s="4"/>
       <c r="S6" s="4"/>
       <c r="T6" s="4"/>
       <c r="U6" s="4"/>
-      <c r="V6" s="4"/>
-      <c r="W6" s="4"/>
-      <c r="X6" s="4"/>
-      <c r="Y6" s="4"/>
     </row>
     <row r="7" ht="15.75" customHeight="1">
       <c r="A7" s="1" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
       <c r="D7" s="1" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="E7" s="1"/>
       <c r="F7" s="1"/>
@@ -681,27 +635,23 @@
       <c r="K7" s="1"/>
       <c r="L7" s="1"/>
       <c r="M7" s="1"/>
-      <c r="N7" s="1"/>
-      <c r="O7" s="1"/>
-      <c r="P7" s="1"/>
-      <c r="Q7" s="1"/>
+      <c r="N7" s="4"/>
+      <c r="O7" s="4"/>
+      <c r="P7" s="4"/>
+      <c r="Q7" s="4"/>
       <c r="R7" s="4"/>
       <c r="S7" s="4"/>
       <c r="T7" s="4"/>
       <c r="U7" s="4"/>
-      <c r="V7" s="4"/>
-      <c r="W7" s="4"/>
-      <c r="X7" s="4"/>
-      <c r="Y7" s="4"/>
     </row>
     <row r="8" ht="15.75" customHeight="1">
       <c r="A8" s="1" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
       <c r="D8" s="1" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="E8" s="1"/>
       <c r="F8" s="1"/>
@@ -712,28 +662,24 @@
       <c r="K8" s="1"/>
       <c r="L8" s="1"/>
       <c r="M8" s="1"/>
-      <c r="N8" s="1"/>
-      <c r="O8" s="1"/>
-      <c r="P8" s="1"/>
-      <c r="Q8" s="1"/>
+      <c r="N8" s="4"/>
+      <c r="O8" s="4"/>
+      <c r="P8" s="4"/>
+      <c r="Q8" s="4"/>
       <c r="R8" s="4"/>
       <c r="S8" s="4"/>
       <c r="T8" s="4"/>
       <c r="U8" s="4"/>
-      <c r="V8" s="4"/>
-      <c r="W8" s="4"/>
-      <c r="X8" s="4"/>
-      <c r="Y8" s="4"/>
     </row>
     <row r="9" ht="15.75" customHeight="1">
       <c r="A9" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
       <c r="D9" s="1"/>
       <c r="E9" s="3" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="F9" s="3"/>
       <c r="G9" s="3"/>
@@ -743,32 +689,28 @@
       <c r="K9" s="1"/>
       <c r="L9" s="1"/>
       <c r="M9" s="1"/>
-      <c r="N9" s="1"/>
-      <c r="O9" s="1"/>
-      <c r="P9" s="1"/>
-      <c r="Q9" s="1"/>
+      <c r="N9" s="4"/>
+      <c r="O9" s="4"/>
+      <c r="P9" s="4"/>
+      <c r="Q9" s="4"/>
       <c r="R9" s="4"/>
       <c r="S9" s="4"/>
       <c r="T9" s="4"/>
       <c r="U9" s="4"/>
-      <c r="V9" s="4"/>
-      <c r="W9" s="4"/>
-      <c r="X9" s="4"/>
-      <c r="Y9" s="4"/>
     </row>
     <row r="10" ht="15.75" customHeight="1">
       <c r="A10" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
       <c r="D10" s="1"/>
       <c r="E10" s="3" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="F10" s="3"/>
       <c r="G10" s="3" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="H10" s="1"/>
       <c r="I10" s="1"/>
@@ -776,32 +718,28 @@
       <c r="K10" s="1"/>
       <c r="L10" s="1"/>
       <c r="M10" s="1"/>
-      <c r="N10" s="1"/>
-      <c r="O10" s="1"/>
-      <c r="P10" s="1"/>
-      <c r="Q10" s="1"/>
+      <c r="N10" s="4"/>
+      <c r="O10" s="4"/>
+      <c r="P10" s="4"/>
+      <c r="Q10" s="4"/>
       <c r="R10" s="4"/>
       <c r="S10" s="4"/>
       <c r="T10" s="4"/>
       <c r="U10" s="4"/>
-      <c r="V10" s="4"/>
-      <c r="W10" s="4"/>
-      <c r="X10" s="4"/>
-      <c r="Y10" s="4"/>
     </row>
     <row r="11" ht="15.75" customHeight="1">
       <c r="A11" s="1" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
       <c r="D11" s="1"/>
       <c r="E11" s="3" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="F11" s="3"/>
       <c r="G11" s="3" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="H11" s="1"/>
       <c r="I11" s="1"/>
@@ -809,35 +747,31 @@
       <c r="K11" s="1"/>
       <c r="L11" s="1"/>
       <c r="M11" s="1"/>
-      <c r="N11" s="1"/>
-      <c r="O11" s="1"/>
-      <c r="P11" s="1"/>
-      <c r="Q11" s="1"/>
+      <c r="N11" s="4"/>
+      <c r="O11" s="4"/>
+      <c r="P11" s="4"/>
+      <c r="Q11" s="4"/>
       <c r="R11" s="4"/>
       <c r="S11" s="4"/>
       <c r="T11" s="4"/>
       <c r="U11" s="4"/>
-      <c r="V11" s="4"/>
-      <c r="W11" s="4"/>
-      <c r="X11" s="4"/>
-      <c r="Y11" s="4"/>
     </row>
     <row r="12" ht="15.75" customHeight="1">
       <c r="A12" s="1" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="D12" s="1"/>
       <c r="E12" s="3" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="G12" s="3"/>
       <c r="H12" s="1"/>
@@ -846,36 +780,32 @@
       <c r="K12" s="1"/>
       <c r="L12" s="1"/>
       <c r="M12" s="1"/>
-      <c r="N12" s="1"/>
-      <c r="O12" s="1"/>
-      <c r="P12" s="1"/>
-      <c r="Q12" s="1"/>
+      <c r="N12" s="4"/>
+      <c r="O12" s="4"/>
+      <c r="P12" s="4"/>
+      <c r="Q12" s="4"/>
       <c r="R12" s="4"/>
       <c r="S12" s="4"/>
       <c r="T12" s="4"/>
       <c r="U12" s="4"/>
-      <c r="V12" s="4"/>
-      <c r="W12" s="4"/>
-      <c r="X12" s="4"/>
-      <c r="Y12" s="4"/>
     </row>
     <row r="13" ht="15.75" customHeight="1">
       <c r="A13" s="1" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="D13" s="1"/>
       <c r="E13" s="3" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="F13" s="1"/>
       <c r="G13" s="3" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="H13" s="1"/>
       <c r="I13" s="1"/>
@@ -883,32 +813,28 @@
       <c r="K13" s="1"/>
       <c r="L13" s="1"/>
       <c r="M13" s="1"/>
-      <c r="N13" s="1"/>
-      <c r="O13" s="1"/>
-      <c r="P13" s="1"/>
-      <c r="Q13" s="1"/>
+      <c r="N13" s="4"/>
+      <c r="O13" s="4"/>
+      <c r="P13" s="4"/>
+      <c r="Q13" s="4"/>
       <c r="R13" s="4"/>
       <c r="S13" s="4"/>
       <c r="T13" s="4"/>
       <c r="U13" s="4"/>
-      <c r="V13" s="4"/>
-      <c r="W13" s="4"/>
-      <c r="X13" s="4"/>
-      <c r="Y13" s="4"/>
     </row>
     <row r="14" ht="15.75" customHeight="1">
       <c r="A14" s="1" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
       <c r="D14" s="1"/>
       <c r="E14" s="3" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="F14" s="1"/>
       <c r="G14" s="3" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="H14" s="1"/>
       <c r="I14" s="1"/>
@@ -916,31 +842,27 @@
       <c r="K14" s="1"/>
       <c r="L14" s="1"/>
       <c r="M14" s="1"/>
-      <c r="N14" s="1"/>
-      <c r="O14" s="1"/>
-      <c r="P14" s="1"/>
-      <c r="Q14" s="1"/>
+      <c r="N14" s="4"/>
+      <c r="O14" s="4"/>
+      <c r="P14" s="4"/>
+      <c r="Q14" s="4"/>
       <c r="R14" s="4"/>
       <c r="S14" s="4"/>
       <c r="T14" s="4"/>
       <c r="U14" s="4"/>
-      <c r="V14" s="4"/>
-      <c r="W14" s="4"/>
-      <c r="X14" s="4"/>
-      <c r="Y14" s="4"/>
     </row>
     <row r="15" ht="15.75" customHeight="1">
       <c r="A15" s="1" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
       <c r="D15" s="1"/>
       <c r="E15" s="3" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="G15" s="1"/>
       <c r="H15" s="1"/>
@@ -949,27 +871,29 @@
       <c r="K15" s="1"/>
       <c r="L15" s="1"/>
       <c r="M15" s="1"/>
-      <c r="N15" s="1"/>
-      <c r="O15" s="1"/>
-      <c r="P15" s="1"/>
-      <c r="Q15" s="1"/>
+      <c r="N15" s="4"/>
+      <c r="O15" s="4"/>
+      <c r="P15" s="4"/>
+      <c r="Q15" s="4"/>
       <c r="R15" s="4"/>
       <c r="S15" s="4"/>
       <c r="T15" s="4"/>
       <c r="U15" s="4"/>
-      <c r="V15" s="4"/>
-      <c r="W15" s="4"/>
-      <c r="X15" s="4"/>
-      <c r="Y15" s="4"/>
     </row>
     <row r="16" ht="15.75" customHeight="1">
       <c r="A16" s="1" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
-      <c r="B16" s="1"/>
-      <c r="C16" s="1"/>
+      <c r="B16" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>14</v>
+      </c>
       <c r="D16" s="1"/>
-      <c r="E16" s="1"/>
+      <c r="E16" s="3" t="s">
+        <v>26</v>
+      </c>
       <c r="F16" s="1"/>
       <c r="G16" s="1"/>
       <c r="H16" s="1"/>
@@ -978,22 +902,18 @@
       <c r="K16" s="1"/>
       <c r="L16" s="1"/>
       <c r="M16" s="1"/>
-      <c r="N16" s="1"/>
-      <c r="O16" s="1"/>
-      <c r="P16" s="1"/>
-      <c r="Q16" s="1"/>
+      <c r="N16" s="4"/>
+      <c r="O16" s="4"/>
+      <c r="P16" s="4"/>
+      <c r="Q16" s="4"/>
       <c r="R16" s="4"/>
       <c r="S16" s="4"/>
       <c r="T16" s="4"/>
       <c r="U16" s="4"/>
-      <c r="V16" s="4"/>
-      <c r="W16" s="4"/>
-      <c r="X16" s="4"/>
-      <c r="Y16" s="4"/>
     </row>
     <row r="17" ht="15.75" customHeight="1">
       <c r="A17" s="1" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B17" s="1"/>
       <c r="C17" s="1"/>
@@ -1007,22 +927,18 @@
       <c r="K17" s="1"/>
       <c r="L17" s="1"/>
       <c r="M17" s="1"/>
-      <c r="N17" s="1"/>
-      <c r="O17" s="1"/>
-      <c r="P17" s="1"/>
-      <c r="Q17" s="1"/>
+      <c r="N17" s="4"/>
+      <c r="O17" s="4"/>
+      <c r="P17" s="4"/>
+      <c r="Q17" s="4"/>
       <c r="R17" s="4"/>
       <c r="S17" s="4"/>
       <c r="T17" s="4"/>
       <c r="U17" s="4"/>
-      <c r="V17" s="4"/>
-      <c r="W17" s="4"/>
-      <c r="X17" s="4"/>
-      <c r="Y17" s="4"/>
     </row>
     <row r="18" ht="15.75" customHeight="1">
       <c r="A18" s="1" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="B18" s="1"/>
       <c r="C18" s="1"/>
@@ -1036,22 +952,18 @@
       <c r="K18" s="1"/>
       <c r="L18" s="1"/>
       <c r="M18" s="1"/>
-      <c r="N18" s="1"/>
-      <c r="O18" s="1"/>
-      <c r="P18" s="1"/>
-      <c r="Q18" s="1"/>
+      <c r="N18" s="4"/>
+      <c r="O18" s="4"/>
+      <c r="P18" s="4"/>
+      <c r="Q18" s="4"/>
       <c r="R18" s="4"/>
       <c r="S18" s="4"/>
       <c r="T18" s="4"/>
       <c r="U18" s="4"/>
-      <c r="V18" s="4"/>
-      <c r="W18" s="4"/>
-      <c r="X18" s="4"/>
-      <c r="Y18" s="4"/>
     </row>
     <row r="19" ht="15.75" customHeight="1">
       <c r="A19" s="1" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="B19" s="1"/>
       <c r="C19" s="1"/>
@@ -1065,22 +977,18 @@
       <c r="K19" s="1"/>
       <c r="L19" s="1"/>
       <c r="M19" s="1"/>
-      <c r="N19" s="1"/>
-      <c r="O19" s="1"/>
-      <c r="P19" s="1"/>
-      <c r="Q19" s="1"/>
+      <c r="N19" s="4"/>
+      <c r="O19" s="4"/>
+      <c r="P19" s="4"/>
+      <c r="Q19" s="4"/>
       <c r="R19" s="4"/>
       <c r="S19" s="4"/>
       <c r="T19" s="4"/>
       <c r="U19" s="4"/>
-      <c r="V19" s="4"/>
-      <c r="W19" s="4"/>
-      <c r="X19" s="4"/>
-      <c r="Y19" s="4"/>
     </row>
     <row r="20" ht="15.75" customHeight="1">
       <c r="A20" s="1" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="B20" s="1"/>
       <c r="C20" s="1"/>
@@ -1094,18 +1002,14 @@
       <c r="K20" s="1"/>
       <c r="L20" s="1"/>
       <c r="M20" s="1"/>
-      <c r="N20" s="1"/>
-      <c r="O20" s="1"/>
-      <c r="P20" s="1"/>
-      <c r="Q20" s="1"/>
+      <c r="N20" s="4"/>
+      <c r="O20" s="4"/>
+      <c r="P20" s="4"/>
+      <c r="Q20" s="4"/>
       <c r="R20" s="4"/>
       <c r="S20" s="4"/>
       <c r="T20" s="4"/>
       <c r="U20" s="4"/>
-      <c r="V20" s="4"/>
-      <c r="W20" s="4"/>
-      <c r="X20" s="4"/>
-      <c r="Y20" s="4"/>
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="4"/>
@@ -1129,10 +1033,6 @@
       <c r="S21" s="4"/>
       <c r="T21" s="4"/>
       <c r="U21" s="4"/>
-      <c r="V21" s="4"/>
-      <c r="W21" s="4"/>
-      <c r="X21" s="4"/>
-      <c r="Y21" s="4"/>
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="4"/>
@@ -1156,10 +1056,6 @@
       <c r="S22" s="4"/>
       <c r="T22" s="4"/>
       <c r="U22" s="4"/>
-      <c r="V22" s="4"/>
-      <c r="W22" s="4"/>
-      <c r="X22" s="4"/>
-      <c r="Y22" s="4"/>
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="4"/>
@@ -1183,10 +1079,6 @@
       <c r="S23" s="4"/>
       <c r="T23" s="4"/>
       <c r="U23" s="4"/>
-      <c r="V23" s="4"/>
-      <c r="W23" s="4"/>
-      <c r="X23" s="4"/>
-      <c r="Y23" s="4"/>
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="4"/>
@@ -1210,10 +1102,6 @@
       <c r="S24" s="4"/>
       <c r="T24" s="4"/>
       <c r="U24" s="4"/>
-      <c r="V24" s="4"/>
-      <c r="W24" s="4"/>
-      <c r="X24" s="4"/>
-      <c r="Y24" s="4"/>
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="4"/>
@@ -1237,10 +1125,6 @@
       <c r="S25" s="4"/>
       <c r="T25" s="4"/>
       <c r="U25" s="4"/>
-      <c r="V25" s="4"/>
-      <c r="W25" s="4"/>
-      <c r="X25" s="4"/>
-      <c r="Y25" s="4"/>
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="4"/>
@@ -1264,10 +1148,6 @@
       <c r="S26" s="4"/>
       <c r="T26" s="4"/>
       <c r="U26" s="4"/>
-      <c r="V26" s="4"/>
-      <c r="W26" s="4"/>
-      <c r="X26" s="4"/>
-      <c r="Y26" s="4"/>
     </row>
     <row r="27" ht="15.75" customHeight="1">
       <c r="A27" s="4"/>
@@ -1291,10 +1171,6 @@
       <c r="S27" s="4"/>
       <c r="T27" s="4"/>
       <c r="U27" s="4"/>
-      <c r="V27" s="4"/>
-      <c r="W27" s="4"/>
-      <c r="X27" s="4"/>
-      <c r="Y27" s="4"/>
     </row>
     <row r="28" ht="15.75" customHeight="1">
       <c r="A28" s="4"/>
@@ -1318,10 +1194,6 @@
       <c r="S28" s="4"/>
       <c r="T28" s="4"/>
       <c r="U28" s="4"/>
-      <c r="V28" s="4"/>
-      <c r="W28" s="4"/>
-      <c r="X28" s="4"/>
-      <c r="Y28" s="4"/>
     </row>
     <row r="29" ht="15.75" customHeight="1">
       <c r="A29" s="4"/>
@@ -1345,10 +1217,6 @@
       <c r="S29" s="4"/>
       <c r="T29" s="4"/>
       <c r="U29" s="4"/>
-      <c r="V29" s="4"/>
-      <c r="W29" s="4"/>
-      <c r="X29" s="4"/>
-      <c r="Y29" s="4"/>
     </row>
     <row r="30" ht="15.75" customHeight="1">
       <c r="A30" s="4"/>
@@ -1372,10 +1240,6 @@
       <c r="S30" s="4"/>
       <c r="T30" s="4"/>
       <c r="U30" s="4"/>
-      <c r="V30" s="4"/>
-      <c r="W30" s="4"/>
-      <c r="X30" s="4"/>
-      <c r="Y30" s="4"/>
     </row>
     <row r="31" ht="15.75" customHeight="1">
       <c r="A31" s="4"/>
@@ -1399,10 +1263,6 @@
       <c r="S31" s="4"/>
       <c r="T31" s="4"/>
       <c r="U31" s="4"/>
-      <c r="V31" s="4"/>
-      <c r="W31" s="4"/>
-      <c r="X31" s="4"/>
-      <c r="Y31" s="4"/>
     </row>
     <row r="32" ht="15.75" customHeight="1">
       <c r="A32" s="4"/>
@@ -1426,10 +1286,6 @@
       <c r="S32" s="4"/>
       <c r="T32" s="4"/>
       <c r="U32" s="4"/>
-      <c r="V32" s="4"/>
-      <c r="W32" s="4"/>
-      <c r="X32" s="4"/>
-      <c r="Y32" s="4"/>
     </row>
     <row r="33" ht="15.75" customHeight="1">
       <c r="A33" s="4"/>
@@ -1453,10 +1309,6 @@
       <c r="S33" s="4"/>
       <c r="T33" s="4"/>
       <c r="U33" s="4"/>
-      <c r="V33" s="4"/>
-      <c r="W33" s="4"/>
-      <c r="X33" s="4"/>
-      <c r="Y33" s="4"/>
     </row>
     <row r="34" ht="15.75" customHeight="1">
       <c r="A34" s="4"/>
@@ -1480,10 +1332,6 @@
       <c r="S34" s="4"/>
       <c r="T34" s="4"/>
       <c r="U34" s="4"/>
-      <c r="V34" s="4"/>
-      <c r="W34" s="4"/>
-      <c r="X34" s="4"/>
-      <c r="Y34" s="4"/>
     </row>
     <row r="35" ht="15.75" customHeight="1">
       <c r="A35" s="4"/>
@@ -1507,10 +1355,6 @@
       <c r="S35" s="4"/>
       <c r="T35" s="4"/>
       <c r="U35" s="4"/>
-      <c r="V35" s="4"/>
-      <c r="W35" s="4"/>
-      <c r="X35" s="4"/>
-      <c r="Y35" s="4"/>
     </row>
     <row r="36" ht="15.75" customHeight="1">
       <c r="A36" s="4"/>
@@ -1534,10 +1378,6 @@
       <c r="S36" s="4"/>
       <c r="T36" s="4"/>
       <c r="U36" s="4"/>
-      <c r="V36" s="4"/>
-      <c r="W36" s="4"/>
-      <c r="X36" s="4"/>
-      <c r="Y36" s="4"/>
     </row>
     <row r="37" ht="15.75" customHeight="1">
       <c r="A37" s="4"/>
@@ -1561,10 +1401,6 @@
       <c r="S37" s="4"/>
       <c r="T37" s="4"/>
       <c r="U37" s="4"/>
-      <c r="V37" s="4"/>
-      <c r="W37" s="4"/>
-      <c r="X37" s="4"/>
-      <c r="Y37" s="4"/>
     </row>
     <row r="38" ht="15.75" customHeight="1">
       <c r="A38" s="4"/>
@@ -1588,10 +1424,6 @@
       <c r="S38" s="4"/>
       <c r="T38" s="4"/>
       <c r="U38" s="4"/>
-      <c r="V38" s="4"/>
-      <c r="W38" s="4"/>
-      <c r="X38" s="4"/>
-      <c r="Y38" s="4"/>
     </row>
     <row r="39" ht="15.75" customHeight="1">
       <c r="A39" s="4"/>
@@ -1615,10 +1447,6 @@
       <c r="S39" s="4"/>
       <c r="T39" s="4"/>
       <c r="U39" s="4"/>
-      <c r="V39" s="4"/>
-      <c r="W39" s="4"/>
-      <c r="X39" s="4"/>
-      <c r="Y39" s="4"/>
     </row>
     <row r="40" ht="15.75" customHeight="1">
       <c r="A40" s="4"/>
@@ -1642,10 +1470,6 @@
       <c r="S40" s="4"/>
       <c r="T40" s="4"/>
       <c r="U40" s="4"/>
-      <c r="V40" s="4"/>
-      <c r="W40" s="4"/>
-      <c r="X40" s="4"/>
-      <c r="Y40" s="4"/>
     </row>
     <row r="41" ht="15.75" customHeight="1">
       <c r="A41" s="4"/>
@@ -1669,10 +1493,6 @@
       <c r="S41" s="4"/>
       <c r="T41" s="4"/>
       <c r="U41" s="4"/>
-      <c r="V41" s="4"/>
-      <c r="W41" s="4"/>
-      <c r="X41" s="4"/>
-      <c r="Y41" s="4"/>
     </row>
     <row r="42" ht="15.75" customHeight="1">
       <c r="A42" s="4"/>
@@ -1696,10 +1516,6 @@
       <c r="S42" s="4"/>
       <c r="T42" s="4"/>
       <c r="U42" s="4"/>
-      <c r="V42" s="4"/>
-      <c r="W42" s="4"/>
-      <c r="X42" s="4"/>
-      <c r="Y42" s="4"/>
     </row>
     <row r="43" ht="15.75" customHeight="1">
       <c r="A43" s="4"/>
@@ -1723,10 +1539,6 @@
       <c r="S43" s="4"/>
       <c r="T43" s="4"/>
       <c r="U43" s="4"/>
-      <c r="V43" s="4"/>
-      <c r="W43" s="4"/>
-      <c r="X43" s="4"/>
-      <c r="Y43" s="4"/>
     </row>
     <row r="44" ht="15.75" customHeight="1">
       <c r="A44" s="4"/>
@@ -1750,10 +1562,6 @@
       <c r="S44" s="4"/>
       <c r="T44" s="4"/>
       <c r="U44" s="4"/>
-      <c r="V44" s="4"/>
-      <c r="W44" s="4"/>
-      <c r="X44" s="4"/>
-      <c r="Y44" s="4"/>
     </row>
     <row r="45" ht="15.75" customHeight="1">
       <c r="A45" s="4"/>
@@ -1777,10 +1585,6 @@
       <c r="S45" s="4"/>
       <c r="T45" s="4"/>
       <c r="U45" s="4"/>
-      <c r="V45" s="4"/>
-      <c r="W45" s="4"/>
-      <c r="X45" s="4"/>
-      <c r="Y45" s="4"/>
     </row>
     <row r="46" ht="15.75" customHeight="1">
       <c r="A46" s="4"/>
@@ -1804,10 +1608,6 @@
       <c r="S46" s="4"/>
       <c r="T46" s="4"/>
       <c r="U46" s="4"/>
-      <c r="V46" s="4"/>
-      <c r="W46" s="4"/>
-      <c r="X46" s="4"/>
-      <c r="Y46" s="4"/>
     </row>
     <row r="47" ht="15.75" customHeight="1">
       <c r="A47" s="4"/>
@@ -1831,10 +1631,6 @@
       <c r="S47" s="4"/>
       <c r="T47" s="4"/>
       <c r="U47" s="4"/>
-      <c r="V47" s="4"/>
-      <c r="W47" s="4"/>
-      <c r="X47" s="4"/>
-      <c r="Y47" s="4"/>
     </row>
     <row r="48" ht="15.75" customHeight="1">
       <c r="A48" s="4"/>
@@ -1858,10 +1654,6 @@
       <c r="S48" s="4"/>
       <c r="T48" s="4"/>
       <c r="U48" s="4"/>
-      <c r="V48" s="4"/>
-      <c r="W48" s="4"/>
-      <c r="X48" s="4"/>
-      <c r="Y48" s="4"/>
     </row>
     <row r="49" ht="15.75" customHeight="1">
       <c r="A49" s="4"/>
@@ -1885,10 +1677,6 @@
       <c r="S49" s="4"/>
       <c r="T49" s="4"/>
       <c r="U49" s="4"/>
-      <c r="V49" s="4"/>
-      <c r="W49" s="4"/>
-      <c r="X49" s="4"/>
-      <c r="Y49" s="4"/>
     </row>
     <row r="50" ht="15.75" customHeight="1">
       <c r="A50" s="4"/>
@@ -1912,10 +1700,6 @@
       <c r="S50" s="4"/>
       <c r="T50" s="4"/>
       <c r="U50" s="4"/>
-      <c r="V50" s="4"/>
-      <c r="W50" s="4"/>
-      <c r="X50" s="4"/>
-      <c r="Y50" s="4"/>
     </row>
     <row r="51" ht="15.75" customHeight="1">
       <c r="A51" s="4"/>
@@ -1939,10 +1723,6 @@
       <c r="S51" s="4"/>
       <c r="T51" s="4"/>
       <c r="U51" s="4"/>
-      <c r="V51" s="4"/>
-      <c r="W51" s="4"/>
-      <c r="X51" s="4"/>
-      <c r="Y51" s="4"/>
     </row>
     <row r="52" ht="15.75" customHeight="1">
       <c r="A52" s="4"/>
@@ -1966,10 +1746,6 @@
       <c r="S52" s="4"/>
       <c r="T52" s="4"/>
       <c r="U52" s="4"/>
-      <c r="V52" s="4"/>
-      <c r="W52" s="4"/>
-      <c r="X52" s="4"/>
-      <c r="Y52" s="4"/>
     </row>
     <row r="53" ht="15.75" customHeight="1">
       <c r="A53" s="4"/>
@@ -1993,10 +1769,6 @@
       <c r="S53" s="4"/>
       <c r="T53" s="4"/>
       <c r="U53" s="4"/>
-      <c r="V53" s="4"/>
-      <c r="W53" s="4"/>
-      <c r="X53" s="4"/>
-      <c r="Y53" s="4"/>
     </row>
     <row r="54" ht="15.75" customHeight="1">
       <c r="A54" s="4"/>
@@ -2020,10 +1792,6 @@
       <c r="S54" s="4"/>
       <c r="T54" s="4"/>
       <c r="U54" s="4"/>
-      <c r="V54" s="4"/>
-      <c r="W54" s="4"/>
-      <c r="X54" s="4"/>
-      <c r="Y54" s="4"/>
     </row>
     <row r="55" ht="15.75" customHeight="1">
       <c r="A55" s="4"/>
@@ -2047,10 +1815,6 @@
       <c r="S55" s="4"/>
       <c r="T55" s="4"/>
       <c r="U55" s="4"/>
-      <c r="V55" s="4"/>
-      <c r="W55" s="4"/>
-      <c r="X55" s="4"/>
-      <c r="Y55" s="4"/>
     </row>
     <row r="56" ht="15.75" customHeight="1">
       <c r="A56" s="4"/>
@@ -2074,10 +1838,6 @@
       <c r="S56" s="4"/>
       <c r="T56" s="4"/>
       <c r="U56" s="4"/>
-      <c r="V56" s="4"/>
-      <c r="W56" s="4"/>
-      <c r="X56" s="4"/>
-      <c r="Y56" s="4"/>
     </row>
     <row r="57" ht="15.75" customHeight="1">
       <c r="A57" s="4"/>
@@ -2101,10 +1861,6 @@
       <c r="S57" s="4"/>
       <c r="T57" s="4"/>
       <c r="U57" s="4"/>
-      <c r="V57" s="4"/>
-      <c r="W57" s="4"/>
-      <c r="X57" s="4"/>
-      <c r="Y57" s="4"/>
     </row>
     <row r="58" ht="15.75" customHeight="1">
       <c r="A58" s="4"/>
@@ -2128,10 +1884,6 @@
       <c r="S58" s="4"/>
       <c r="T58" s="4"/>
       <c r="U58" s="4"/>
-      <c r="V58" s="4"/>
-      <c r="W58" s="4"/>
-      <c r="X58" s="4"/>
-      <c r="Y58" s="4"/>
     </row>
     <row r="59" ht="15.75" customHeight="1">
       <c r="A59" s="4"/>
@@ -2155,10 +1907,6 @@
       <c r="S59" s="4"/>
       <c r="T59" s="4"/>
       <c r="U59" s="4"/>
-      <c r="V59" s="4"/>
-      <c r="W59" s="4"/>
-      <c r="X59" s="4"/>
-      <c r="Y59" s="4"/>
     </row>
     <row r="60" ht="15.75" customHeight="1">
       <c r="A60" s="4"/>
@@ -2182,10 +1930,6 @@
       <c r="S60" s="4"/>
       <c r="T60" s="4"/>
       <c r="U60" s="4"/>
-      <c r="V60" s="4"/>
-      <c r="W60" s="4"/>
-      <c r="X60" s="4"/>
-      <c r="Y60" s="4"/>
     </row>
     <row r="61" ht="15.75" customHeight="1">
       <c r="A61" s="4"/>
@@ -2209,10 +1953,6 @@
       <c r="S61" s="4"/>
       <c r="T61" s="4"/>
       <c r="U61" s="4"/>
-      <c r="V61" s="4"/>
-      <c r="W61" s="4"/>
-      <c r="X61" s="4"/>
-      <c r="Y61" s="4"/>
     </row>
     <row r="62" ht="15.75" customHeight="1">
       <c r="A62" s="4"/>
@@ -2236,10 +1976,6 @@
       <c r="S62" s="4"/>
       <c r="T62" s="4"/>
       <c r="U62" s="4"/>
-      <c r="V62" s="4"/>
-      <c r="W62" s="4"/>
-      <c r="X62" s="4"/>
-      <c r="Y62" s="4"/>
     </row>
     <row r="63" ht="15.75" customHeight="1">
       <c r="A63" s="4"/>
@@ -2263,10 +1999,6 @@
       <c r="S63" s="4"/>
       <c r="T63" s="4"/>
       <c r="U63" s="4"/>
-      <c r="V63" s="4"/>
-      <c r="W63" s="4"/>
-      <c r="X63" s="4"/>
-      <c r="Y63" s="4"/>
     </row>
     <row r="64" ht="15.75" customHeight="1">
       <c r="A64" s="4"/>
@@ -2290,10 +2022,6 @@
       <c r="S64" s="4"/>
       <c r="T64" s="4"/>
       <c r="U64" s="4"/>
-      <c r="V64" s="4"/>
-      <c r="W64" s="4"/>
-      <c r="X64" s="4"/>
-      <c r="Y64" s="4"/>
     </row>
     <row r="65" ht="15.75" customHeight="1">
       <c r="A65" s="4"/>
@@ -2317,10 +2045,6 @@
       <c r="S65" s="4"/>
       <c r="T65" s="4"/>
       <c r="U65" s="4"/>
-      <c r="V65" s="4"/>
-      <c r="W65" s="4"/>
-      <c r="X65" s="4"/>
-      <c r="Y65" s="4"/>
     </row>
     <row r="66" ht="15.75" customHeight="1">
       <c r="A66" s="4"/>
@@ -2344,10 +2068,6 @@
       <c r="S66" s="4"/>
       <c r="T66" s="4"/>
       <c r="U66" s="4"/>
-      <c r="V66" s="4"/>
-      <c r="W66" s="4"/>
-      <c r="X66" s="4"/>
-      <c r="Y66" s="4"/>
     </row>
     <row r="67" ht="15.75" customHeight="1">
       <c r="A67" s="4"/>
@@ -2371,10 +2091,6 @@
       <c r="S67" s="4"/>
       <c r="T67" s="4"/>
       <c r="U67" s="4"/>
-      <c r="V67" s="4"/>
-      <c r="W67" s="4"/>
-      <c r="X67" s="4"/>
-      <c r="Y67" s="4"/>
     </row>
     <row r="68" ht="15.75" customHeight="1">
       <c r="A68" s="4"/>
@@ -2398,10 +2114,6 @@
       <c r="S68" s="4"/>
       <c r="T68" s="4"/>
       <c r="U68" s="4"/>
-      <c r="V68" s="4"/>
-      <c r="W68" s="4"/>
-      <c r="X68" s="4"/>
-      <c r="Y68" s="4"/>
     </row>
     <row r="69" ht="15.75" customHeight="1">
       <c r="A69" s="4"/>
@@ -2425,10 +2137,6 @@
       <c r="S69" s="4"/>
       <c r="T69" s="4"/>
       <c r="U69" s="4"/>
-      <c r="V69" s="4"/>
-      <c r="W69" s="4"/>
-      <c r="X69" s="4"/>
-      <c r="Y69" s="4"/>
     </row>
     <row r="70" ht="15.75" customHeight="1">
       <c r="A70" s="4"/>
@@ -2452,10 +2160,6 @@
       <c r="S70" s="4"/>
       <c r="T70" s="4"/>
       <c r="U70" s="4"/>
-      <c r="V70" s="4"/>
-      <c r="W70" s="4"/>
-      <c r="X70" s="4"/>
-      <c r="Y70" s="4"/>
     </row>
     <row r="71" ht="15.75" customHeight="1">
       <c r="A71" s="4"/>
@@ -2479,10 +2183,6 @@
       <c r="S71" s="4"/>
       <c r="T71" s="4"/>
       <c r="U71" s="4"/>
-      <c r="V71" s="4"/>
-      <c r="W71" s="4"/>
-      <c r="X71" s="4"/>
-      <c r="Y71" s="4"/>
     </row>
     <row r="72" ht="15.75" customHeight="1">
       <c r="A72" s="4"/>
@@ -2506,10 +2206,6 @@
       <c r="S72" s="4"/>
       <c r="T72" s="4"/>
       <c r="U72" s="4"/>
-      <c r="V72" s="4"/>
-      <c r="W72" s="4"/>
-      <c r="X72" s="4"/>
-      <c r="Y72" s="4"/>
     </row>
     <row r="73" ht="15.75" customHeight="1">
       <c r="A73" s="4"/>
@@ -2533,10 +2229,6 @@
       <c r="S73" s="4"/>
       <c r="T73" s="4"/>
       <c r="U73" s="4"/>
-      <c r="V73" s="4"/>
-      <c r="W73" s="4"/>
-      <c r="X73" s="4"/>
-      <c r="Y73" s="4"/>
     </row>
     <row r="74" ht="15.75" customHeight="1">
       <c r="A74" s="4"/>
@@ -2560,10 +2252,6 @@
       <c r="S74" s="4"/>
       <c r="T74" s="4"/>
       <c r="U74" s="4"/>
-      <c r="V74" s="4"/>
-      <c r="W74" s="4"/>
-      <c r="X74" s="4"/>
-      <c r="Y74" s="4"/>
     </row>
     <row r="75" ht="15.75" customHeight="1">
       <c r="A75" s="4"/>
@@ -2587,10 +2275,6 @@
       <c r="S75" s="4"/>
       <c r="T75" s="4"/>
       <c r="U75" s="4"/>
-      <c r="V75" s="4"/>
-      <c r="W75" s="4"/>
-      <c r="X75" s="4"/>
-      <c r="Y75" s="4"/>
     </row>
     <row r="76" ht="15.75" customHeight="1">
       <c r="A76" s="4"/>
@@ -2614,10 +2298,6 @@
       <c r="S76" s="4"/>
       <c r="T76" s="4"/>
       <c r="U76" s="4"/>
-      <c r="V76" s="4"/>
-      <c r="W76" s="4"/>
-      <c r="X76" s="4"/>
-      <c r="Y76" s="4"/>
     </row>
     <row r="77" ht="15.75" customHeight="1">
       <c r="A77" s="4"/>
@@ -2641,10 +2321,6 @@
       <c r="S77" s="4"/>
       <c r="T77" s="4"/>
       <c r="U77" s="4"/>
-      <c r="V77" s="4"/>
-      <c r="W77" s="4"/>
-      <c r="X77" s="4"/>
-      <c r="Y77" s="4"/>
     </row>
     <row r="78" ht="15.75" customHeight="1">
       <c r="A78" s="4"/>
@@ -2668,10 +2344,6 @@
       <c r="S78" s="4"/>
       <c r="T78" s="4"/>
       <c r="U78" s="4"/>
-      <c r="V78" s="4"/>
-      <c r="W78" s="4"/>
-      <c r="X78" s="4"/>
-      <c r="Y78" s="4"/>
     </row>
     <row r="79" ht="15.75" customHeight="1">
       <c r="A79" s="4"/>
@@ -2695,10 +2367,6 @@
       <c r="S79" s="4"/>
       <c r="T79" s="4"/>
       <c r="U79" s="4"/>
-      <c r="V79" s="4"/>
-      <c r="W79" s="4"/>
-      <c r="X79" s="4"/>
-      <c r="Y79" s="4"/>
     </row>
     <row r="80" ht="15.75" customHeight="1">
       <c r="A80" s="4"/>
@@ -2722,10 +2390,6 @@
       <c r="S80" s="4"/>
       <c r="T80" s="4"/>
       <c r="U80" s="4"/>
-      <c r="V80" s="4"/>
-      <c r="W80" s="4"/>
-      <c r="X80" s="4"/>
-      <c r="Y80" s="4"/>
     </row>
     <row r="81" ht="15.75" customHeight="1">
       <c r="A81" s="4"/>
@@ -2749,10 +2413,6 @@
       <c r="S81" s="4"/>
       <c r="T81" s="4"/>
       <c r="U81" s="4"/>
-      <c r="V81" s="4"/>
-      <c r="W81" s="4"/>
-      <c r="X81" s="4"/>
-      <c r="Y81" s="4"/>
     </row>
     <row r="82" ht="15.75" customHeight="1">
       <c r="A82" s="4"/>
@@ -2776,10 +2436,6 @@
       <c r="S82" s="4"/>
       <c r="T82" s="4"/>
       <c r="U82" s="4"/>
-      <c r="V82" s="4"/>
-      <c r="W82" s="4"/>
-      <c r="X82" s="4"/>
-      <c r="Y82" s="4"/>
     </row>
     <row r="83" ht="15.75" customHeight="1">
       <c r="A83" s="4"/>
@@ -2803,10 +2459,6 @@
       <c r="S83" s="4"/>
       <c r="T83" s="4"/>
       <c r="U83" s="4"/>
-      <c r="V83" s="4"/>
-      <c r="W83" s="4"/>
-      <c r="X83" s="4"/>
-      <c r="Y83" s="4"/>
     </row>
     <row r="84" ht="15.75" customHeight="1">
       <c r="A84" s="4"/>
@@ -2830,10 +2482,6 @@
       <c r="S84" s="4"/>
       <c r="T84" s="4"/>
       <c r="U84" s="4"/>
-      <c r="V84" s="4"/>
-      <c r="W84" s="4"/>
-      <c r="X84" s="4"/>
-      <c r="Y84" s="4"/>
     </row>
     <row r="85" ht="15.75" customHeight="1">
       <c r="A85" s="4"/>
@@ -2857,10 +2505,6 @@
       <c r="S85" s="4"/>
       <c r="T85" s="4"/>
       <c r="U85" s="4"/>
-      <c r="V85" s="4"/>
-      <c r="W85" s="4"/>
-      <c r="X85" s="4"/>
-      <c r="Y85" s="4"/>
     </row>
     <row r="86" ht="15.75" customHeight="1">
       <c r="A86" s="4"/>
@@ -2884,10 +2528,6 @@
       <c r="S86" s="4"/>
       <c r="T86" s="4"/>
       <c r="U86" s="4"/>
-      <c r="V86" s="4"/>
-      <c r="W86" s="4"/>
-      <c r="X86" s="4"/>
-      <c r="Y86" s="4"/>
     </row>
     <row r="87" ht="15.75" customHeight="1">
       <c r="A87" s="4"/>
@@ -2911,10 +2551,6 @@
       <c r="S87" s="4"/>
       <c r="T87" s="4"/>
       <c r="U87" s="4"/>
-      <c r="V87" s="4"/>
-      <c r="W87" s="4"/>
-      <c r="X87" s="4"/>
-      <c r="Y87" s="4"/>
     </row>
     <row r="88" ht="15.75" customHeight="1">
       <c r="A88" s="4"/>
@@ -2938,10 +2574,6 @@
       <c r="S88" s="4"/>
       <c r="T88" s="4"/>
       <c r="U88" s="4"/>
-      <c r="V88" s="4"/>
-      <c r="W88" s="4"/>
-      <c r="X88" s="4"/>
-      <c r="Y88" s="4"/>
     </row>
     <row r="89" ht="15.75" customHeight="1">
       <c r="A89" s="4"/>
@@ -2965,10 +2597,6 @@
       <c r="S89" s="4"/>
       <c r="T89" s="4"/>
       <c r="U89" s="4"/>
-      <c r="V89" s="4"/>
-      <c r="W89" s="4"/>
-      <c r="X89" s="4"/>
-      <c r="Y89" s="4"/>
     </row>
     <row r="90" ht="15.75" customHeight="1">
       <c r="A90" s="4"/>
@@ -2992,10 +2620,6 @@
       <c r="S90" s="4"/>
       <c r="T90" s="4"/>
       <c r="U90" s="4"/>
-      <c r="V90" s="4"/>
-      <c r="W90" s="4"/>
-      <c r="X90" s="4"/>
-      <c r="Y90" s="4"/>
     </row>
     <row r="91" ht="15.75" customHeight="1">
       <c r="A91" s="4"/>
@@ -3019,10 +2643,6 @@
       <c r="S91" s="4"/>
       <c r="T91" s="4"/>
       <c r="U91" s="4"/>
-      <c r="V91" s="4"/>
-      <c r="W91" s="4"/>
-      <c r="X91" s="4"/>
-      <c r="Y91" s="4"/>
     </row>
     <row r="92" ht="15.75" customHeight="1">
       <c r="A92" s="4"/>
@@ -3046,10 +2666,6 @@
       <c r="S92" s="4"/>
       <c r="T92" s="4"/>
       <c r="U92" s="4"/>
-      <c r="V92" s="4"/>
-      <c r="W92" s="4"/>
-      <c r="X92" s="4"/>
-      <c r="Y92" s="4"/>
     </row>
     <row r="93" ht="15.75" customHeight="1">
       <c r="A93" s="4"/>
@@ -3073,10 +2689,6 @@
       <c r="S93" s="4"/>
       <c r="T93" s="4"/>
       <c r="U93" s="4"/>
-      <c r="V93" s="4"/>
-      <c r="W93" s="4"/>
-      <c r="X93" s="4"/>
-      <c r="Y93" s="4"/>
     </row>
     <row r="94" ht="15.75" customHeight="1">
       <c r="A94" s="4"/>
@@ -3100,10 +2712,6 @@
       <c r="S94" s="4"/>
       <c r="T94" s="4"/>
       <c r="U94" s="4"/>
-      <c r="V94" s="4"/>
-      <c r="W94" s="4"/>
-      <c r="X94" s="4"/>
-      <c r="Y94" s="4"/>
     </row>
     <row r="95" ht="15.75" customHeight="1">
       <c r="A95" s="4"/>
@@ -3127,10 +2735,6 @@
       <c r="S95" s="4"/>
       <c r="T95" s="4"/>
       <c r="U95" s="4"/>
-      <c r="V95" s="4"/>
-      <c r="W95" s="4"/>
-      <c r="X95" s="4"/>
-      <c r="Y95" s="4"/>
     </row>
     <row r="96" ht="15.75" customHeight="1">
       <c r="A96" s="4"/>
@@ -3154,10 +2758,6 @@
       <c r="S96" s="4"/>
       <c r="T96" s="4"/>
       <c r="U96" s="4"/>
-      <c r="V96" s="4"/>
-      <c r="W96" s="4"/>
-      <c r="X96" s="4"/>
-      <c r="Y96" s="4"/>
     </row>
     <row r="97" ht="15.75" customHeight="1">
       <c r="A97" s="4"/>
@@ -3181,10 +2781,6 @@
       <c r="S97" s="4"/>
       <c r="T97" s="4"/>
       <c r="U97" s="4"/>
-      <c r="V97" s="4"/>
-      <c r="W97" s="4"/>
-      <c r="X97" s="4"/>
-      <c r="Y97" s="4"/>
     </row>
     <row r="98" ht="15.75" customHeight="1">
       <c r="A98" s="4"/>
@@ -3208,10 +2804,6 @@
       <c r="S98" s="4"/>
       <c r="T98" s="4"/>
       <c r="U98" s="4"/>
-      <c r="V98" s="4"/>
-      <c r="W98" s="4"/>
-      <c r="X98" s="4"/>
-      <c r="Y98" s="4"/>
     </row>
     <row r="99" ht="15.75" customHeight="1">
       <c r="A99" s="4"/>
@@ -3235,10 +2827,6 @@
       <c r="S99" s="4"/>
       <c r="T99" s="4"/>
       <c r="U99" s="4"/>
-      <c r="V99" s="4"/>
-      <c r="W99" s="4"/>
-      <c r="X99" s="4"/>
-      <c r="Y99" s="4"/>
     </row>
     <row r="100" ht="15.75" customHeight="1">
       <c r="A100" s="4"/>
@@ -3262,10 +2850,6 @@
       <c r="S100" s="4"/>
       <c r="T100" s="4"/>
       <c r="U100" s="4"/>
-      <c r="V100" s="4"/>
-      <c r="W100" s="4"/>
-      <c r="X100" s="4"/>
-      <c r="Y100" s="4"/>
     </row>
     <row r="101" ht="15.75" customHeight="1">
       <c r="A101" s="4"/>
@@ -3289,10 +2873,6 @@
       <c r="S101" s="4"/>
       <c r="T101" s="4"/>
       <c r="U101" s="4"/>
-      <c r="V101" s="4"/>
-      <c r="W101" s="4"/>
-      <c r="X101" s="4"/>
-      <c r="Y101" s="4"/>
     </row>
     <row r="102" ht="15.75" customHeight="1">
       <c r="A102" s="4"/>
@@ -3316,10 +2896,6 @@
       <c r="S102" s="4"/>
       <c r="T102" s="4"/>
       <c r="U102" s="4"/>
-      <c r="V102" s="4"/>
-      <c r="W102" s="4"/>
-      <c r="X102" s="4"/>
-      <c r="Y102" s="4"/>
     </row>
     <row r="103" ht="15.75" customHeight="1">
       <c r="A103" s="4"/>
@@ -3343,10 +2919,6 @@
       <c r="S103" s="4"/>
       <c r="T103" s="4"/>
       <c r="U103" s="4"/>
-      <c r="V103" s="4"/>
-      <c r="W103" s="4"/>
-      <c r="X103" s="4"/>
-      <c r="Y103" s="4"/>
     </row>
     <row r="104" ht="15.75" customHeight="1">
       <c r="A104" s="4"/>
@@ -3370,10 +2942,6 @@
       <c r="S104" s="4"/>
       <c r="T104" s="4"/>
       <c r="U104" s="4"/>
-      <c r="V104" s="4"/>
-      <c r="W104" s="4"/>
-      <c r="X104" s="4"/>
-      <c r="Y104" s="4"/>
     </row>
     <row r="105" ht="15.75" customHeight="1">
       <c r="A105" s="4"/>
@@ -3397,10 +2965,6 @@
       <c r="S105" s="4"/>
       <c r="T105" s="4"/>
       <c r="U105" s="4"/>
-      <c r="V105" s="4"/>
-      <c r="W105" s="4"/>
-      <c r="X105" s="4"/>
-      <c r="Y105" s="4"/>
     </row>
     <row r="106" ht="15.75" customHeight="1">
       <c r="A106" s="4"/>
@@ -3424,10 +2988,6 @@
       <c r="S106" s="4"/>
       <c r="T106" s="4"/>
       <c r="U106" s="4"/>
-      <c r="V106" s="4"/>
-      <c r="W106" s="4"/>
-      <c r="X106" s="4"/>
-      <c r="Y106" s="4"/>
     </row>
     <row r="107" ht="15.75" customHeight="1">
       <c r="A107" s="4"/>
@@ -3451,10 +3011,6 @@
       <c r="S107" s="4"/>
       <c r="T107" s="4"/>
       <c r="U107" s="4"/>
-      <c r="V107" s="4"/>
-      <c r="W107" s="4"/>
-      <c r="X107" s="4"/>
-      <c r="Y107" s="4"/>
     </row>
     <row r="108" ht="15.75" customHeight="1">
       <c r="A108" s="4"/>
@@ -3478,10 +3034,6 @@
       <c r="S108" s="4"/>
       <c r="T108" s="4"/>
       <c r="U108" s="4"/>
-      <c r="V108" s="4"/>
-      <c r="W108" s="4"/>
-      <c r="X108" s="4"/>
-      <c r="Y108" s="4"/>
     </row>
     <row r="109" ht="15.75" customHeight="1">
       <c r="A109" s="4"/>
@@ -3505,10 +3057,6 @@
       <c r="S109" s="4"/>
       <c r="T109" s="4"/>
       <c r="U109" s="4"/>
-      <c r="V109" s="4"/>
-      <c r="W109" s="4"/>
-      <c r="X109" s="4"/>
-      <c r="Y109" s="4"/>
     </row>
     <row r="110" ht="15.75" customHeight="1">
       <c r="A110" s="4"/>
@@ -3532,10 +3080,6 @@
       <c r="S110" s="4"/>
       <c r="T110" s="4"/>
       <c r="U110" s="4"/>
-      <c r="V110" s="4"/>
-      <c r="W110" s="4"/>
-      <c r="X110" s="4"/>
-      <c r="Y110" s="4"/>
     </row>
     <row r="111" ht="15.75" customHeight="1">
       <c r="A111" s="4"/>
@@ -3559,10 +3103,6 @@
       <c r="S111" s="4"/>
       <c r="T111" s="4"/>
       <c r="U111" s="4"/>
-      <c r="V111" s="4"/>
-      <c r="W111" s="4"/>
-      <c r="X111" s="4"/>
-      <c r="Y111" s="4"/>
     </row>
     <row r="112" ht="15.75" customHeight="1">
       <c r="A112" s="4"/>
@@ -3586,10 +3126,6 @@
       <c r="S112" s="4"/>
       <c r="T112" s="4"/>
       <c r="U112" s="4"/>
-      <c r="V112" s="4"/>
-      <c r="W112" s="4"/>
-      <c r="X112" s="4"/>
-      <c r="Y112" s="4"/>
     </row>
     <row r="113" ht="15.75" customHeight="1">
       <c r="A113" s="4"/>
@@ -3613,10 +3149,6 @@
       <c r="S113" s="4"/>
       <c r="T113" s="4"/>
       <c r="U113" s="4"/>
-      <c r="V113" s="4"/>
-      <c r="W113" s="4"/>
-      <c r="X113" s="4"/>
-      <c r="Y113" s="4"/>
     </row>
     <row r="114" ht="15.75" customHeight="1">
       <c r="A114" s="4"/>
@@ -3640,10 +3172,6 @@
       <c r="S114" s="4"/>
       <c r="T114" s="4"/>
       <c r="U114" s="4"/>
-      <c r="V114" s="4"/>
-      <c r="W114" s="4"/>
-      <c r="X114" s="4"/>
-      <c r="Y114" s="4"/>
     </row>
     <row r="115" ht="15.75" customHeight="1">
       <c r="A115" s="4"/>
@@ -3667,10 +3195,6 @@
       <c r="S115" s="4"/>
       <c r="T115" s="4"/>
       <c r="U115" s="4"/>
-      <c r="V115" s="4"/>
-      <c r="W115" s="4"/>
-      <c r="X115" s="4"/>
-      <c r="Y115" s="4"/>
     </row>
     <row r="116" ht="15.75" customHeight="1">
       <c r="A116" s="4"/>
@@ -3694,10 +3218,6 @@
       <c r="S116" s="4"/>
       <c r="T116" s="4"/>
       <c r="U116" s="4"/>
-      <c r="V116" s="4"/>
-      <c r="W116" s="4"/>
-      <c r="X116" s="4"/>
-      <c r="Y116" s="4"/>
     </row>
     <row r="117" ht="15.75" customHeight="1">
       <c r="A117" s="4"/>
@@ -3721,10 +3241,6 @@
       <c r="S117" s="4"/>
       <c r="T117" s="4"/>
       <c r="U117" s="4"/>
-      <c r="V117" s="4"/>
-      <c r="W117" s="4"/>
-      <c r="X117" s="4"/>
-      <c r="Y117" s="4"/>
     </row>
     <row r="118" ht="15.75" customHeight="1">
       <c r="A118" s="4"/>
@@ -3748,10 +3264,6 @@
       <c r="S118" s="4"/>
       <c r="T118" s="4"/>
       <c r="U118" s="4"/>
-      <c r="V118" s="4"/>
-      <c r="W118" s="4"/>
-      <c r="X118" s="4"/>
-      <c r="Y118" s="4"/>
     </row>
     <row r="119" ht="15.75" customHeight="1">
       <c r="A119" s="4"/>
@@ -3775,10 +3287,6 @@
       <c r="S119" s="4"/>
       <c r="T119" s="4"/>
       <c r="U119" s="4"/>
-      <c r="V119" s="4"/>
-      <c r="W119" s="4"/>
-      <c r="X119" s="4"/>
-      <c r="Y119" s="4"/>
     </row>
     <row r="120" ht="15.75" customHeight="1">
       <c r="A120" s="4"/>
@@ -3802,10 +3310,6 @@
       <c r="S120" s="4"/>
       <c r="T120" s="4"/>
       <c r="U120" s="4"/>
-      <c r="V120" s="4"/>
-      <c r="W120" s="4"/>
-      <c r="X120" s="4"/>
-      <c r="Y120" s="4"/>
     </row>
     <row r="121" ht="15.75" customHeight="1">
       <c r="A121" s="4"/>
@@ -3829,10 +3333,6 @@
       <c r="S121" s="4"/>
       <c r="T121" s="4"/>
       <c r="U121" s="4"/>
-      <c r="V121" s="4"/>
-      <c r="W121" s="4"/>
-      <c r="X121" s="4"/>
-      <c r="Y121" s="4"/>
     </row>
     <row r="122" ht="15.75" customHeight="1">
       <c r="A122" s="4"/>
@@ -3856,10 +3356,6 @@
       <c r="S122" s="4"/>
       <c r="T122" s="4"/>
       <c r="U122" s="4"/>
-      <c r="V122" s="4"/>
-      <c r="W122" s="4"/>
-      <c r="X122" s="4"/>
-      <c r="Y122" s="4"/>
     </row>
     <row r="123" ht="15.75" customHeight="1">
       <c r="A123" s="4"/>
@@ -3883,10 +3379,6 @@
       <c r="S123" s="4"/>
       <c r="T123" s="4"/>
       <c r="U123" s="4"/>
-      <c r="V123" s="4"/>
-      <c r="W123" s="4"/>
-      <c r="X123" s="4"/>
-      <c r="Y123" s="4"/>
     </row>
     <row r="124" ht="15.75" customHeight="1">
       <c r="A124" s="4"/>
@@ -3910,10 +3402,6 @@
       <c r="S124" s="4"/>
       <c r="T124" s="4"/>
       <c r="U124" s="4"/>
-      <c r="V124" s="4"/>
-      <c r="W124" s="4"/>
-      <c r="X124" s="4"/>
-      <c r="Y124" s="4"/>
     </row>
     <row r="125" ht="15.75" customHeight="1">
       <c r="A125" s="4"/>
@@ -3937,10 +3425,6 @@
       <c r="S125" s="4"/>
       <c r="T125" s="4"/>
       <c r="U125" s="4"/>
-      <c r="V125" s="4"/>
-      <c r="W125" s="4"/>
-      <c r="X125" s="4"/>
-      <c r="Y125" s="4"/>
     </row>
     <row r="126" ht="15.75" customHeight="1">
       <c r="A126" s="4"/>
@@ -3964,10 +3448,6 @@
       <c r="S126" s="4"/>
       <c r="T126" s="4"/>
       <c r="U126" s="4"/>
-      <c r="V126" s="4"/>
-      <c r="W126" s="4"/>
-      <c r="X126" s="4"/>
-      <c r="Y126" s="4"/>
     </row>
     <row r="127" ht="15.75" customHeight="1">
       <c r="A127" s="4"/>
@@ -3991,10 +3471,6 @@
       <c r="S127" s="4"/>
       <c r="T127" s="4"/>
       <c r="U127" s="4"/>
-      <c r="V127" s="4"/>
-      <c r="W127" s="4"/>
-      <c r="X127" s="4"/>
-      <c r="Y127" s="4"/>
     </row>
     <row r="128" ht="15.75" customHeight="1">
       <c r="A128" s="4"/>
@@ -4018,10 +3494,6 @@
       <c r="S128" s="4"/>
       <c r="T128" s="4"/>
       <c r="U128" s="4"/>
-      <c r="V128" s="4"/>
-      <c r="W128" s="4"/>
-      <c r="X128" s="4"/>
-      <c r="Y128" s="4"/>
     </row>
     <row r="129" ht="15.75" customHeight="1">
       <c r="A129" s="4"/>
@@ -4045,10 +3517,6 @@
       <c r="S129" s="4"/>
       <c r="T129" s="4"/>
       <c r="U129" s="4"/>
-      <c r="V129" s="4"/>
-      <c r="W129" s="4"/>
-      <c r="X129" s="4"/>
-      <c r="Y129" s="4"/>
     </row>
     <row r="130" ht="15.75" customHeight="1">
       <c r="A130" s="4"/>
@@ -4072,10 +3540,6 @@
       <c r="S130" s="4"/>
       <c r="T130" s="4"/>
       <c r="U130" s="4"/>
-      <c r="V130" s="4"/>
-      <c r="W130" s="4"/>
-      <c r="X130" s="4"/>
-      <c r="Y130" s="4"/>
     </row>
     <row r="131" ht="15.75" customHeight="1">
       <c r="A131" s="4"/>
@@ -4099,10 +3563,6 @@
       <c r="S131" s="4"/>
       <c r="T131" s="4"/>
       <c r="U131" s="4"/>
-      <c r="V131" s="4"/>
-      <c r="W131" s="4"/>
-      <c r="X131" s="4"/>
-      <c r="Y131" s="4"/>
     </row>
     <row r="132" ht="15.75" customHeight="1">
       <c r="A132" s="4"/>
@@ -4126,10 +3586,6 @@
       <c r="S132" s="4"/>
       <c r="T132" s="4"/>
       <c r="U132" s="4"/>
-      <c r="V132" s="4"/>
-      <c r="W132" s="4"/>
-      <c r="X132" s="4"/>
-      <c r="Y132" s="4"/>
     </row>
     <row r="133" ht="15.75" customHeight="1">
       <c r="A133" s="4"/>
@@ -4153,10 +3609,6 @@
       <c r="S133" s="4"/>
       <c r="T133" s="4"/>
       <c r="U133" s="4"/>
-      <c r="V133" s="4"/>
-      <c r="W133" s="4"/>
-      <c r="X133" s="4"/>
-      <c r="Y133" s="4"/>
     </row>
     <row r="134" ht="15.75" customHeight="1">
       <c r="A134" s="4"/>
@@ -4180,10 +3632,6 @@
       <c r="S134" s="4"/>
       <c r="T134" s="4"/>
       <c r="U134" s="4"/>
-      <c r="V134" s="4"/>
-      <c r="W134" s="4"/>
-      <c r="X134" s="4"/>
-      <c r="Y134" s="4"/>
     </row>
     <row r="135" ht="15.75" customHeight="1">
       <c r="A135" s="4"/>
@@ -4207,10 +3655,6 @@
       <c r="S135" s="4"/>
       <c r="T135" s="4"/>
       <c r="U135" s="4"/>
-      <c r="V135" s="4"/>
-      <c r="W135" s="4"/>
-      <c r="X135" s="4"/>
-      <c r="Y135" s="4"/>
     </row>
     <row r="136" ht="15.75" customHeight="1">
       <c r="A136" s="4"/>
@@ -4234,10 +3678,6 @@
       <c r="S136" s="4"/>
       <c r="T136" s="4"/>
       <c r="U136" s="4"/>
-      <c r="V136" s="4"/>
-      <c r="W136" s="4"/>
-      <c r="X136" s="4"/>
-      <c r="Y136" s="4"/>
     </row>
     <row r="137" ht="15.75" customHeight="1">
       <c r="A137" s="4"/>
@@ -4261,10 +3701,6 @@
       <c r="S137" s="4"/>
       <c r="T137" s="4"/>
       <c r="U137" s="4"/>
-      <c r="V137" s="4"/>
-      <c r="W137" s="4"/>
-      <c r="X137" s="4"/>
-      <c r="Y137" s="4"/>
     </row>
     <row r="138" ht="15.75" customHeight="1">
       <c r="A138" s="4"/>
@@ -4288,10 +3724,6 @@
       <c r="S138" s="4"/>
       <c r="T138" s="4"/>
       <c r="U138" s="4"/>
-      <c r="V138" s="4"/>
-      <c r="W138" s="4"/>
-      <c r="X138" s="4"/>
-      <c r="Y138" s="4"/>
     </row>
     <row r="139" ht="15.75" customHeight="1">
       <c r="A139" s="4"/>
@@ -4315,10 +3747,6 @@
       <c r="S139" s="4"/>
       <c r="T139" s="4"/>
       <c r="U139" s="4"/>
-      <c r="V139" s="4"/>
-      <c r="W139" s="4"/>
-      <c r="X139" s="4"/>
-      <c r="Y139" s="4"/>
     </row>
     <row r="140" ht="15.75" customHeight="1">
       <c r="A140" s="4"/>
@@ -4342,10 +3770,6 @@
       <c r="S140" s="4"/>
       <c r="T140" s="4"/>
       <c r="U140" s="4"/>
-      <c r="V140" s="4"/>
-      <c r="W140" s="4"/>
-      <c r="X140" s="4"/>
-      <c r="Y140" s="4"/>
     </row>
     <row r="141" ht="15.75" customHeight="1">
       <c r="A141" s="4"/>
@@ -4369,10 +3793,6 @@
       <c r="S141" s="4"/>
       <c r="T141" s="4"/>
       <c r="U141" s="4"/>
-      <c r="V141" s="4"/>
-      <c r="W141" s="4"/>
-      <c r="X141" s="4"/>
-      <c r="Y141" s="4"/>
     </row>
     <row r="142" ht="15.75" customHeight="1">
       <c r="A142" s="4"/>
@@ -4396,10 +3816,6 @@
       <c r="S142" s="4"/>
       <c r="T142" s="4"/>
       <c r="U142" s="4"/>
-      <c r="V142" s="4"/>
-      <c r="W142" s="4"/>
-      <c r="X142" s="4"/>
-      <c r="Y142" s="4"/>
     </row>
     <row r="143" ht="15.75" customHeight="1">
       <c r="A143" s="4"/>
@@ -4423,10 +3839,6 @@
       <c r="S143" s="4"/>
       <c r="T143" s="4"/>
       <c r="U143" s="4"/>
-      <c r="V143" s="4"/>
-      <c r="W143" s="4"/>
-      <c r="X143" s="4"/>
-      <c r="Y143" s="4"/>
     </row>
     <row r="144" ht="15.75" customHeight="1">
       <c r="A144" s="4"/>
@@ -4450,10 +3862,6 @@
       <c r="S144" s="4"/>
       <c r="T144" s="4"/>
       <c r="U144" s="4"/>
-      <c r="V144" s="4"/>
-      <c r="W144" s="4"/>
-      <c r="X144" s="4"/>
-      <c r="Y144" s="4"/>
     </row>
     <row r="145" ht="15.75" customHeight="1">
       <c r="A145" s="4"/>
@@ -4477,10 +3885,6 @@
       <c r="S145" s="4"/>
       <c r="T145" s="4"/>
       <c r="U145" s="4"/>
-      <c r="V145" s="4"/>
-      <c r="W145" s="4"/>
-      <c r="X145" s="4"/>
-      <c r="Y145" s="4"/>
     </row>
     <row r="146" ht="15.75" customHeight="1">
       <c r="A146" s="4"/>
@@ -4504,10 +3908,6 @@
       <c r="S146" s="4"/>
       <c r="T146" s="4"/>
       <c r="U146" s="4"/>
-      <c r="V146" s="4"/>
-      <c r="W146" s="4"/>
-      <c r="X146" s="4"/>
-      <c r="Y146" s="4"/>
     </row>
     <row r="147" ht="15.75" customHeight="1">
       <c r="A147" s="4"/>
@@ -4531,10 +3931,6 @@
       <c r="S147" s="4"/>
       <c r="T147" s="4"/>
       <c r="U147" s="4"/>
-      <c r="V147" s="4"/>
-      <c r="W147" s="4"/>
-      <c r="X147" s="4"/>
-      <c r="Y147" s="4"/>
     </row>
     <row r="148" ht="15.75" customHeight="1">
       <c r="A148" s="4"/>
@@ -4558,10 +3954,6 @@
       <c r="S148" s="4"/>
       <c r="T148" s="4"/>
       <c r="U148" s="4"/>
-      <c r="V148" s="4"/>
-      <c r="W148" s="4"/>
-      <c r="X148" s="4"/>
-      <c r="Y148" s="4"/>
     </row>
     <row r="149" ht="15.75" customHeight="1">
       <c r="A149" s="4"/>
@@ -4585,10 +3977,6 @@
       <c r="S149" s="4"/>
       <c r="T149" s="4"/>
       <c r="U149" s="4"/>
-      <c r="V149" s="4"/>
-      <c r="W149" s="4"/>
-      <c r="X149" s="4"/>
-      <c r="Y149" s="4"/>
     </row>
     <row r="150" ht="15.75" customHeight="1">
       <c r="A150" s="4"/>
@@ -4612,10 +4000,6 @@
       <c r="S150" s="4"/>
       <c r="T150" s="4"/>
       <c r="U150" s="4"/>
-      <c r="V150" s="4"/>
-      <c r="W150" s="4"/>
-      <c r="X150" s="4"/>
-      <c r="Y150" s="4"/>
     </row>
     <row r="151" ht="15.75" customHeight="1">
       <c r="A151" s="4"/>
@@ -4639,10 +4023,6 @@
       <c r="S151" s="4"/>
       <c r="T151" s="4"/>
       <c r="U151" s="4"/>
-      <c r="V151" s="4"/>
-      <c r="W151" s="4"/>
-      <c r="X151" s="4"/>
-      <c r="Y151" s="4"/>
     </row>
     <row r="152" ht="15.75" customHeight="1">
       <c r="A152" s="4"/>
@@ -4666,10 +4046,6 @@
       <c r="S152" s="4"/>
       <c r="T152" s="4"/>
       <c r="U152" s="4"/>
-      <c r="V152" s="4"/>
-      <c r="W152" s="4"/>
-      <c r="X152" s="4"/>
-      <c r="Y152" s="4"/>
     </row>
     <row r="153" ht="15.75" customHeight="1">
       <c r="A153" s="4"/>
@@ -4693,10 +4069,6 @@
       <c r="S153" s="4"/>
       <c r="T153" s="4"/>
       <c r="U153" s="4"/>
-      <c r="V153" s="4"/>
-      <c r="W153" s="4"/>
-      <c r="X153" s="4"/>
-      <c r="Y153" s="4"/>
     </row>
     <row r="154" ht="15.75" customHeight="1">
       <c r="A154" s="4"/>
@@ -4720,10 +4092,6 @@
       <c r="S154" s="4"/>
       <c r="T154" s="4"/>
       <c r="U154" s="4"/>
-      <c r="V154" s="4"/>
-      <c r="W154" s="4"/>
-      <c r="X154" s="4"/>
-      <c r="Y154" s="4"/>
     </row>
     <row r="155" ht="15.75" customHeight="1">
       <c r="A155" s="4"/>
@@ -4747,10 +4115,6 @@
       <c r="S155" s="4"/>
       <c r="T155" s="4"/>
       <c r="U155" s="4"/>
-      <c r="V155" s="4"/>
-      <c r="W155" s="4"/>
-      <c r="X155" s="4"/>
-      <c r="Y155" s="4"/>
     </row>
     <row r="156" ht="15.75" customHeight="1">
       <c r="A156" s="4"/>
@@ -4774,10 +4138,6 @@
       <c r="S156" s="4"/>
       <c r="T156" s="4"/>
       <c r="U156" s="4"/>
-      <c r="V156" s="4"/>
-      <c r="W156" s="4"/>
-      <c r="X156" s="4"/>
-      <c r="Y156" s="4"/>
     </row>
     <row r="157" ht="15.75" customHeight="1">
       <c r="A157" s="4"/>
@@ -4801,10 +4161,6 @@
       <c r="S157" s="4"/>
       <c r="T157" s="4"/>
       <c r="U157" s="4"/>
-      <c r="V157" s="4"/>
-      <c r="W157" s="4"/>
-      <c r="X157" s="4"/>
-      <c r="Y157" s="4"/>
     </row>
     <row r="158" ht="15.75" customHeight="1">
       <c r="A158" s="4"/>
@@ -4828,10 +4184,6 @@
       <c r="S158" s="4"/>
       <c r="T158" s="4"/>
       <c r="U158" s="4"/>
-      <c r="V158" s="4"/>
-      <c r="W158" s="4"/>
-      <c r="X158" s="4"/>
-      <c r="Y158" s="4"/>
     </row>
     <row r="159" ht="15.75" customHeight="1">
       <c r="A159" s="4"/>
@@ -4855,10 +4207,6 @@
       <c r="S159" s="4"/>
       <c r="T159" s="4"/>
       <c r="U159" s="4"/>
-      <c r="V159" s="4"/>
-      <c r="W159" s="4"/>
-      <c r="X159" s="4"/>
-      <c r="Y159" s="4"/>
     </row>
     <row r="160" ht="15.75" customHeight="1">
       <c r="A160" s="4"/>
@@ -4882,10 +4230,6 @@
       <c r="S160" s="4"/>
       <c r="T160" s="4"/>
       <c r="U160" s="4"/>
-      <c r="V160" s="4"/>
-      <c r="W160" s="4"/>
-      <c r="X160" s="4"/>
-      <c r="Y160" s="4"/>
     </row>
     <row r="161" ht="15.75" customHeight="1">
       <c r="A161" s="4"/>
@@ -4909,10 +4253,6 @@
       <c r="S161" s="4"/>
       <c r="T161" s="4"/>
       <c r="U161" s="4"/>
-      <c r="V161" s="4"/>
-      <c r="W161" s="4"/>
-      <c r="X161" s="4"/>
-      <c r="Y161" s="4"/>
     </row>
     <row r="162" ht="15.75" customHeight="1">
       <c r="A162" s="4"/>
@@ -4936,10 +4276,6 @@
       <c r="S162" s="4"/>
       <c r="T162" s="4"/>
       <c r="U162" s="4"/>
-      <c r="V162" s="4"/>
-      <c r="W162" s="4"/>
-      <c r="X162" s="4"/>
-      <c r="Y162" s="4"/>
     </row>
     <row r="163" ht="15.75" customHeight="1">
       <c r="A163" s="4"/>
@@ -4963,10 +4299,6 @@
       <c r="S163" s="4"/>
       <c r="T163" s="4"/>
       <c r="U163" s="4"/>
-      <c r="V163" s="4"/>
-      <c r="W163" s="4"/>
-      <c r="X163" s="4"/>
-      <c r="Y163" s="4"/>
     </row>
     <row r="164" ht="15.75" customHeight="1">
       <c r="A164" s="4"/>
@@ -4990,10 +4322,6 @@
       <c r="S164" s="4"/>
       <c r="T164" s="4"/>
       <c r="U164" s="4"/>
-      <c r="V164" s="4"/>
-      <c r="W164" s="4"/>
-      <c r="X164" s="4"/>
-      <c r="Y164" s="4"/>
     </row>
     <row r="165" ht="15.75" customHeight="1">
       <c r="A165" s="4"/>
@@ -5017,10 +4345,6 @@
       <c r="S165" s="4"/>
       <c r="T165" s="4"/>
       <c r="U165" s="4"/>
-      <c r="V165" s="4"/>
-      <c r="W165" s="4"/>
-      <c r="X165" s="4"/>
-      <c r="Y165" s="4"/>
     </row>
     <row r="166" ht="15.75" customHeight="1">
       <c r="A166" s="4"/>
@@ -5044,10 +4368,6 @@
       <c r="S166" s="4"/>
       <c r="T166" s="4"/>
       <c r="U166" s="4"/>
-      <c r="V166" s="4"/>
-      <c r="W166" s="4"/>
-      <c r="X166" s="4"/>
-      <c r="Y166" s="4"/>
     </row>
     <row r="167" ht="15.75" customHeight="1">
       <c r="A167" s="4"/>
@@ -5071,10 +4391,6 @@
       <c r="S167" s="4"/>
       <c r="T167" s="4"/>
       <c r="U167" s="4"/>
-      <c r="V167" s="4"/>
-      <c r="W167" s="4"/>
-      <c r="X167" s="4"/>
-      <c r="Y167" s="4"/>
     </row>
     <row r="168" ht="15.75" customHeight="1">
       <c r="A168" s="4"/>
@@ -5098,10 +4414,6 @@
       <c r="S168" s="4"/>
       <c r="T168" s="4"/>
       <c r="U168" s="4"/>
-      <c r="V168" s="4"/>
-      <c r="W168" s="4"/>
-      <c r="X168" s="4"/>
-      <c r="Y168" s="4"/>
     </row>
     <row r="169" ht="15.75" customHeight="1">
       <c r="A169" s="4"/>
@@ -5125,10 +4437,6 @@
       <c r="S169" s="4"/>
       <c r="T169" s="4"/>
       <c r="U169" s="4"/>
-      <c r="V169" s="4"/>
-      <c r="W169" s="4"/>
-      <c r="X169" s="4"/>
-      <c r="Y169" s="4"/>
     </row>
     <row r="170" ht="15.75" customHeight="1">
       <c r="A170" s="4"/>
@@ -5152,10 +4460,6 @@
       <c r="S170" s="4"/>
       <c r="T170" s="4"/>
       <c r="U170" s="4"/>
-      <c r="V170" s="4"/>
-      <c r="W170" s="4"/>
-      <c r="X170" s="4"/>
-      <c r="Y170" s="4"/>
     </row>
     <row r="171" ht="15.75" customHeight="1">
       <c r="A171" s="4"/>
@@ -5179,10 +4483,6 @@
       <c r="S171" s="4"/>
       <c r="T171" s="4"/>
       <c r="U171" s="4"/>
-      <c r="V171" s="4"/>
-      <c r="W171" s="4"/>
-      <c r="X171" s="4"/>
-      <c r="Y171" s="4"/>
     </row>
     <row r="172" ht="15.75" customHeight="1">
       <c r="A172" s="4"/>
@@ -5206,10 +4506,6 @@
       <c r="S172" s="4"/>
       <c r="T172" s="4"/>
       <c r="U172" s="4"/>
-      <c r="V172" s="4"/>
-      <c r="W172" s="4"/>
-      <c r="X172" s="4"/>
-      <c r="Y172" s="4"/>
     </row>
     <row r="173" ht="15.75" customHeight="1">
       <c r="A173" s="4"/>
@@ -5233,10 +4529,6 @@
       <c r="S173" s="4"/>
       <c r="T173" s="4"/>
       <c r="U173" s="4"/>
-      <c r="V173" s="4"/>
-      <c r="W173" s="4"/>
-      <c r="X173" s="4"/>
-      <c r="Y173" s="4"/>
     </row>
     <row r="174" ht="15.75" customHeight="1">
       <c r="A174" s="4"/>
@@ -5260,10 +4552,6 @@
       <c r="S174" s="4"/>
       <c r="T174" s="4"/>
       <c r="U174" s="4"/>
-      <c r="V174" s="4"/>
-      <c r="W174" s="4"/>
-      <c r="X174" s="4"/>
-      <c r="Y174" s="4"/>
     </row>
     <row r="175" ht="15.75" customHeight="1">
       <c r="A175" s="4"/>
@@ -5287,10 +4575,6 @@
       <c r="S175" s="4"/>
       <c r="T175" s="4"/>
       <c r="U175" s="4"/>
-      <c r="V175" s="4"/>
-      <c r="W175" s="4"/>
-      <c r="X175" s="4"/>
-      <c r="Y175" s="4"/>
     </row>
     <row r="176" ht="15.75" customHeight="1">
       <c r="A176" s="4"/>
@@ -5314,10 +4598,6 @@
       <c r="S176" s="4"/>
       <c r="T176" s="4"/>
       <c r="U176" s="4"/>
-      <c r="V176" s="4"/>
-      <c r="W176" s="4"/>
-      <c r="X176" s="4"/>
-      <c r="Y176" s="4"/>
     </row>
     <row r="177" ht="15.75" customHeight="1">
       <c r="A177" s="4"/>
@@ -5341,10 +4621,6 @@
       <c r="S177" s="4"/>
       <c r="T177" s="4"/>
       <c r="U177" s="4"/>
-      <c r="V177" s="4"/>
-      <c r="W177" s="4"/>
-      <c r="X177" s="4"/>
-      <c r="Y177" s="4"/>
     </row>
     <row r="178" ht="15.75" customHeight="1">
       <c r="A178" s="4"/>
@@ -5368,10 +4644,6 @@
       <c r="S178" s="4"/>
       <c r="T178" s="4"/>
       <c r="U178" s="4"/>
-      <c r="V178" s="4"/>
-      <c r="W178" s="4"/>
-      <c r="X178" s="4"/>
-      <c r="Y178" s="4"/>
     </row>
     <row r="179" ht="15.75" customHeight="1">
       <c r="A179" s="4"/>
@@ -5395,10 +4667,6 @@
       <c r="S179" s="4"/>
       <c r="T179" s="4"/>
       <c r="U179" s="4"/>
-      <c r="V179" s="4"/>
-      <c r="W179" s="4"/>
-      <c r="X179" s="4"/>
-      <c r="Y179" s="4"/>
     </row>
     <row r="180" ht="15.75" customHeight="1">
       <c r="A180" s="4"/>
@@ -5422,10 +4690,6 @@
       <c r="S180" s="4"/>
       <c r="T180" s="4"/>
       <c r="U180" s="4"/>
-      <c r="V180" s="4"/>
-      <c r="W180" s="4"/>
-      <c r="X180" s="4"/>
-      <c r="Y180" s="4"/>
     </row>
     <row r="181" ht="15.75" customHeight="1">
       <c r="A181" s="4"/>
@@ -5449,10 +4713,6 @@
       <c r="S181" s="4"/>
       <c r="T181" s="4"/>
       <c r="U181" s="4"/>
-      <c r="V181" s="4"/>
-      <c r="W181" s="4"/>
-      <c r="X181" s="4"/>
-      <c r="Y181" s="4"/>
     </row>
     <row r="182" ht="15.75" customHeight="1">
       <c r="A182" s="4"/>
@@ -5476,10 +4736,6 @@
       <c r="S182" s="4"/>
       <c r="T182" s="4"/>
       <c r="U182" s="4"/>
-      <c r="V182" s="4"/>
-      <c r="W182" s="4"/>
-      <c r="X182" s="4"/>
-      <c r="Y182" s="4"/>
     </row>
     <row r="183" ht="15.75" customHeight="1">
       <c r="A183" s="4"/>
@@ -5503,10 +4759,6 @@
       <c r="S183" s="4"/>
       <c r="T183" s="4"/>
       <c r="U183" s="4"/>
-      <c r="V183" s="4"/>
-      <c r="W183" s="4"/>
-      <c r="X183" s="4"/>
-      <c r="Y183" s="4"/>
     </row>
     <row r="184" ht="15.75" customHeight="1">
       <c r="A184" s="4"/>
@@ -5530,10 +4782,6 @@
       <c r="S184" s="4"/>
       <c r="T184" s="4"/>
       <c r="U184" s="4"/>
-      <c r="V184" s="4"/>
-      <c r="W184" s="4"/>
-      <c r="X184" s="4"/>
-      <c r="Y184" s="4"/>
     </row>
     <row r="185" ht="15.75" customHeight="1">
       <c r="A185" s="4"/>
@@ -5557,10 +4805,6 @@
       <c r="S185" s="4"/>
       <c r="T185" s="4"/>
       <c r="U185" s="4"/>
-      <c r="V185" s="4"/>
-      <c r="W185" s="4"/>
-      <c r="X185" s="4"/>
-      <c r="Y185" s="4"/>
     </row>
     <row r="186" ht="15.75" customHeight="1">
       <c r="A186" s="4"/>
@@ -5584,10 +4828,6 @@
       <c r="S186" s="4"/>
       <c r="T186" s="4"/>
       <c r="U186" s="4"/>
-      <c r="V186" s="4"/>
-      <c r="W186" s="4"/>
-      <c r="X186" s="4"/>
-      <c r="Y186" s="4"/>
     </row>
     <row r="187" ht="15.75" customHeight="1">
       <c r="A187" s="4"/>
@@ -5611,10 +4851,6 @@
       <c r="S187" s="4"/>
       <c r="T187" s="4"/>
       <c r="U187" s="4"/>
-      <c r="V187" s="4"/>
-      <c r="W187" s="4"/>
-      <c r="X187" s="4"/>
-      <c r="Y187" s="4"/>
     </row>
     <row r="188" ht="15.75" customHeight="1">
       <c r="A188" s="4"/>
@@ -5638,10 +4874,6 @@
       <c r="S188" s="4"/>
       <c r="T188" s="4"/>
       <c r="U188" s="4"/>
-      <c r="V188" s="4"/>
-      <c r="W188" s="4"/>
-      <c r="X188" s="4"/>
-      <c r="Y188" s="4"/>
     </row>
     <row r="189" ht="15.75" customHeight="1">
       <c r="A189" s="4"/>
@@ -5665,10 +4897,6 @@
       <c r="S189" s="4"/>
       <c r="T189" s="4"/>
       <c r="U189" s="4"/>
-      <c r="V189" s="4"/>
-      <c r="W189" s="4"/>
-      <c r="X189" s="4"/>
-      <c r="Y189" s="4"/>
     </row>
     <row r="190" ht="15.75" customHeight="1">
       <c r="A190" s="4"/>
@@ -5692,10 +4920,6 @@
       <c r="S190" s="4"/>
       <c r="T190" s="4"/>
       <c r="U190" s="4"/>
-      <c r="V190" s="4"/>
-      <c r="W190" s="4"/>
-      <c r="X190" s="4"/>
-      <c r="Y190" s="4"/>
     </row>
     <row r="191" ht="15.75" customHeight="1">
       <c r="A191" s="4"/>
@@ -5719,10 +4943,6 @@
       <c r="S191" s="4"/>
       <c r="T191" s="4"/>
       <c r="U191" s="4"/>
-      <c r="V191" s="4"/>
-      <c r="W191" s="4"/>
-      <c r="X191" s="4"/>
-      <c r="Y191" s="4"/>
     </row>
     <row r="192" ht="15.75" customHeight="1">
       <c r="A192" s="4"/>
@@ -5746,10 +4966,6 @@
       <c r="S192" s="4"/>
       <c r="T192" s="4"/>
       <c r="U192" s="4"/>
-      <c r="V192" s="4"/>
-      <c r="W192" s="4"/>
-      <c r="X192" s="4"/>
-      <c r="Y192" s="4"/>
     </row>
     <row r="193" ht="15.75" customHeight="1">
       <c r="A193" s="4"/>
@@ -5773,10 +4989,6 @@
       <c r="S193" s="4"/>
       <c r="T193" s="4"/>
       <c r="U193" s="4"/>
-      <c r="V193" s="4"/>
-      <c r="W193" s="4"/>
-      <c r="X193" s="4"/>
-      <c r="Y193" s="4"/>
     </row>
     <row r="194" ht="15.75" customHeight="1">
       <c r="A194" s="4"/>
@@ -5800,10 +5012,6 @@
       <c r="S194" s="4"/>
       <c r="T194" s="4"/>
       <c r="U194" s="4"/>
-      <c r="V194" s="4"/>
-      <c r="W194" s="4"/>
-      <c r="X194" s="4"/>
-      <c r="Y194" s="4"/>
     </row>
     <row r="195" ht="15.75" customHeight="1">
       <c r="A195" s="4"/>
@@ -5827,10 +5035,6 @@
       <c r="S195" s="4"/>
       <c r="T195" s="4"/>
       <c r="U195" s="4"/>
-      <c r="V195" s="4"/>
-      <c r="W195" s="4"/>
-      <c r="X195" s="4"/>
-      <c r="Y195" s="4"/>
     </row>
     <row r="196" ht="15.75" customHeight="1">
       <c r="A196" s="4"/>
@@ -5854,10 +5058,6 @@
       <c r="S196" s="4"/>
       <c r="T196" s="4"/>
       <c r="U196" s="4"/>
-      <c r="V196" s="4"/>
-      <c r="W196" s="4"/>
-      <c r="X196" s="4"/>
-      <c r="Y196" s="4"/>
     </row>
     <row r="197" ht="15.75" customHeight="1">
       <c r="A197" s="4"/>
@@ -5881,10 +5081,6 @@
       <c r="S197" s="4"/>
       <c r="T197" s="4"/>
       <c r="U197" s="4"/>
-      <c r="V197" s="4"/>
-      <c r="W197" s="4"/>
-      <c r="X197" s="4"/>
-      <c r="Y197" s="4"/>
     </row>
     <row r="198" ht="15.75" customHeight="1">
       <c r="A198" s="4"/>
@@ -5908,10 +5104,6 @@
       <c r="S198" s="4"/>
       <c r="T198" s="4"/>
       <c r="U198" s="4"/>
-      <c r="V198" s="4"/>
-      <c r="W198" s="4"/>
-      <c r="X198" s="4"/>
-      <c r="Y198" s="4"/>
     </row>
     <row r="199" ht="15.75" customHeight="1">
       <c r="A199" s="4"/>
@@ -5935,10 +5127,6 @@
       <c r="S199" s="4"/>
       <c r="T199" s="4"/>
       <c r="U199" s="4"/>
-      <c r="V199" s="4"/>
-      <c r="W199" s="4"/>
-      <c r="X199" s="4"/>
-      <c r="Y199" s="4"/>
     </row>
     <row r="200" ht="15.75" customHeight="1">
       <c r="A200" s="4"/>
@@ -5962,10 +5150,6 @@
       <c r="S200" s="4"/>
       <c r="T200" s="4"/>
       <c r="U200" s="4"/>
-      <c r="V200" s="4"/>
-      <c r="W200" s="4"/>
-      <c r="X200" s="4"/>
-      <c r="Y200" s="4"/>
     </row>
     <row r="201" ht="15.75" customHeight="1">
       <c r="A201" s="4"/>
@@ -5989,10 +5173,6 @@
       <c r="S201" s="4"/>
       <c r="T201" s="4"/>
       <c r="U201" s="4"/>
-      <c r="V201" s="4"/>
-      <c r="W201" s="4"/>
-      <c r="X201" s="4"/>
-      <c r="Y201" s="4"/>
     </row>
     <row r="202" ht="15.75" customHeight="1">
       <c r="A202" s="4"/>
@@ -6016,10 +5196,6 @@
       <c r="S202" s="4"/>
       <c r="T202" s="4"/>
       <c r="U202" s="4"/>
-      <c r="V202" s="4"/>
-      <c r="W202" s="4"/>
-      <c r="X202" s="4"/>
-      <c r="Y202" s="4"/>
     </row>
     <row r="203" ht="15.75" customHeight="1">
       <c r="A203" s="4"/>
@@ -6043,10 +5219,6 @@
       <c r="S203" s="4"/>
       <c r="T203" s="4"/>
       <c r="U203" s="4"/>
-      <c r="V203" s="4"/>
-      <c r="W203" s="4"/>
-      <c r="X203" s="4"/>
-      <c r="Y203" s="4"/>
     </row>
     <row r="204" ht="15.75" customHeight="1">
       <c r="A204" s="4"/>
@@ -6070,10 +5242,6 @@
       <c r="S204" s="4"/>
       <c r="T204" s="4"/>
       <c r="U204" s="4"/>
-      <c r="V204" s="4"/>
-      <c r="W204" s="4"/>
-      <c r="X204" s="4"/>
-      <c r="Y204" s="4"/>
     </row>
     <row r="205" ht="15.75" customHeight="1">
       <c r="A205" s="4"/>
@@ -6097,10 +5265,6 @@
       <c r="S205" s="4"/>
       <c r="T205" s="4"/>
       <c r="U205" s="4"/>
-      <c r="V205" s="4"/>
-      <c r="W205" s="4"/>
-      <c r="X205" s="4"/>
-      <c r="Y205" s="4"/>
     </row>
     <row r="206" ht="15.75" customHeight="1">
       <c r="A206" s="4"/>
@@ -6124,10 +5288,6 @@
       <c r="S206" s="4"/>
       <c r="T206" s="4"/>
       <c r="U206" s="4"/>
-      <c r="V206" s="4"/>
-      <c r="W206" s="4"/>
-      <c r="X206" s="4"/>
-      <c r="Y206" s="4"/>
     </row>
     <row r="207" ht="15.75" customHeight="1">
       <c r="A207" s="4"/>
@@ -6151,10 +5311,6 @@
       <c r="S207" s="4"/>
       <c r="T207" s="4"/>
       <c r="U207" s="4"/>
-      <c r="V207" s="4"/>
-      <c r="W207" s="4"/>
-      <c r="X207" s="4"/>
-      <c r="Y207" s="4"/>
     </row>
     <row r="208" ht="15.75" customHeight="1">
       <c r="A208" s="4"/>
@@ -6178,10 +5334,6 @@
       <c r="S208" s="4"/>
       <c r="T208" s="4"/>
       <c r="U208" s="4"/>
-      <c r="V208" s="4"/>
-      <c r="W208" s="4"/>
-      <c r="X208" s="4"/>
-      <c r="Y208" s="4"/>
     </row>
     <row r="209" ht="15.75" customHeight="1">
       <c r="A209" s="4"/>
@@ -6205,10 +5357,6 @@
       <c r="S209" s="4"/>
       <c r="T209" s="4"/>
       <c r="U209" s="4"/>
-      <c r="V209" s="4"/>
-      <c r="W209" s="4"/>
-      <c r="X209" s="4"/>
-      <c r="Y209" s="4"/>
     </row>
     <row r="210" ht="15.75" customHeight="1">
       <c r="A210" s="4"/>
@@ -6232,10 +5380,6 @@
       <c r="S210" s="4"/>
       <c r="T210" s="4"/>
       <c r="U210" s="4"/>
-      <c r="V210" s="4"/>
-      <c r="W210" s="4"/>
-      <c r="X210" s="4"/>
-      <c r="Y210" s="4"/>
     </row>
     <row r="211" ht="15.75" customHeight="1">
       <c r="A211" s="4"/>
@@ -6259,10 +5403,6 @@
       <c r="S211" s="4"/>
       <c r="T211" s="4"/>
       <c r="U211" s="4"/>
-      <c r="V211" s="4"/>
-      <c r="W211" s="4"/>
-      <c r="X211" s="4"/>
-      <c r="Y211" s="4"/>
     </row>
     <row r="212" ht="15.75" customHeight="1">
       <c r="A212" s="4"/>
@@ -6286,10 +5426,6 @@
       <c r="S212" s="4"/>
       <c r="T212" s="4"/>
       <c r="U212" s="4"/>
-      <c r="V212" s="4"/>
-      <c r="W212" s="4"/>
-      <c r="X212" s="4"/>
-      <c r="Y212" s="4"/>
     </row>
     <row r="213" ht="15.75" customHeight="1">
       <c r="A213" s="4"/>
@@ -6313,10 +5449,6 @@
       <c r="S213" s="4"/>
       <c r="T213" s="4"/>
       <c r="U213" s="4"/>
-      <c r="V213" s="4"/>
-      <c r="W213" s="4"/>
-      <c r="X213" s="4"/>
-      <c r="Y213" s="4"/>
     </row>
     <row r="214" ht="15.75" customHeight="1">
       <c r="A214" s="4"/>
@@ -6340,10 +5472,6 @@
       <c r="S214" s="4"/>
       <c r="T214" s="4"/>
       <c r="U214" s="4"/>
-      <c r="V214" s="4"/>
-      <c r="W214" s="4"/>
-      <c r="X214" s="4"/>
-      <c r="Y214" s="4"/>
     </row>
     <row r="215" ht="15.75" customHeight="1">
       <c r="A215" s="4"/>
@@ -6367,10 +5495,6 @@
       <c r="S215" s="4"/>
       <c r="T215" s="4"/>
       <c r="U215" s="4"/>
-      <c r="V215" s="4"/>
-      <c r="W215" s="4"/>
-      <c r="X215" s="4"/>
-      <c r="Y215" s="4"/>
     </row>
     <row r="216" ht="15.75" customHeight="1">
       <c r="A216" s="4"/>
@@ -6394,10 +5518,6 @@
       <c r="S216" s="4"/>
       <c r="T216" s="4"/>
       <c r="U216" s="4"/>
-      <c r="V216" s="4"/>
-      <c r="W216" s="4"/>
-      <c r="X216" s="4"/>
-      <c r="Y216" s="4"/>
     </row>
     <row r="217" ht="15.75" customHeight="1">
       <c r="A217" s="4"/>
@@ -6421,10 +5541,6 @@
       <c r="S217" s="4"/>
       <c r="T217" s="4"/>
       <c r="U217" s="4"/>
-      <c r="V217" s="4"/>
-      <c r="W217" s="4"/>
-      <c r="X217" s="4"/>
-      <c r="Y217" s="4"/>
     </row>
     <row r="218" ht="15.75" customHeight="1">
       <c r="A218" s="4"/>
@@ -6448,10 +5564,6 @@
       <c r="S218" s="4"/>
       <c r="T218" s="4"/>
       <c r="U218" s="4"/>
-      <c r="V218" s="4"/>
-      <c r="W218" s="4"/>
-      <c r="X218" s="4"/>
-      <c r="Y218" s="4"/>
     </row>
     <row r="219" ht="15.75" customHeight="1">
       <c r="A219" s="4"/>
@@ -6475,10 +5587,6 @@
       <c r="S219" s="4"/>
       <c r="T219" s="4"/>
       <c r="U219" s="4"/>
-      <c r="V219" s="4"/>
-      <c r="W219" s="4"/>
-      <c r="X219" s="4"/>
-      <c r="Y219" s="4"/>
     </row>
     <row r="220" ht="15.75" customHeight="1">
       <c r="A220" s="4"/>
@@ -6502,10 +5610,6 @@
       <c r="S220" s="4"/>
       <c r="T220" s="4"/>
       <c r="U220" s="4"/>
-      <c r="V220" s="4"/>
-      <c r="W220" s="4"/>
-      <c r="X220" s="4"/>
-      <c r="Y220" s="4"/>
     </row>
     <row r="221" ht="15.75" customHeight="1"/>
     <row r="222" ht="15.75" customHeight="1"/>

</xml_diff>

<commit_message>
test: validate payment error message
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/testData_Appium_myDemoApp.xlsx
+++ b/src/test/resources/testData/testData_Appium_myDemoApp.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="46">
   <si>
     <t>CT</t>
   </si>
@@ -52,10 +52,16 @@
     <t>CARD_NUMBER</t>
   </si>
   <si>
+    <t>EXPIRATION_DATE</t>
+  </si>
+  <si>
+    <t>SECURITY_CODE</t>
+  </si>
+  <si>
     <t>001</t>
   </si>
   <si>
-    <t>TESTE</t>
+    <t>TEST</t>
   </si>
   <si>
     <t>002</t>
@@ -125,6 +131,15 @@
   </si>
   <si>
     <t>016</t>
+  </si>
+  <si>
+    <t>TEST TEST</t>
+  </si>
+  <si>
+    <t>TESTE</t>
+  </si>
+  <si>
+    <t>12345</t>
   </si>
   <si>
     <t>017</t>
@@ -424,11 +439,13 @@
     <col customWidth="1" min="5" max="5" width="33.25"/>
     <col customWidth="1" min="6" max="6" width="42.88"/>
     <col customWidth="1" min="7" max="7" width="31.38"/>
-    <col customWidth="1" min="8" max="8" width="18.63"/>
+    <col customWidth="1" min="8" max="8" width="21.13"/>
     <col customWidth="1" min="9" max="9" width="17.13"/>
     <col customWidth="1" min="10" max="10" width="15.75"/>
     <col customWidth="1" min="11" max="11" width="14.38"/>
     <col customWidth="1" min="13" max="13" width="27.0"/>
+    <col customWidth="1" min="14" max="14" width="28.13"/>
+    <col customWidth="1" min="15" max="15" width="26.5"/>
   </cols>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
@@ -471,8 +488,12 @@
       <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="4"/>
-      <c r="O1" s="4"/>
+      <c r="N1" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="3" t="s">
+        <v>14</v>
+      </c>
       <c r="P1" s="4"/>
       <c r="Q1" s="4"/>
       <c r="R1" s="4"/>
@@ -482,13 +503,13 @@
     </row>
     <row r="2" ht="15.75" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>16</v>
       </c>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
@@ -500,8 +521,8 @@
       <c r="K2" s="1"/>
       <c r="L2" s="1"/>
       <c r="M2" s="1"/>
-      <c r="N2" s="4"/>
-      <c r="O2" s="4"/>
+      <c r="N2" s="1"/>
+      <c r="O2" s="1"/>
       <c r="P2" s="4"/>
       <c r="Q2" s="4"/>
       <c r="R2" s="4"/>
@@ -511,7 +532,7 @@
     </row>
     <row r="3" ht="15.75" customHeight="1">
       <c r="A3" s="2" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
@@ -525,8 +546,8 @@
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
-      <c r="N3" s="4"/>
-      <c r="O3" s="4"/>
+      <c r="N3" s="1"/>
+      <c r="O3" s="1"/>
       <c r="P3" s="4"/>
       <c r="Q3" s="4"/>
       <c r="R3" s="4"/>
@@ -536,13 +557,13 @@
     </row>
     <row r="4" ht="15.75" customHeight="1">
       <c r="A4" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>14</v>
+      <c r="C4" s="3" t="s">
+        <v>16</v>
       </c>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
@@ -554,8 +575,8 @@
       <c r="K4" s="1"/>
       <c r="L4" s="1"/>
       <c r="M4" s="1"/>
-      <c r="N4" s="4"/>
-      <c r="O4" s="4"/>
+      <c r="N4" s="1"/>
+      <c r="O4" s="1"/>
       <c r="P4" s="4"/>
       <c r="Q4" s="4"/>
       <c r="R4" s="4"/>
@@ -565,12 +586,12 @@
     </row>
     <row r="5" ht="15.75" customHeight="1">
       <c r="A5" s="1" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
       <c r="D5" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="E5" s="1"/>
       <c r="F5" s="1"/>
@@ -581,8 +602,8 @@
       <c r="K5" s="1"/>
       <c r="L5" s="1"/>
       <c r="M5" s="1"/>
-      <c r="N5" s="4"/>
-      <c r="O5" s="4"/>
+      <c r="N5" s="1"/>
+      <c r="O5" s="1"/>
       <c r="P5" s="4"/>
       <c r="Q5" s="4"/>
       <c r="R5" s="4"/>
@@ -592,12 +613,12 @@
     </row>
     <row r="6" ht="15.75" customHeight="1">
       <c r="A6" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
       <c r="D6" s="1" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E6" s="1"/>
       <c r="F6" s="1"/>
@@ -608,8 +629,8 @@
       <c r="K6" s="1"/>
       <c r="L6" s="1"/>
       <c r="M6" s="1"/>
-      <c r="N6" s="4"/>
-      <c r="O6" s="4"/>
+      <c r="N6" s="1"/>
+      <c r="O6" s="1"/>
       <c r="P6" s="4"/>
       <c r="Q6" s="4"/>
       <c r="R6" s="4"/>
@@ -619,12 +640,12 @@
     </row>
     <row r="7" ht="15.75" customHeight="1">
       <c r="A7" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
       <c r="D7" s="1" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="E7" s="1"/>
       <c r="F7" s="1"/>
@@ -635,8 +656,8 @@
       <c r="K7" s="1"/>
       <c r="L7" s="1"/>
       <c r="M7" s="1"/>
-      <c r="N7" s="4"/>
-      <c r="O7" s="4"/>
+      <c r="N7" s="1"/>
+      <c r="O7" s="1"/>
       <c r="P7" s="4"/>
       <c r="Q7" s="4"/>
       <c r="R7" s="4"/>
@@ -646,12 +667,12 @@
     </row>
     <row r="8" ht="15.75" customHeight="1">
       <c r="A8" s="1" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
       <c r="D8" s="1" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E8" s="1"/>
       <c r="F8" s="1"/>
@@ -662,8 +683,8 @@
       <c r="K8" s="1"/>
       <c r="L8" s="1"/>
       <c r="M8" s="1"/>
-      <c r="N8" s="4"/>
-      <c r="O8" s="4"/>
+      <c r="N8" s="1"/>
+      <c r="O8" s="1"/>
       <c r="P8" s="4"/>
       <c r="Q8" s="4"/>
       <c r="R8" s="4"/>
@@ -673,13 +694,13 @@
     </row>
     <row r="9" ht="15.75" customHeight="1">
       <c r="A9" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
       <c r="D9" s="1"/>
       <c r="E9" s="3" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F9" s="3"/>
       <c r="G9" s="3"/>
@@ -689,8 +710,8 @@
       <c r="K9" s="1"/>
       <c r="L9" s="1"/>
       <c r="M9" s="1"/>
-      <c r="N9" s="4"/>
-      <c r="O9" s="4"/>
+      <c r="N9" s="1"/>
+      <c r="O9" s="1"/>
       <c r="P9" s="4"/>
       <c r="Q9" s="4"/>
       <c r="R9" s="4"/>
@@ -700,17 +721,17 @@
     </row>
     <row r="10" ht="15.75" customHeight="1">
       <c r="A10" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
       <c r="D10" s="1"/>
       <c r="E10" s="3" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F10" s="3"/>
       <c r="G10" s="3" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="H10" s="1"/>
       <c r="I10" s="1"/>
@@ -718,8 +739,8 @@
       <c r="K10" s="1"/>
       <c r="L10" s="1"/>
       <c r="M10" s="1"/>
-      <c r="N10" s="4"/>
-      <c r="O10" s="4"/>
+      <c r="N10" s="1"/>
+      <c r="O10" s="1"/>
       <c r="P10" s="4"/>
       <c r="Q10" s="4"/>
       <c r="R10" s="4"/>
@@ -729,17 +750,17 @@
     </row>
     <row r="11" ht="15.75" customHeight="1">
       <c r="A11" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
       <c r="D11" s="1"/>
       <c r="E11" s="3" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F11" s="3"/>
       <c r="G11" s="3" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="H11" s="1"/>
       <c r="I11" s="1"/>
@@ -747,8 +768,8 @@
       <c r="K11" s="1"/>
       <c r="L11" s="1"/>
       <c r="M11" s="1"/>
-      <c r="N11" s="4"/>
-      <c r="O11" s="4"/>
+      <c r="N11" s="1"/>
+      <c r="O11" s="1"/>
       <c r="P11" s="4"/>
       <c r="Q11" s="4"/>
       <c r="R11" s="4"/>
@@ -758,20 +779,20 @@
     </row>
     <row r="12" ht="15.75" customHeight="1">
       <c r="A12" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>16</v>
       </c>
       <c r="D12" s="1"/>
       <c r="E12" s="3" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G12" s="3"/>
       <c r="H12" s="1"/>
@@ -780,8 +801,8 @@
       <c r="K12" s="1"/>
       <c r="L12" s="1"/>
       <c r="M12" s="1"/>
-      <c r="N12" s="4"/>
-      <c r="O12" s="4"/>
+      <c r="N12" s="1"/>
+      <c r="O12" s="1"/>
       <c r="P12" s="4"/>
       <c r="Q12" s="4"/>
       <c r="R12" s="4"/>
@@ -791,21 +812,21 @@
     </row>
     <row r="13" ht="15.75" customHeight="1">
       <c r="A13" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>16</v>
       </c>
       <c r="D13" s="1"/>
       <c r="E13" s="3" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F13" s="1"/>
       <c r="G13" s="3" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="H13" s="1"/>
       <c r="I13" s="1"/>
@@ -813,8 +834,8 @@
       <c r="K13" s="1"/>
       <c r="L13" s="1"/>
       <c r="M13" s="1"/>
-      <c r="N13" s="4"/>
-      <c r="O13" s="4"/>
+      <c r="N13" s="1"/>
+      <c r="O13" s="1"/>
       <c r="P13" s="4"/>
       <c r="Q13" s="4"/>
       <c r="R13" s="4"/>
@@ -824,17 +845,17 @@
     </row>
     <row r="14" ht="15.75" customHeight="1">
       <c r="A14" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
       <c r="D14" s="1"/>
       <c r="E14" s="3" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F14" s="1"/>
       <c r="G14" s="3" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="H14" s="1"/>
       <c r="I14" s="1"/>
@@ -842,8 +863,8 @@
       <c r="K14" s="1"/>
       <c r="L14" s="1"/>
       <c r="M14" s="1"/>
-      <c r="N14" s="4"/>
-      <c r="O14" s="4"/>
+      <c r="N14" s="1"/>
+      <c r="O14" s="1"/>
       <c r="P14" s="4"/>
       <c r="Q14" s="4"/>
       <c r="R14" s="4"/>
@@ -853,16 +874,16 @@
     </row>
     <row r="15" ht="15.75" customHeight="1">
       <c r="A15" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
       <c r="D15" s="1"/>
       <c r="E15" s="3" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="G15" s="1"/>
       <c r="H15" s="1"/>
@@ -871,8 +892,8 @@
       <c r="K15" s="1"/>
       <c r="L15" s="1"/>
       <c r="M15" s="1"/>
-      <c r="N15" s="4"/>
-      <c r="O15" s="4"/>
+      <c r="N15" s="1"/>
+      <c r="O15" s="1"/>
       <c r="P15" s="4"/>
       <c r="Q15" s="4"/>
       <c r="R15" s="4"/>
@@ -882,17 +903,17 @@
     </row>
     <row r="16" ht="15.75" customHeight="1">
       <c r="A16" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>16</v>
       </c>
       <c r="D16" s="1"/>
       <c r="E16" s="3" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F16" s="1"/>
       <c r="G16" s="1"/>
@@ -902,8 +923,8 @@
       <c r="K16" s="1"/>
       <c r="L16" s="1"/>
       <c r="M16" s="1"/>
-      <c r="N16" s="4"/>
-      <c r="O16" s="4"/>
+      <c r="N16" s="1"/>
+      <c r="O16" s="1"/>
       <c r="P16" s="4"/>
       <c r="Q16" s="4"/>
       <c r="R16" s="4"/>
@@ -913,22 +934,38 @@
     </row>
     <row r="17" ht="15.75" customHeight="1">
       <c r="A17" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="B17" s="1"/>
-      <c r="C17" s="1"/>
+        <v>39</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>16</v>
+      </c>
       <c r="D17" s="1"/>
-      <c r="E17" s="1"/>
+      <c r="E17" s="3" t="s">
+        <v>28</v>
+      </c>
       <c r="F17" s="1"/>
       <c r="G17" s="1"/>
-      <c r="H17" s="1"/>
-      <c r="I17" s="1"/>
-      <c r="J17" s="1"/>
-      <c r="K17" s="1"/>
-      <c r="L17" s="1"/>
+      <c r="H17" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="I17" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="J17" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="K17" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="L17" s="3" t="s">
+        <v>16</v>
+      </c>
       <c r="M17" s="1"/>
-      <c r="N17" s="4"/>
-      <c r="O17" s="4"/>
+      <c r="N17" s="1"/>
+      <c r="O17" s="1"/>
       <c r="P17" s="4"/>
       <c r="Q17" s="4"/>
       <c r="R17" s="4"/>
@@ -938,7 +975,7 @@
     </row>
     <row r="18" ht="15.75" customHeight="1">
       <c r="A18" s="1" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="B18" s="1"/>
       <c r="C18" s="1"/>
@@ -952,8 +989,8 @@
       <c r="K18" s="1"/>
       <c r="L18" s="1"/>
       <c r="M18" s="1"/>
-      <c r="N18" s="4"/>
-      <c r="O18" s="4"/>
+      <c r="N18" s="1"/>
+      <c r="O18" s="1"/>
       <c r="P18" s="4"/>
       <c r="Q18" s="4"/>
       <c r="R18" s="4"/>
@@ -963,7 +1000,7 @@
     </row>
     <row r="19" ht="15.75" customHeight="1">
       <c r="A19" s="1" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="B19" s="1"/>
       <c r="C19" s="1"/>
@@ -977,8 +1014,8 @@
       <c r="K19" s="1"/>
       <c r="L19" s="1"/>
       <c r="M19" s="1"/>
-      <c r="N19" s="4"/>
-      <c r="O19" s="4"/>
+      <c r="N19" s="1"/>
+      <c r="O19" s="1"/>
       <c r="P19" s="4"/>
       <c r="Q19" s="4"/>
       <c r="R19" s="4"/>
@@ -988,7 +1025,7 @@
     </row>
     <row r="20" ht="15.75" customHeight="1">
       <c r="A20" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="B20" s="1"/>
       <c r="C20" s="1"/>
@@ -1002,8 +1039,8 @@
       <c r="K20" s="1"/>
       <c r="L20" s="1"/>
       <c r="M20" s="1"/>
-      <c r="N20" s="4"/>
-      <c r="O20" s="4"/>
+      <c r="N20" s="1"/>
+      <c r="O20" s="1"/>
       <c r="P20" s="4"/>
       <c r="Q20" s="4"/>
       <c r="R20" s="4"/>

</xml_diff>

<commit_message>
test: validate successful checkout
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/testData_Appium_myDemoApp.xlsx
+++ b/src/test/resources/testData/testData_Appium_myDemoApp.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="45">
   <si>
     <t>CT</t>
   </si>
@@ -145,10 +145,7 @@
     <t>017</t>
   </si>
   <si>
-    <t>018</t>
-  </si>
-  <si>
-    <t>019</t>
+    <t>1111111111111111</t>
   </si>
 </sst>
 </file>
@@ -977,20 +974,42 @@
       <c r="A18" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="B18" s="1"/>
-      <c r="C18" s="1"/>
+      <c r="B18" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>16</v>
+      </c>
       <c r="D18" s="1"/>
-      <c r="E18" s="1"/>
+      <c r="E18" s="3" t="s">
+        <v>28</v>
+      </c>
       <c r="F18" s="1"/>
       <c r="G18" s="1"/>
-      <c r="H18" s="1"/>
-      <c r="I18" s="1"/>
-      <c r="J18" s="1"/>
-      <c r="K18" s="1"/>
-      <c r="L18" s="1"/>
-      <c r="M18" s="1"/>
-      <c r="N18" s="1"/>
-      <c r="O18" s="1"/>
+      <c r="H18" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="I18" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="J18" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="K18" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="L18" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="M18" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="N18" s="3">
+        <v>1111.0</v>
+      </c>
+      <c r="O18" s="3">
+        <v>111.0</v>
+      </c>
       <c r="P18" s="4"/>
       <c r="Q18" s="4"/>
       <c r="R18" s="4"/>
@@ -999,23 +1018,21 @@
       <c r="U18" s="4"/>
     </row>
     <row r="19" ht="15.75" customHeight="1">
-      <c r="A19" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="B19" s="1"/>
-      <c r="C19" s="1"/>
-      <c r="D19" s="1"/>
-      <c r="E19" s="1"/>
-      <c r="F19" s="1"/>
-      <c r="G19" s="1"/>
-      <c r="H19" s="1"/>
-      <c r="I19" s="1"/>
-      <c r="J19" s="1"/>
-      <c r="K19" s="1"/>
-      <c r="L19" s="1"/>
-      <c r="M19" s="1"/>
-      <c r="N19" s="1"/>
-      <c r="O19" s="1"/>
+      <c r="A19" s="4"/>
+      <c r="B19" s="4"/>
+      <c r="C19" s="4"/>
+      <c r="D19" s="4"/>
+      <c r="E19" s="4"/>
+      <c r="F19" s="4"/>
+      <c r="G19" s="4"/>
+      <c r="H19" s="4"/>
+      <c r="I19" s="4"/>
+      <c r="J19" s="4"/>
+      <c r="K19" s="4"/>
+      <c r="L19" s="4"/>
+      <c r="M19" s="4"/>
+      <c r="N19" s="4"/>
+      <c r="O19" s="4"/>
       <c r="P19" s="4"/>
       <c r="Q19" s="4"/>
       <c r="R19" s="4"/>
@@ -1024,23 +1041,21 @@
       <c r="U19" s="4"/>
     </row>
     <row r="20" ht="15.75" customHeight="1">
-      <c r="A20" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="B20" s="1"/>
-      <c r="C20" s="1"/>
-      <c r="D20" s="1"/>
-      <c r="E20" s="1"/>
-      <c r="F20" s="1"/>
-      <c r="G20" s="1"/>
-      <c r="H20" s="1"/>
-      <c r="I20" s="1"/>
-      <c r="J20" s="1"/>
-      <c r="K20" s="1"/>
-      <c r="L20" s="1"/>
-      <c r="M20" s="1"/>
-      <c r="N20" s="1"/>
-      <c r="O20" s="1"/>
+      <c r="A20" s="4"/>
+      <c r="B20" s="4"/>
+      <c r="C20" s="4"/>
+      <c r="D20" s="4"/>
+      <c r="E20" s="4"/>
+      <c r="F20" s="4"/>
+      <c r="G20" s="4"/>
+      <c r="H20" s="4"/>
+      <c r="I20" s="4"/>
+      <c r="J20" s="4"/>
+      <c r="K20" s="4"/>
+      <c r="L20" s="4"/>
+      <c r="M20" s="4"/>
+      <c r="N20" s="4"/>
+      <c r="O20" s="4"/>
       <c r="P20" s="4"/>
       <c r="Q20" s="4"/>
       <c r="R20" s="4"/>
@@ -5602,52 +5617,8 @@
       <c r="T218" s="4"/>
       <c r="U218" s="4"/>
     </row>
-    <row r="219" ht="15.75" customHeight="1">
-      <c r="A219" s="4"/>
-      <c r="B219" s="4"/>
-      <c r="C219" s="4"/>
-      <c r="D219" s="4"/>
-      <c r="E219" s="4"/>
-      <c r="F219" s="4"/>
-      <c r="G219" s="4"/>
-      <c r="H219" s="4"/>
-      <c r="I219" s="4"/>
-      <c r="J219" s="4"/>
-      <c r="K219" s="4"/>
-      <c r="L219" s="4"/>
-      <c r="M219" s="4"/>
-      <c r="N219" s="4"/>
-      <c r="O219" s="4"/>
-      <c r="P219" s="4"/>
-      <c r="Q219" s="4"/>
-      <c r="R219" s="4"/>
-      <c r="S219" s="4"/>
-      <c r="T219" s="4"/>
-      <c r="U219" s="4"/>
-    </row>
-    <row r="220" ht="15.75" customHeight="1">
-      <c r="A220" s="4"/>
-      <c r="B220" s="4"/>
-      <c r="C220" s="4"/>
-      <c r="D220" s="4"/>
-      <c r="E220" s="4"/>
-      <c r="F220" s="4"/>
-      <c r="G220" s="4"/>
-      <c r="H220" s="4"/>
-      <c r="I220" s="4"/>
-      <c r="J220" s="4"/>
-      <c r="K220" s="4"/>
-      <c r="L220" s="4"/>
-      <c r="M220" s="4"/>
-      <c r="N220" s="4"/>
-      <c r="O220" s="4"/>
-      <c r="P220" s="4"/>
-      <c r="Q220" s="4"/>
-      <c r="R220" s="4"/>
-      <c r="S220" s="4"/>
-      <c r="T220" s="4"/>
-      <c r="U220" s="4"/>
-    </row>
+    <row r="219" ht="15.75" customHeight="1"/>
+    <row r="220" ht="15.75" customHeight="1"/>
     <row r="221" ht="15.75" customHeight="1"/>
     <row r="222" ht="15.75" customHeight="1"/>
     <row r="223" ht="15.75" customHeight="1"/>
@@ -6426,8 +6397,6 @@
     <row r="996" ht="15.75" customHeight="1"/>
     <row r="997" ht="15.75" customHeight="1"/>
     <row r="998" ht="15.75" customHeight="1"/>
-    <row r="999" ht="15.75" customHeight="1"/>
-    <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>